<commit_message>
Initialisation d'un projet : nouvel écran, routes /admin/projects/import, création par phases
- Écran ProjetInit.dc.html livré (4 étapes) ; contrôle et création par le serveur (admin-api.js : validateXlsx, bindInit), exemple ORION simulé.
- API : POST /projects/import/validate (vue de l'écran + 5 contrôles), POST /projects/import/commit (recontrôle complet, 409/422, transaction tout ou rien, PREPARATION, audit sensible), GET /projects/import/{jobId} (phase, pourcentage), DELETE /projects/import/{jobId} (réinitialiser la session) ; anciennes routes /project-imports retirées.
- Création écrite dans l'ordre des 5 phases affichées, avancement réel suivi par l'écran sans le devancer.
- Modèle Excel : liste Sous-phase des jalons dépendante de la phase choisie.
- Tests : 387 verts ; recette § 6 (6 points) vérifiée.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontends/Referentiel RISE - initialisation.xlsx
+++ b/frontends/Referentiel RISE - initialisation.xlsx
@@ -9154,8 +9154,8 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste. Elle se remplit à partir de l’onglet correspondant." sqref="E10:E108">
       <formula1>L_SousPhases</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste. Elle se remplit à partir de l’onglet correspondant." sqref="E9:E108">
-      <formula1>L_SousPhases</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valeur hors liste" error="Choisissez une sous-phase de la phase de la colonne Phase (onglet 08 Sous-phases)." sqref="E9:E108">
+      <formula1>IF($D9="",L_SousPhases,OFFSET('08 Sous-phases'!$B$9,IFERROR(MATCH(LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*",'08 Sous-phases'!$B$9:$B$88,0)-1,0),0,MAX(1,COUNTIF('08 Sous-phases'!$B$9:$B$88,LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*"))))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste. Elle se remplit à partir de l’onglet correspondant." sqref="F10:F108">
       <formula1>L_Chantiers</formula1>

</xml_diff>

<commit_message>
Initialisation d'un projet : préremplissage par IA depuis la proposition commerciale
- Écran « Initialisation projet » (maquette v2, 9 états) relié à l'API : dépôt avec progression, analyse suivie par SSE, reprise, annulation, liste « À vérifier » filtrable, Excel prérempli ; écarts dans docs/NOTE - ecarts maquette Initialisation projet v2.md
- Serveur : contrôle du fichier (extension, taille, signature, lisibilité), analyse onglet par onglet par la nouvelle fonction d'IA « Initialisation projet », Excel écrit dans le XML du modèle (cellules à vérifier en ambre et commentées), purge à 24 h ; tables prefill_documents et prefill_tasks
- Fournisseurs et modèles : fonction « Initialisation projet » dans l'Affectation (principal, secours, coût mensuel estimé)
- Modèle Excel : onglets numérotés 01 à 14 (06 Info projet, 07 Lots…)
- Tests des critères d'acceptation (e2e, unitaires, recette navigateur avec modèle d'IA simulé)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontends/Referentiel RISE - initialisation.xlsx
+++ b/frontends/Referentiel RISE - initialisation.xlsx
@@ -11,15 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Personnes" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Affectations" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Projet" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05b Info projet" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Phases" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Sous-phases" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Chantiers" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Instances" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Membres" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Jalons" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Livrables" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Info projet" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Phases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Sous-phases" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Chantiers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Instances" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Membres" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Jalons" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Livrables" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="18" state="veryHidden" r:id="rId18"/>
   </sheets>
   <definedNames>
@@ -37,11 +37,11 @@
     <definedName name="L_Equipes">'01 Équipes'!$B$9:$B$38</definedName>
     <definedName name="L_Roles">'02 Rôles'!$B$9:$B$48</definedName>
     <definedName name="L_Personnes">'03 Personnes'!$B$9:$B$158</definedName>
-    <definedName name="L_Lots">'06 Lots'!$B$9:$B$38</definedName>
-    <definedName name="L_Phases">'07 Phases'!$B$9:$B$38</definedName>
-    <definedName name="L_SousPhases">'08 Sous-phases'!$B$9:$B$88</definedName>
-    <definedName name="L_Chantiers">'09 Chantiers'!$C$9:$C$38</definedName>
-    <definedName name="L_Instances">'10 Instances'!$B$9:$B$28</definedName>
+    <definedName name="L_Lots">'07 Lots'!$B$9:$B$38</definedName>
+    <definedName name="L_Phases">'08 Phases'!$B$9:$B$38</definedName>
+    <definedName name="L_SousPhases">'09 Sous-phases'!$B$9:$B$88</definedName>
+    <definedName name="L_Chantiers">'10 Chantiers'!$C$9:$C$38</definedName>
+    <definedName name="L_Instances">'11 Instances'!$B$9:$B$28</definedName>
     <definedName name="L_Rubriques">Listes!$L$2:$L$9</definedName>
     <definedName name="L_RubriquesPaires">Listes!$M$2:$M$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'01 Équipes'!$B$8:$E$8</definedName>
@@ -52,22 +52,22 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'03 Personnes'!$8:$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'04 Affectations'!$B$8:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'04 Affectations'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'06 Lots'!$B$8:$I$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'06 Lots'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'07 Phases'!$B$8:$J$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'07 Phases'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'08 Sous-phases'!$B$8:$J$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="11">'08 Sous-phases'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'09 Chantiers'!$B$8:$G$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="12">'09 Chantiers'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'10 Instances'!$B$8:$J$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="13">'10 Instances'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'11 Membres'!$B$8:$E$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="14">'11 Membres'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'12 Jalons'!$B$8:$K$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="15">'12 Jalons'!$8:$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'13 Livrables'!$B$8:$H$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="16">'13 Livrables'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'07 Lots'!$B$8:$I$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'07 Lots'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'08 Phases'!$B$8:$J$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'08 Phases'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'09 Sous-phases'!$B$8:$J$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'09 Sous-phases'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'10 Chantiers'!$B$8:$G$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'10 Chantiers'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'11 Instances'!$B$8:$J$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="13">'11 Instances'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'12 Membres'!$B$8:$E$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">'12 Membres'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'13 Jalons'!$B$8:$K$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="15">'13 Jalons'!$8:$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'14 Livrables'!$B$8:$H$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">'14 Livrables'!$8:$8</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:L38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1952,7 +1952,7 @@
     <row r="24" ht="26" customHeight="1">
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>05b</t>
+          <t>06</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="F24" s="17">
-        <f>SUMPRODUCT(((('05b Info projet'!$B$9:$B$128&lt;&gt;"")+('05b Info projet'!$C$9:$C$128&lt;&gt;"")+('05b Info projet'!$D$9:$D$128&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('06 Info projet'!$B$9:$B$128&lt;&gt;"")+('06 Info projet'!$C$9:$C$128&lt;&gt;"")+('06 Info projet'!$D$9:$D$128&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G24" s="18">
@@ -1991,7 +1991,7 @@
         <v/>
       </c>
       <c r="K24" s="21">
-        <f>(COUNTIFS('05b Info projet'!$B$9:$B$128,"Programme en une phrase",'05b Info projet'!$D$9:$D$128,"&lt;&gt;")&gt;0)+(COUNTIFS('05b Info projet'!$B$9:$B$128,"Enjeux stratégiques",'05b Info projet'!$D$9:$D$128,"&lt;&gt;")&gt;0)</f>
+        <f>(COUNTIFS('06 Info projet'!$B$9:$B$128,"Programme en une phrase",'06 Info projet'!$D$9:$D$128,"&lt;&gt;")&gt;0)+(COUNTIFS('06 Info projet'!$B$9:$B$128,"Enjeux stratégiques",'06 Info projet'!$D$9:$D$128,"&lt;&gt;")&gt;0)</f>
         <v/>
       </c>
       <c r="L24" s="21">
@@ -2002,7 +2002,7 @@
     <row r="25" ht="26" customHeight="1">
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -2021,7 +2021,7 @@
         </is>
       </c>
       <c r="F25" s="17">
-        <f>SUMPRODUCT(((('06 Lots'!$C$9:$C$38&lt;&gt;"")+('06 Lots'!$D$9:$D$38&lt;&gt;"")+('06 Lots'!$E$9:$E$38&lt;&gt;"")+('06 Lots'!$F$9:$F$38&lt;&gt;"")+('06 Lots'!$G$9:$G$38&lt;&gt;"")+('06 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('07 Lots'!$C$9:$C$38&lt;&gt;"")+('07 Lots'!$D$9:$D$38&lt;&gt;"")+('07 Lots'!$E$9:$E$38&lt;&gt;"")+('07 Lots'!$F$9:$F$38&lt;&gt;"")+('07 Lots'!$G$9:$G$38&lt;&gt;"")+('07 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G25" s="18">
@@ -2041,7 +2041,7 @@
         <v/>
       </c>
       <c r="K25" s="21">
-        <f>SUMPRODUCT(((('06 Lots'!$C$9:$C$38&lt;&gt;"")+('06 Lots'!$D$9:$D$38&lt;&gt;"")+('06 Lots'!$E$9:$E$38&lt;&gt;"")+('06 Lots'!$F$9:$F$38&lt;&gt;"")+('06 Lots'!$G$9:$G$38&lt;&gt;"")+('06 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('06 Lots'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('06 Lots'!$C$9:$C$38&lt;&gt;"")+('06 Lots'!$D$9:$D$38&lt;&gt;"")+('06 Lots'!$E$9:$E$38&lt;&gt;"")+('06 Lots'!$F$9:$F$38&lt;&gt;"")+('06 Lots'!$G$9:$G$38&lt;&gt;"")+('06 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('06 Lots'!$D$9:$D$38&lt;&gt;""))+SUMPRODUCT(((('06 Lots'!$C$9:$C$38&lt;&gt;"")+('06 Lots'!$D$9:$D$38&lt;&gt;"")+('06 Lots'!$E$9:$E$38&lt;&gt;"")+('06 Lots'!$F$9:$F$38&lt;&gt;"")+('06 Lots'!$G$9:$G$38&lt;&gt;"")+('06 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('06 Lots'!$E$9:$E$38&lt;&gt;""))+SUMPRODUCT(((('06 Lots'!$C$9:$C$38&lt;&gt;"")+('06 Lots'!$D$9:$D$38&lt;&gt;"")+('06 Lots'!$E$9:$E$38&lt;&gt;"")+('06 Lots'!$F$9:$F$38&lt;&gt;"")+('06 Lots'!$G$9:$G$38&lt;&gt;"")+('06 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('06 Lots'!$F$9:$F$38&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('07 Lots'!$C$9:$C$38&lt;&gt;"")+('07 Lots'!$D$9:$D$38&lt;&gt;"")+('07 Lots'!$E$9:$E$38&lt;&gt;"")+('07 Lots'!$F$9:$F$38&lt;&gt;"")+('07 Lots'!$G$9:$G$38&lt;&gt;"")+('07 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('07 Lots'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('07 Lots'!$C$9:$C$38&lt;&gt;"")+('07 Lots'!$D$9:$D$38&lt;&gt;"")+('07 Lots'!$E$9:$E$38&lt;&gt;"")+('07 Lots'!$F$9:$F$38&lt;&gt;"")+('07 Lots'!$G$9:$G$38&lt;&gt;"")+('07 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('07 Lots'!$D$9:$D$38&lt;&gt;""))+SUMPRODUCT(((('07 Lots'!$C$9:$C$38&lt;&gt;"")+('07 Lots'!$D$9:$D$38&lt;&gt;"")+('07 Lots'!$E$9:$E$38&lt;&gt;"")+('07 Lots'!$F$9:$F$38&lt;&gt;"")+('07 Lots'!$G$9:$G$38&lt;&gt;"")+('07 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('07 Lots'!$E$9:$E$38&lt;&gt;""))+SUMPRODUCT(((('07 Lots'!$C$9:$C$38&lt;&gt;"")+('07 Lots'!$D$9:$D$38&lt;&gt;"")+('07 Lots'!$E$9:$E$38&lt;&gt;"")+('07 Lots'!$F$9:$F$38&lt;&gt;"")+('07 Lots'!$G$9:$G$38&lt;&gt;"")+('07 Lots'!$H$9:$H$38&lt;&gt;""))&gt;0)*('07 Lots'!$F$9:$F$38&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L25" s="21">
@@ -2052,7 +2052,7 @@
     <row r="26" ht="26" customHeight="1">
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>08</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="F26" s="17">
-        <f>SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G26" s="18">
@@ -2091,7 +2091,7 @@
         <v/>
       </c>
       <c r="K26" s="21">
-        <f>SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('07 Phases'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('07 Phases'!$D$9:$D$38&lt;&gt;""))+SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('07 Phases'!$E$9:$E$38&lt;&gt;""))+SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('07 Phases'!$F$9:$F$38&lt;&gt;""))+SUMPRODUCT(((('07 Phases'!$C$9:$C$38&lt;&gt;"")+('07 Phases'!$D$9:$D$38&lt;&gt;"")+('07 Phases'!$E$9:$E$38&lt;&gt;"")+('07 Phases'!$F$9:$F$38&lt;&gt;"")+('07 Phases'!$G$9:$G$38&lt;&gt;"")+('07 Phases'!$H$9:$H$38&lt;&gt;"")+('07 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('07 Phases'!$G$9:$G$38&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('08 Phases'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('08 Phases'!$D$9:$D$38&lt;&gt;""))+SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('08 Phases'!$E$9:$E$38&lt;&gt;""))+SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('08 Phases'!$F$9:$F$38&lt;&gt;""))+SUMPRODUCT(((('08 Phases'!$C$9:$C$38&lt;&gt;"")+('08 Phases'!$D$9:$D$38&lt;&gt;"")+('08 Phases'!$E$9:$E$38&lt;&gt;"")+('08 Phases'!$F$9:$F$38&lt;&gt;"")+('08 Phases'!$G$9:$G$38&lt;&gt;"")+('08 Phases'!$H$9:$H$38&lt;&gt;"")+('08 Phases'!$I$9:$I$38&lt;&gt;""))&gt;0)*('08 Phases'!$G$9:$G$38&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L26" s="21">
@@ -2102,7 +2102,7 @@
     <row r="27" ht="26" customHeight="1">
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>09</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="F27" s="17">
-        <f>SUMPRODUCT(((('08 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('08 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('08 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('08 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('08 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('08 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('08 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('09 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('09 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('09 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('09 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('09 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('09 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('09 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G27" s="18">
@@ -2141,7 +2141,7 @@
         <v/>
       </c>
       <c r="K27" s="21">
-        <f>SUMPRODUCT(((('08 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('08 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('08 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('08 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('08 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('08 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('08 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('08 Sous-phases'!$C$9:$C$88&lt;&gt;""))+SUMPRODUCT(((('08 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('08 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('08 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('08 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('08 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('08 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('08 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('08 Sous-phases'!$D$9:$D$88&lt;&gt;""))+SUMPRODUCT(((('08 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('08 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('08 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('08 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('08 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('08 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('08 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('08 Sous-phases'!$E$9:$E$88&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('09 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('09 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('09 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('09 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('09 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('09 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('09 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('09 Sous-phases'!$C$9:$C$88&lt;&gt;""))+SUMPRODUCT(((('09 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('09 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('09 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('09 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('09 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('09 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('09 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('09 Sous-phases'!$D$9:$D$88&lt;&gt;""))+SUMPRODUCT(((('09 Sous-phases'!$C$9:$C$88&lt;&gt;"")+('09 Sous-phases'!$D$9:$D$88&lt;&gt;"")+('09 Sous-phases'!$E$9:$E$88&lt;&gt;"")+('09 Sous-phases'!$F$9:$F$88&lt;&gt;"")+('09 Sous-phases'!$G$9:$G$88&lt;&gt;"")+('09 Sous-phases'!$H$9:$H$88&lt;&gt;"")+('09 Sous-phases'!$I$9:$I$88&lt;&gt;""))&gt;0)*('09 Sous-phases'!$E$9:$E$88&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L27" s="21">
@@ -2152,7 +2152,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="F28" s="17">
-        <f>SUMPRODUCT(((('09 Chantiers'!$C$9:$C$38&lt;&gt;"")+('09 Chantiers'!$D$9:$D$38&lt;&gt;"")+('09 Chantiers'!$E$9:$E$38&lt;&gt;"")+('09 Chantiers'!$F$9:$F$38&lt;&gt;"")+('09 Chantiers'!$G$9:$G$38&lt;&gt;"")+('09 Chantiers'!$H$9:$H$38&lt;&gt;"")+('09 Chantiers'!$I$9:$I$38&lt;&gt;"")+('09 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('10 Chantiers'!$C$9:$C$38&lt;&gt;"")+('10 Chantiers'!$D$9:$D$38&lt;&gt;"")+('10 Chantiers'!$E$9:$E$38&lt;&gt;"")+('10 Chantiers'!$F$9:$F$38&lt;&gt;"")+('10 Chantiers'!$G$9:$G$38&lt;&gt;"")+('10 Chantiers'!$H$9:$H$38&lt;&gt;"")+('10 Chantiers'!$I$9:$I$38&lt;&gt;"")+('10 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G28" s="18">
@@ -2191,7 +2191,7 @@
         <v/>
       </c>
       <c r="K28" s="21">
-        <f>SUMPRODUCT(((('09 Chantiers'!$C$9:$C$38&lt;&gt;"")+('09 Chantiers'!$D$9:$D$38&lt;&gt;"")+('09 Chantiers'!$E$9:$E$38&lt;&gt;"")+('09 Chantiers'!$F$9:$F$38&lt;&gt;"")+('09 Chantiers'!$G$9:$G$38&lt;&gt;"")+('09 Chantiers'!$H$9:$H$38&lt;&gt;"")+('09 Chantiers'!$I$9:$I$38&lt;&gt;"")+('09 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*('09 Chantiers'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('09 Chantiers'!$C$9:$C$38&lt;&gt;"")+('09 Chantiers'!$D$9:$D$38&lt;&gt;"")+('09 Chantiers'!$E$9:$E$38&lt;&gt;"")+('09 Chantiers'!$F$9:$F$38&lt;&gt;"")+('09 Chantiers'!$G$9:$G$38&lt;&gt;"")+('09 Chantiers'!$H$9:$H$38&lt;&gt;"")+('09 Chantiers'!$I$9:$I$38&lt;&gt;"")+('09 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*('09 Chantiers'!$D$9:$D$38&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('10 Chantiers'!$C$9:$C$38&lt;&gt;"")+('10 Chantiers'!$D$9:$D$38&lt;&gt;"")+('10 Chantiers'!$E$9:$E$38&lt;&gt;"")+('10 Chantiers'!$F$9:$F$38&lt;&gt;"")+('10 Chantiers'!$G$9:$G$38&lt;&gt;"")+('10 Chantiers'!$H$9:$H$38&lt;&gt;"")+('10 Chantiers'!$I$9:$I$38&lt;&gt;"")+('10 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*('10 Chantiers'!$C$9:$C$38&lt;&gt;""))+SUMPRODUCT(((('10 Chantiers'!$C$9:$C$38&lt;&gt;"")+('10 Chantiers'!$D$9:$D$38&lt;&gt;"")+('10 Chantiers'!$E$9:$E$38&lt;&gt;"")+('10 Chantiers'!$F$9:$F$38&lt;&gt;"")+('10 Chantiers'!$G$9:$G$38&lt;&gt;"")+('10 Chantiers'!$H$9:$H$38&lt;&gt;"")+('10 Chantiers'!$I$9:$I$38&lt;&gt;"")+('10 Chantiers'!$J$9:$J$38&lt;&gt;""))&gt;0)*('10 Chantiers'!$D$9:$D$38&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L28" s="21">
@@ -2209,7 +2209,7 @@
     <row r="30" ht="26" customHeight="1">
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="F30" s="17">
-        <f>SUMPRODUCT(((('10 Instances'!$B$9:$B$28&lt;&gt;"")+('10 Instances'!$C$9:$C$28&lt;&gt;"")+('10 Instances'!$D$9:$D$28&lt;&gt;"")+('10 Instances'!$F$9:$F$28&lt;&gt;"")+('10 Instances'!$G$9:$G$28&lt;&gt;"")+('10 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('11 Instances'!$B$9:$B$28&lt;&gt;"")+('11 Instances'!$C$9:$C$28&lt;&gt;"")+('11 Instances'!$D$9:$D$28&lt;&gt;"")+('11 Instances'!$F$9:$F$28&lt;&gt;"")+('11 Instances'!$G$9:$G$28&lt;&gt;"")+('11 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G30" s="18">
@@ -2248,7 +2248,7 @@
         <v/>
       </c>
       <c r="K30" s="21">
-        <f>SUMPRODUCT(((('10 Instances'!$B$9:$B$28&lt;&gt;"")+('10 Instances'!$C$9:$C$28&lt;&gt;"")+('10 Instances'!$D$9:$D$28&lt;&gt;"")+('10 Instances'!$F$9:$F$28&lt;&gt;"")+('10 Instances'!$G$9:$G$28&lt;&gt;"")+('10 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('10 Instances'!$B$9:$B$28&lt;&gt;""))+SUMPRODUCT(((('10 Instances'!$B$9:$B$28&lt;&gt;"")+('10 Instances'!$C$9:$C$28&lt;&gt;"")+('10 Instances'!$D$9:$D$28&lt;&gt;"")+('10 Instances'!$F$9:$F$28&lt;&gt;"")+('10 Instances'!$G$9:$G$28&lt;&gt;"")+('10 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('10 Instances'!$C$9:$C$28&lt;&gt;""))+SUMPRODUCT(((('10 Instances'!$B$9:$B$28&lt;&gt;"")+('10 Instances'!$C$9:$C$28&lt;&gt;"")+('10 Instances'!$D$9:$D$28&lt;&gt;"")+('10 Instances'!$F$9:$F$28&lt;&gt;"")+('10 Instances'!$G$9:$G$28&lt;&gt;"")+('10 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('10 Instances'!$D$9:$D$28&lt;&gt;""))+SUMPRODUCT(((('10 Instances'!$B$9:$B$28&lt;&gt;"")+('10 Instances'!$C$9:$C$28&lt;&gt;"")+('10 Instances'!$D$9:$D$28&lt;&gt;"")+('10 Instances'!$F$9:$F$28&lt;&gt;"")+('10 Instances'!$G$9:$G$28&lt;&gt;"")+('10 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('10 Instances'!$F$9:$F$28&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('11 Instances'!$B$9:$B$28&lt;&gt;"")+('11 Instances'!$C$9:$C$28&lt;&gt;"")+('11 Instances'!$D$9:$D$28&lt;&gt;"")+('11 Instances'!$F$9:$F$28&lt;&gt;"")+('11 Instances'!$G$9:$G$28&lt;&gt;"")+('11 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('11 Instances'!$B$9:$B$28&lt;&gt;""))+SUMPRODUCT(((('11 Instances'!$B$9:$B$28&lt;&gt;"")+('11 Instances'!$C$9:$C$28&lt;&gt;"")+('11 Instances'!$D$9:$D$28&lt;&gt;"")+('11 Instances'!$F$9:$F$28&lt;&gt;"")+('11 Instances'!$G$9:$G$28&lt;&gt;"")+('11 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('11 Instances'!$C$9:$C$28&lt;&gt;""))+SUMPRODUCT(((('11 Instances'!$B$9:$B$28&lt;&gt;"")+('11 Instances'!$C$9:$C$28&lt;&gt;"")+('11 Instances'!$D$9:$D$28&lt;&gt;"")+('11 Instances'!$F$9:$F$28&lt;&gt;"")+('11 Instances'!$G$9:$G$28&lt;&gt;"")+('11 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('11 Instances'!$D$9:$D$28&lt;&gt;""))+SUMPRODUCT(((('11 Instances'!$B$9:$B$28&lt;&gt;"")+('11 Instances'!$C$9:$C$28&lt;&gt;"")+('11 Instances'!$D$9:$D$28&lt;&gt;"")+('11 Instances'!$F$9:$F$28&lt;&gt;"")+('11 Instances'!$G$9:$G$28&lt;&gt;"")+('11 Instances'!$H$9:$H$28&lt;&gt;""))&gt;0)*('11 Instances'!$F$9:$F$28&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L30" s="21">
@@ -2259,7 +2259,7 @@
     <row r="31" ht="26" customHeight="1">
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="F31" s="17">
-        <f>SUMPRODUCT(((('11 Membres'!$B$9:$B$208&lt;&gt;"")+('11 Membres'!$C$9:$C$208&lt;&gt;"")+('11 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('12 Membres'!$B$9:$B$208&lt;&gt;"")+('12 Membres'!$C$9:$C$208&lt;&gt;"")+('12 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G31" s="18">
@@ -2298,7 +2298,7 @@
         <v/>
       </c>
       <c r="K31" s="21">
-        <f>SUMPRODUCT(((('11 Membres'!$B$9:$B$208&lt;&gt;"")+('11 Membres'!$C$9:$C$208&lt;&gt;"")+('11 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*('11 Membres'!$B$9:$B$208&lt;&gt;""))+SUMPRODUCT(((('11 Membres'!$B$9:$B$208&lt;&gt;"")+('11 Membres'!$C$9:$C$208&lt;&gt;"")+('11 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*('11 Membres'!$C$9:$C$208&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('12 Membres'!$B$9:$B$208&lt;&gt;"")+('12 Membres'!$C$9:$C$208&lt;&gt;"")+('12 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*('12 Membres'!$B$9:$B$208&lt;&gt;""))+SUMPRODUCT(((('12 Membres'!$B$9:$B$208&lt;&gt;"")+('12 Membres'!$C$9:$C$208&lt;&gt;"")+('12 Membres'!$D$9:$D$208&lt;&gt;""))&gt;0)*('12 Membres'!$C$9:$C$208&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L31" s="21">
@@ -2316,7 +2316,7 @@
     <row r="33" ht="26" customHeight="1">
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="F33" s="17">
-        <f>SUMPRODUCT(((('12 Jalons'!$C$9:$C$108&lt;&gt;"")+('12 Jalons'!$D$9:$D$108&lt;&gt;"")+('12 Jalons'!$E$9:$E$108&lt;&gt;"")+('12 Jalons'!$F$9:$F$108&lt;&gt;"")+('12 Jalons'!$G$9:$G$108&lt;&gt;"")+('12 Jalons'!$H$9:$H$108&lt;&gt;"")+('12 Jalons'!$I$9:$I$108&lt;&gt;"")+('12 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('13 Jalons'!$C$9:$C$108&lt;&gt;"")+('13 Jalons'!$D$9:$D$108&lt;&gt;"")+('13 Jalons'!$E$9:$E$108&lt;&gt;"")+('13 Jalons'!$F$9:$F$108&lt;&gt;"")+('13 Jalons'!$G$9:$G$108&lt;&gt;"")+('13 Jalons'!$H$9:$H$108&lt;&gt;"")+('13 Jalons'!$I$9:$I$108&lt;&gt;"")+('13 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G33" s="18">
@@ -2355,7 +2355,7 @@
         <v/>
       </c>
       <c r="K33" s="21">
-        <f>SUMPRODUCT(((('12 Jalons'!$C$9:$C$108&lt;&gt;"")+('12 Jalons'!$D$9:$D$108&lt;&gt;"")+('12 Jalons'!$E$9:$E$108&lt;&gt;"")+('12 Jalons'!$F$9:$F$108&lt;&gt;"")+('12 Jalons'!$G$9:$G$108&lt;&gt;"")+('12 Jalons'!$H$9:$H$108&lt;&gt;"")+('12 Jalons'!$I$9:$I$108&lt;&gt;"")+('12 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('12 Jalons'!$C$9:$C$108&lt;&gt;""))+SUMPRODUCT(((('12 Jalons'!$C$9:$C$108&lt;&gt;"")+('12 Jalons'!$D$9:$D$108&lt;&gt;"")+('12 Jalons'!$E$9:$E$108&lt;&gt;"")+('12 Jalons'!$F$9:$F$108&lt;&gt;"")+('12 Jalons'!$G$9:$G$108&lt;&gt;"")+('12 Jalons'!$H$9:$H$108&lt;&gt;"")+('12 Jalons'!$I$9:$I$108&lt;&gt;"")+('12 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('12 Jalons'!$D$9:$D$108&lt;&gt;""))+SUMPRODUCT(((('12 Jalons'!$C$9:$C$108&lt;&gt;"")+('12 Jalons'!$D$9:$D$108&lt;&gt;"")+('12 Jalons'!$E$9:$E$108&lt;&gt;"")+('12 Jalons'!$F$9:$F$108&lt;&gt;"")+('12 Jalons'!$G$9:$G$108&lt;&gt;"")+('12 Jalons'!$H$9:$H$108&lt;&gt;"")+('12 Jalons'!$I$9:$I$108&lt;&gt;"")+('12 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('12 Jalons'!$I$9:$I$108&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('13 Jalons'!$C$9:$C$108&lt;&gt;"")+('13 Jalons'!$D$9:$D$108&lt;&gt;"")+('13 Jalons'!$E$9:$E$108&lt;&gt;"")+('13 Jalons'!$F$9:$F$108&lt;&gt;"")+('13 Jalons'!$G$9:$G$108&lt;&gt;"")+('13 Jalons'!$H$9:$H$108&lt;&gt;"")+('13 Jalons'!$I$9:$I$108&lt;&gt;"")+('13 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('13 Jalons'!$C$9:$C$108&lt;&gt;""))+SUMPRODUCT(((('13 Jalons'!$C$9:$C$108&lt;&gt;"")+('13 Jalons'!$D$9:$D$108&lt;&gt;"")+('13 Jalons'!$E$9:$E$108&lt;&gt;"")+('13 Jalons'!$F$9:$F$108&lt;&gt;"")+('13 Jalons'!$G$9:$G$108&lt;&gt;"")+('13 Jalons'!$H$9:$H$108&lt;&gt;"")+('13 Jalons'!$I$9:$I$108&lt;&gt;"")+('13 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('13 Jalons'!$D$9:$D$108&lt;&gt;""))+SUMPRODUCT(((('13 Jalons'!$C$9:$C$108&lt;&gt;"")+('13 Jalons'!$D$9:$D$108&lt;&gt;"")+('13 Jalons'!$E$9:$E$108&lt;&gt;"")+('13 Jalons'!$F$9:$F$108&lt;&gt;"")+('13 Jalons'!$G$9:$G$108&lt;&gt;"")+('13 Jalons'!$H$9:$H$108&lt;&gt;"")+('13 Jalons'!$I$9:$I$108&lt;&gt;"")+('13 Jalons'!$J$9:$J$108&lt;&gt;""))&gt;0)*('13 Jalons'!$I$9:$I$108&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L33" s="21">
@@ -2366,7 +2366,7 @@
     <row r="34" ht="26" customHeight="1">
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="F34" s="17">
-        <f>SUMPRODUCT(((('13 Livrables'!$B$9:$B$158&lt;&gt;"")+('13 Livrables'!$C$9:$C$158&lt;&gt;"")+('13 Livrables'!$D$9:$D$158&lt;&gt;"")+('13 Livrables'!$E$9:$E$158&lt;&gt;"")+('13 Livrables'!$F$9:$F$158&lt;&gt;"")+('13 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*1)</f>
+        <f>SUMPRODUCT(((('14 Livrables'!$B$9:$B$158&lt;&gt;"")+('14 Livrables'!$C$9:$C$158&lt;&gt;"")+('14 Livrables'!$D$9:$D$158&lt;&gt;"")+('14 Livrables'!$E$9:$E$158&lt;&gt;"")+('14 Livrables'!$F$9:$F$158&lt;&gt;"")+('14 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*1)</f>
         <v/>
       </c>
       <c r="G34" s="18">
@@ -2405,7 +2405,7 @@
         <v/>
       </c>
       <c r="K34" s="21">
-        <f>SUMPRODUCT(((('13 Livrables'!$B$9:$B$158&lt;&gt;"")+('13 Livrables'!$C$9:$C$158&lt;&gt;"")+('13 Livrables'!$D$9:$D$158&lt;&gt;"")+('13 Livrables'!$E$9:$E$158&lt;&gt;"")+('13 Livrables'!$F$9:$F$158&lt;&gt;"")+('13 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('13 Livrables'!$B$9:$B$158&lt;&gt;""))+SUMPRODUCT(((('13 Livrables'!$B$9:$B$158&lt;&gt;"")+('13 Livrables'!$C$9:$C$158&lt;&gt;"")+('13 Livrables'!$D$9:$D$158&lt;&gt;"")+('13 Livrables'!$E$9:$E$158&lt;&gt;"")+('13 Livrables'!$F$9:$F$158&lt;&gt;"")+('13 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('13 Livrables'!$C$9:$C$158&lt;&gt;""))+SUMPRODUCT(((('13 Livrables'!$B$9:$B$158&lt;&gt;"")+('13 Livrables'!$C$9:$C$158&lt;&gt;"")+('13 Livrables'!$D$9:$D$158&lt;&gt;"")+('13 Livrables'!$E$9:$E$158&lt;&gt;"")+('13 Livrables'!$F$9:$F$158&lt;&gt;"")+('13 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('13 Livrables'!$E$9:$E$158&lt;&gt;""))+SUMPRODUCT(((('13 Livrables'!$B$9:$B$158&lt;&gt;"")+('13 Livrables'!$C$9:$C$158&lt;&gt;"")+('13 Livrables'!$D$9:$D$158&lt;&gt;"")+('13 Livrables'!$E$9:$E$158&lt;&gt;"")+('13 Livrables'!$F$9:$F$158&lt;&gt;"")+('13 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('13 Livrables'!$G$9:$G$158&lt;&gt;""))</f>
+        <f>SUMPRODUCT(((('14 Livrables'!$B$9:$B$158&lt;&gt;"")+('14 Livrables'!$C$9:$C$158&lt;&gt;"")+('14 Livrables'!$D$9:$D$158&lt;&gt;"")+('14 Livrables'!$E$9:$E$158&lt;&gt;"")+('14 Livrables'!$F$9:$F$158&lt;&gt;"")+('14 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('14 Livrables'!$B$9:$B$158&lt;&gt;""))+SUMPRODUCT(((('14 Livrables'!$B$9:$B$158&lt;&gt;"")+('14 Livrables'!$C$9:$C$158&lt;&gt;"")+('14 Livrables'!$D$9:$D$158&lt;&gt;"")+('14 Livrables'!$E$9:$E$158&lt;&gt;"")+('14 Livrables'!$F$9:$F$158&lt;&gt;"")+('14 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('14 Livrables'!$C$9:$C$158&lt;&gt;""))+SUMPRODUCT(((('14 Livrables'!$B$9:$B$158&lt;&gt;"")+('14 Livrables'!$C$9:$C$158&lt;&gt;"")+('14 Livrables'!$D$9:$D$158&lt;&gt;"")+('14 Livrables'!$E$9:$E$158&lt;&gt;"")+('14 Livrables'!$F$9:$F$158&lt;&gt;"")+('14 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('14 Livrables'!$E$9:$E$158&lt;&gt;""))+SUMPRODUCT(((('14 Livrables'!$B$9:$B$158&lt;&gt;"")+('14 Livrables'!$C$9:$C$158&lt;&gt;"")+('14 Livrables'!$D$9:$D$158&lt;&gt;"")+('14 Livrables'!$E$9:$E$158&lt;&gt;"")+('14 Livrables'!$F$9:$F$158&lt;&gt;"")+('14 Livrables'!$G$9:$G$158&lt;&gt;""))&gt;0)*('14 Livrables'!$G$9:$G$158&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="L34" s="21">
@@ -2459,20 +2459,20 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" location="#'01 Équipes'!A1" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" location="#'02 Rôles'!A1" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" location="#'03 Personnes'!A1" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" location="#'04 Affectations'!A1" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" location="#'05 Projet'!A1" r:id="rId5"/>
-    <hyperlink ref="C24" location="'05b Info projet'!A1" display="Info projet"/>
-    <hyperlink ref="C25" location="#'06 Lots'!A1" display="Lots"/>
-    <hyperlink ref="C26" location="#'07 Phases'!A1" display="Phases"/>
-    <hyperlink ref="C27" location="#'08 Sous-phases'!A1" display="Sous-phases"/>
-    <hyperlink ref="C28" location="#'09 Chantiers'!A1" display="Chantiers"/>
-    <hyperlink ref="C30" location="#'10 Instances'!A1" display="Instances de pilotage"/>
-    <hyperlink ref="C31" location="#'11 Membres'!A1" display="Membres des instances"/>
-    <hyperlink ref="C33" location="#'12 Jalons'!A1" display="Jalons"/>
-    <hyperlink ref="C34" location="#'13 Livrables'!A1" display="Livrables"/>
+    <hyperlink ref="C18" location="#'01 Équipes'!A1"/>
+    <hyperlink ref="C19" location="#'02 Rôles'!A1"/>
+    <hyperlink ref="C20" location="#'03 Personnes'!A1"/>
+    <hyperlink ref="C21" location="#'04 Affectations'!A1"/>
+    <hyperlink ref="C23" location="#'05 Projet'!A1"/>
+    <hyperlink ref="C24" location="'06 Info projet'!A1" display="Info projet"/>
+    <hyperlink ref="C25" location="#'07 Lots'!A1" display="Lots"/>
+    <hyperlink ref="C26" location="#'08 Phases'!A1" display="Phases"/>
+    <hyperlink ref="C27" location="#'09 Sous-phases'!A1" display="Sous-phases"/>
+    <hyperlink ref="C28" location="#'10 Chantiers'!A1" display="Chantiers"/>
+    <hyperlink ref="C30" location="#'11 Instances'!A1" display="Instances de pilotage"/>
+    <hyperlink ref="C31" location="#'12 Membres'!A1" display="Membres des instances"/>
+    <hyperlink ref="C33" location="#'13 Jalons'!A1" display="Jalons"/>
+    <hyperlink ref="C34" location="#'14 Livrables'!A1" display="Livrables"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2486,7 +2486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:I38"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2541,7 +2541,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 06    </t>
+            <t xml:space="preserve">Étape 07    </t>
           </r>
           <r>
             <rPr>
@@ -3186,7 +3186,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="I3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3200,7 +3200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:J38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3257,7 +3257,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 07    </t>
+            <t xml:space="preserve">Étape 08    </t>
           </r>
           <r>
             <rPr>
@@ -3947,7 +3947,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="J3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3961,7 +3961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:J88"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4018,7 +4018,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 08    </t>
+            <t xml:space="preserve">Étape 09    </t>
           </r>
           <r>
             <rPr>
@@ -4146,7 +4146,7 @@
       <c r="H9" s="46" t="n"/>
       <c r="I9" s="46" t="n"/>
       <c r="J9" s="48">
-        <f>IF(OR(C9="",D9=""),"",IF(LEFT(D9,LEN(LEFT(C9,FIND(" ·",C9&amp;" ·")-1))+1)&lt;&gt;LEFT(C9,FIND(" ·",C9&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F9&lt;&gt;"",G9&lt;&gt;"",G9&lt;F9),"⚠ Fin avant début",IF(AND(F9&lt;&gt;"",IFERROR(F9&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C9,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G9&lt;&gt;"",IFERROR(G9&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C9,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C9="",D9=""),"",IF(LEFT(D9,LEN(LEFT(C9,FIND(" ·",C9&amp;" ·")-1))+1)&lt;&gt;LEFT(C9,FIND(" ·",C9&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F9&lt;&gt;"",G9&lt;&gt;"",G9&lt;F9),"⚠ Fin avant début",IF(AND(F9&lt;&gt;"",IFERROR(F9&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G9&lt;&gt;"",IFERROR(G9&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
       <c r="J10" s="48">
-        <f>IF(OR(C10="",D10=""),"",IF(LEFT(D10,LEN(LEFT(C10,FIND(" ·",C10&amp;" ·")-1))+1)&lt;&gt;LEFT(C10,FIND(" ·",C10&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F10&lt;&gt;"",G10&lt;&gt;"",G10&lt;F10),"⚠ Fin avant début",IF(AND(F10&lt;&gt;"",IFERROR(F10&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C10,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G10&lt;&gt;"",IFERROR(G10&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C10,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C10="",D10=""),"",IF(LEFT(D10,LEN(LEFT(C10,FIND(" ·",C10&amp;" ·")-1))+1)&lt;&gt;LEFT(C10,FIND(" ·",C10&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F10&lt;&gt;"",G10&lt;&gt;"",G10&lt;F10),"⚠ Fin avant début",IF(AND(F10&lt;&gt;"",IFERROR(F10&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G10&lt;&gt;"",IFERROR(G10&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       <c r="H11" s="46" t="n"/>
       <c r="I11" s="46" t="n"/>
       <c r="J11" s="48">
-        <f>IF(OR(C11="",D11=""),"",IF(LEFT(D11,LEN(LEFT(C11,FIND(" ·",C11&amp;" ·")-1))+1)&lt;&gt;LEFT(C11,FIND(" ·",C11&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F11&lt;&gt;"",G11&lt;&gt;"",G11&lt;F11),"⚠ Fin avant début",IF(AND(F11&lt;&gt;"",IFERROR(F11&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C11,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G11&lt;&gt;"",IFERROR(G11&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C11,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C11="",D11=""),"",IF(LEFT(D11,LEN(LEFT(C11,FIND(" ·",C11&amp;" ·")-1))+1)&lt;&gt;LEFT(C11,FIND(" ·",C11&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F11&lt;&gt;"",G11&lt;&gt;"",G11&lt;F11),"⚠ Fin avant début",IF(AND(F11&lt;&gt;"",IFERROR(F11&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G11&lt;&gt;"",IFERROR(G11&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="46" t="n"/>
       <c r="J12" s="48">
-        <f>IF(OR(C12="",D12=""),"",IF(LEFT(D12,LEN(LEFT(C12,FIND(" ·",C12&amp;" ·")-1))+1)&lt;&gt;LEFT(C12,FIND(" ·",C12&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F12&lt;&gt;"",G12&lt;&gt;"",G12&lt;F12),"⚠ Fin avant début",IF(AND(F12&lt;&gt;"",IFERROR(F12&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C12,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G12&lt;&gt;"",IFERROR(G12&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C12,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C12="",D12=""),"",IF(LEFT(D12,LEN(LEFT(C12,FIND(" ·",C12&amp;" ·")-1))+1)&lt;&gt;LEFT(C12,FIND(" ·",C12&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F12&lt;&gt;"",G12&lt;&gt;"",G12&lt;F12),"⚠ Fin avant début",IF(AND(F12&lt;&gt;"",IFERROR(F12&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G12&lt;&gt;"",IFERROR(G12&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       <c r="H13" s="46" t="n"/>
       <c r="I13" s="46" t="n"/>
       <c r="J13" s="48">
-        <f>IF(OR(C13="",D13=""),"",IF(LEFT(D13,LEN(LEFT(C13,FIND(" ·",C13&amp;" ·")-1))+1)&lt;&gt;LEFT(C13,FIND(" ·",C13&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F13&lt;&gt;"",G13&lt;&gt;"",G13&lt;F13),"⚠ Fin avant début",IF(AND(F13&lt;&gt;"",IFERROR(F13&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C13,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G13&lt;&gt;"",IFERROR(G13&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C13,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C13="",D13=""),"",IF(LEFT(D13,LEN(LEFT(C13,FIND(" ·",C13&amp;" ·")-1))+1)&lt;&gt;LEFT(C13,FIND(" ·",C13&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F13&lt;&gt;"",G13&lt;&gt;"",G13&lt;F13),"⚠ Fin avant début",IF(AND(F13&lt;&gt;"",IFERROR(F13&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G13&lt;&gt;"",IFERROR(G13&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
       <c r="J14" s="48">
-        <f>IF(OR(C14="",D14=""),"",IF(LEFT(D14,LEN(LEFT(C14,FIND(" ·",C14&amp;" ·")-1))+1)&lt;&gt;LEFT(C14,FIND(" ·",C14&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F14&lt;&gt;"",G14&lt;&gt;"",G14&lt;F14),"⚠ Fin avant début",IF(AND(F14&lt;&gt;"",IFERROR(F14&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C14,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G14&lt;&gt;"",IFERROR(G14&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C14,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C14="",D14=""),"",IF(LEFT(D14,LEN(LEFT(C14,FIND(" ·",C14&amp;" ·")-1))+1)&lt;&gt;LEFT(C14,FIND(" ·",C14&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F14&lt;&gt;"",G14&lt;&gt;"",G14&lt;F14),"⚠ Fin avant début",IF(AND(F14&lt;&gt;"",IFERROR(F14&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G14&lt;&gt;"",IFERROR(G14&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="46" t="n"/>
       <c r="J15" s="48">
-        <f>IF(OR(C15="",D15=""),"",IF(LEFT(D15,LEN(LEFT(C15,FIND(" ·",C15&amp;" ·")-1))+1)&lt;&gt;LEFT(C15,FIND(" ·",C15&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F15&lt;&gt;"",G15&lt;&gt;"",G15&lt;F15),"⚠ Fin avant début",IF(AND(F15&lt;&gt;"",IFERROR(F15&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C15,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G15&lt;&gt;"",IFERROR(G15&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C15,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C15="",D15=""),"",IF(LEFT(D15,LEN(LEFT(C15,FIND(" ·",C15&amp;" ·")-1))+1)&lt;&gt;LEFT(C15,FIND(" ·",C15&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F15&lt;&gt;"",G15&lt;&gt;"",G15&lt;F15),"⚠ Fin avant début",IF(AND(F15&lt;&gt;"",IFERROR(F15&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G15&lt;&gt;"",IFERROR(G15&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
       <c r="H16" s="46" t="n"/>
       <c r="I16" s="46" t="n"/>
       <c r="J16" s="48">
-        <f>IF(OR(C16="",D16=""),"",IF(LEFT(D16,LEN(LEFT(C16,FIND(" ·",C16&amp;" ·")-1))+1)&lt;&gt;LEFT(C16,FIND(" ·",C16&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F16&lt;&gt;"",G16&lt;&gt;"",G16&lt;F16),"⚠ Fin avant début",IF(AND(F16&lt;&gt;"",IFERROR(F16&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C16,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G16&lt;&gt;"",IFERROR(G16&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C16,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C16="",D16=""),"",IF(LEFT(D16,LEN(LEFT(C16,FIND(" ·",C16&amp;" ·")-1))+1)&lt;&gt;LEFT(C16,FIND(" ·",C16&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F16&lt;&gt;"",G16&lt;&gt;"",G16&lt;F16),"⚠ Fin avant début",IF(AND(F16&lt;&gt;"",IFERROR(F16&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G16&lt;&gt;"",IFERROR(G16&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       <c r="H17" s="46" t="n"/>
       <c r="I17" s="46" t="n"/>
       <c r="J17" s="48">
-        <f>IF(OR(C17="",D17=""),"",IF(LEFT(D17,LEN(LEFT(C17,FIND(" ·",C17&amp;" ·")-1))+1)&lt;&gt;LEFT(C17,FIND(" ·",C17&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F17&lt;&gt;"",G17&lt;&gt;"",G17&lt;F17),"⚠ Fin avant début",IF(AND(F17&lt;&gt;"",IFERROR(F17&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C17,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G17&lt;&gt;"",IFERROR(G17&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C17,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C17="",D17=""),"",IF(LEFT(D17,LEN(LEFT(C17,FIND(" ·",C17&amp;" ·")-1))+1)&lt;&gt;LEFT(C17,FIND(" ·",C17&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F17&lt;&gt;"",G17&lt;&gt;"",G17&lt;F17),"⚠ Fin avant début",IF(AND(F17&lt;&gt;"",IFERROR(F17&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G17&lt;&gt;"",IFERROR(G17&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4299,7 +4299,7 @@
       <c r="H18" s="46" t="n"/>
       <c r="I18" s="46" t="n"/>
       <c r="J18" s="48">
-        <f>IF(OR(C18="",D18=""),"",IF(LEFT(D18,LEN(LEFT(C18,FIND(" ·",C18&amp;" ·")-1))+1)&lt;&gt;LEFT(C18,FIND(" ·",C18&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F18&lt;&gt;"",G18&lt;&gt;"",G18&lt;F18),"⚠ Fin avant début",IF(AND(F18&lt;&gt;"",IFERROR(F18&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C18,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G18&lt;&gt;"",IFERROR(G18&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C18,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C18="",D18=""),"",IF(LEFT(D18,LEN(LEFT(C18,FIND(" ·",C18&amp;" ·")-1))+1)&lt;&gt;LEFT(C18,FIND(" ·",C18&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F18&lt;&gt;"",G18&lt;&gt;"",G18&lt;F18),"⚠ Fin avant début",IF(AND(F18&lt;&gt;"",IFERROR(F18&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G18&lt;&gt;"",IFERROR(G18&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4316,7 +4316,7 @@
       <c r="H19" s="46" t="n"/>
       <c r="I19" s="46" t="n"/>
       <c r="J19" s="48">
-        <f>IF(OR(C19="",D19=""),"",IF(LEFT(D19,LEN(LEFT(C19,FIND(" ·",C19&amp;" ·")-1))+1)&lt;&gt;LEFT(C19,FIND(" ·",C19&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F19&lt;&gt;"",G19&lt;&gt;"",G19&lt;F19),"⚠ Fin avant début",IF(AND(F19&lt;&gt;"",IFERROR(F19&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C19,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G19&lt;&gt;"",IFERROR(G19&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C19,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C19="",D19=""),"",IF(LEFT(D19,LEN(LEFT(C19,FIND(" ·",C19&amp;" ·")-1))+1)&lt;&gt;LEFT(C19,FIND(" ·",C19&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F19&lt;&gt;"",G19&lt;&gt;"",G19&lt;F19),"⚠ Fin avant début",IF(AND(F19&lt;&gt;"",IFERROR(F19&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G19&lt;&gt;"",IFERROR(G19&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       <c r="H20" s="46" t="n"/>
       <c r="I20" s="46" t="n"/>
       <c r="J20" s="48">
-        <f>IF(OR(C20="",D20=""),"",IF(LEFT(D20,LEN(LEFT(C20,FIND(" ·",C20&amp;" ·")-1))+1)&lt;&gt;LEFT(C20,FIND(" ·",C20&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F20&lt;&gt;"",G20&lt;&gt;"",G20&lt;F20),"⚠ Fin avant début",IF(AND(F20&lt;&gt;"",IFERROR(F20&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C20,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G20&lt;&gt;"",IFERROR(G20&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C20,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C20="",D20=""),"",IF(LEFT(D20,LEN(LEFT(C20,FIND(" ·",C20&amp;" ·")-1))+1)&lt;&gt;LEFT(C20,FIND(" ·",C20&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F20&lt;&gt;"",G20&lt;&gt;"",G20&lt;F20),"⚠ Fin avant début",IF(AND(F20&lt;&gt;"",IFERROR(F20&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G20&lt;&gt;"",IFERROR(G20&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4350,7 +4350,7 @@
       <c r="H21" s="46" t="n"/>
       <c r="I21" s="46" t="n"/>
       <c r="J21" s="48">
-        <f>IF(OR(C21="",D21=""),"",IF(LEFT(D21,LEN(LEFT(C21,FIND(" ·",C21&amp;" ·")-1))+1)&lt;&gt;LEFT(C21,FIND(" ·",C21&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F21&lt;&gt;"",G21&lt;&gt;"",G21&lt;F21),"⚠ Fin avant début",IF(AND(F21&lt;&gt;"",IFERROR(F21&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C21,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G21&lt;&gt;"",IFERROR(G21&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C21,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C21="",D21=""),"",IF(LEFT(D21,LEN(LEFT(C21,FIND(" ·",C21&amp;" ·")-1))+1)&lt;&gt;LEFT(C21,FIND(" ·",C21&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F21&lt;&gt;"",G21&lt;&gt;"",G21&lt;F21),"⚠ Fin avant début",IF(AND(F21&lt;&gt;"",IFERROR(F21&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G21&lt;&gt;"",IFERROR(G21&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       <c r="H22" s="46" t="n"/>
       <c r="I22" s="46" t="n"/>
       <c r="J22" s="48">
-        <f>IF(OR(C22="",D22=""),"",IF(LEFT(D22,LEN(LEFT(C22,FIND(" ·",C22&amp;" ·")-1))+1)&lt;&gt;LEFT(C22,FIND(" ·",C22&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F22&lt;&gt;"",G22&lt;&gt;"",G22&lt;F22),"⚠ Fin avant début",IF(AND(F22&lt;&gt;"",IFERROR(F22&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C22,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G22&lt;&gt;"",IFERROR(G22&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C22,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C22="",D22=""),"",IF(LEFT(D22,LEN(LEFT(C22,FIND(" ·",C22&amp;" ·")-1))+1)&lt;&gt;LEFT(C22,FIND(" ·",C22&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F22&lt;&gt;"",G22&lt;&gt;"",G22&lt;F22),"⚠ Fin avant début",IF(AND(F22&lt;&gt;"",IFERROR(F22&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G22&lt;&gt;"",IFERROR(G22&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4384,7 +4384,7 @@
       <c r="H23" s="46" t="n"/>
       <c r="I23" s="46" t="n"/>
       <c r="J23" s="48">
-        <f>IF(OR(C23="",D23=""),"",IF(LEFT(D23,LEN(LEFT(C23,FIND(" ·",C23&amp;" ·")-1))+1)&lt;&gt;LEFT(C23,FIND(" ·",C23&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F23&lt;&gt;"",G23&lt;&gt;"",G23&lt;F23),"⚠ Fin avant début",IF(AND(F23&lt;&gt;"",IFERROR(F23&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C23,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G23&lt;&gt;"",IFERROR(G23&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C23,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C23="",D23=""),"",IF(LEFT(D23,LEN(LEFT(C23,FIND(" ·",C23&amp;" ·")-1))+1)&lt;&gt;LEFT(C23,FIND(" ·",C23&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F23&lt;&gt;"",G23&lt;&gt;"",G23&lt;F23),"⚠ Fin avant début",IF(AND(F23&lt;&gt;"",IFERROR(F23&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G23&lt;&gt;"",IFERROR(G23&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       <c r="H24" s="46" t="n"/>
       <c r="I24" s="46" t="n"/>
       <c r="J24" s="48">
-        <f>IF(OR(C24="",D24=""),"",IF(LEFT(D24,LEN(LEFT(C24,FIND(" ·",C24&amp;" ·")-1))+1)&lt;&gt;LEFT(C24,FIND(" ·",C24&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F24&lt;&gt;"",G24&lt;&gt;"",G24&lt;F24),"⚠ Fin avant début",IF(AND(F24&lt;&gt;"",IFERROR(F24&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C24,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G24&lt;&gt;"",IFERROR(G24&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C24,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C24="",D24=""),"",IF(LEFT(D24,LEN(LEFT(C24,FIND(" ·",C24&amp;" ·")-1))+1)&lt;&gt;LEFT(C24,FIND(" ·",C24&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F24&lt;&gt;"",G24&lt;&gt;"",G24&lt;F24),"⚠ Fin avant début",IF(AND(F24&lt;&gt;"",IFERROR(F24&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G24&lt;&gt;"",IFERROR(G24&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4418,7 +4418,7 @@
       <c r="H25" s="46" t="n"/>
       <c r="I25" s="46" t="n"/>
       <c r="J25" s="48">
-        <f>IF(OR(C25="",D25=""),"",IF(LEFT(D25,LEN(LEFT(C25,FIND(" ·",C25&amp;" ·")-1))+1)&lt;&gt;LEFT(C25,FIND(" ·",C25&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F25&lt;&gt;"",G25&lt;&gt;"",G25&lt;F25),"⚠ Fin avant début",IF(AND(F25&lt;&gt;"",IFERROR(F25&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C25,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G25&lt;&gt;"",IFERROR(G25&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C25,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C25="",D25=""),"",IF(LEFT(D25,LEN(LEFT(C25,FIND(" ·",C25&amp;" ·")-1))+1)&lt;&gt;LEFT(C25,FIND(" ·",C25&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F25&lt;&gt;"",G25&lt;&gt;"",G25&lt;F25),"⚠ Fin avant début",IF(AND(F25&lt;&gt;"",IFERROR(F25&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G25&lt;&gt;"",IFERROR(G25&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       <c r="H26" s="46" t="n"/>
       <c r="I26" s="46" t="n"/>
       <c r="J26" s="48">
-        <f>IF(OR(C26="",D26=""),"",IF(LEFT(D26,LEN(LEFT(C26,FIND(" ·",C26&amp;" ·")-1))+1)&lt;&gt;LEFT(C26,FIND(" ·",C26&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F26&lt;&gt;"",G26&lt;&gt;"",G26&lt;F26),"⚠ Fin avant début",IF(AND(F26&lt;&gt;"",IFERROR(F26&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C26,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G26&lt;&gt;"",IFERROR(G26&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C26,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C26="",D26=""),"",IF(LEFT(D26,LEN(LEFT(C26,FIND(" ·",C26&amp;" ·")-1))+1)&lt;&gt;LEFT(C26,FIND(" ·",C26&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F26&lt;&gt;"",G26&lt;&gt;"",G26&lt;F26),"⚠ Fin avant début",IF(AND(F26&lt;&gt;"",IFERROR(F26&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G26&lt;&gt;"",IFERROR(G26&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       <c r="H27" s="46" t="n"/>
       <c r="I27" s="46" t="n"/>
       <c r="J27" s="48">
-        <f>IF(OR(C27="",D27=""),"",IF(LEFT(D27,LEN(LEFT(C27,FIND(" ·",C27&amp;" ·")-1))+1)&lt;&gt;LEFT(C27,FIND(" ·",C27&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F27&lt;&gt;"",G27&lt;&gt;"",G27&lt;F27),"⚠ Fin avant début",IF(AND(F27&lt;&gt;"",IFERROR(F27&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C27,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G27&lt;&gt;"",IFERROR(G27&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C27,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C27="",D27=""),"",IF(LEFT(D27,LEN(LEFT(C27,FIND(" ·",C27&amp;" ·")-1))+1)&lt;&gt;LEFT(C27,FIND(" ·",C27&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F27&lt;&gt;"",G27&lt;&gt;"",G27&lt;F27),"⚠ Fin avant début",IF(AND(F27&lt;&gt;"",IFERROR(F27&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G27&lt;&gt;"",IFERROR(G27&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
       <c r="H28" s="46" t="n"/>
       <c r="I28" s="46" t="n"/>
       <c r="J28" s="48">
-        <f>IF(OR(C28="",D28=""),"",IF(LEFT(D28,LEN(LEFT(C28,FIND(" ·",C28&amp;" ·")-1))+1)&lt;&gt;LEFT(C28,FIND(" ·",C28&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F28&lt;&gt;"",G28&lt;&gt;"",G28&lt;F28),"⚠ Fin avant début",IF(AND(F28&lt;&gt;"",IFERROR(F28&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C28,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G28&lt;&gt;"",IFERROR(G28&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C28,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C28="",D28=""),"",IF(LEFT(D28,LEN(LEFT(C28,FIND(" ·",C28&amp;" ·")-1))+1)&lt;&gt;LEFT(C28,FIND(" ·",C28&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F28&lt;&gt;"",G28&lt;&gt;"",G28&lt;F28),"⚠ Fin avant début",IF(AND(F28&lt;&gt;"",IFERROR(F28&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G28&lt;&gt;"",IFERROR(G28&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       <c r="H29" s="46" t="n"/>
       <c r="I29" s="46" t="n"/>
       <c r="J29" s="48">
-        <f>IF(OR(C29="",D29=""),"",IF(LEFT(D29,LEN(LEFT(C29,FIND(" ·",C29&amp;" ·")-1))+1)&lt;&gt;LEFT(C29,FIND(" ·",C29&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F29&lt;&gt;"",G29&lt;&gt;"",G29&lt;F29),"⚠ Fin avant début",IF(AND(F29&lt;&gt;"",IFERROR(F29&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C29,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G29&lt;&gt;"",IFERROR(G29&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C29,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C29="",D29=""),"",IF(LEFT(D29,LEN(LEFT(C29,FIND(" ·",C29&amp;" ·")-1))+1)&lt;&gt;LEFT(C29,FIND(" ·",C29&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F29&lt;&gt;"",G29&lt;&gt;"",G29&lt;F29),"⚠ Fin avant début",IF(AND(F29&lt;&gt;"",IFERROR(F29&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G29&lt;&gt;"",IFERROR(G29&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       <c r="H30" s="46" t="n"/>
       <c r="I30" s="46" t="n"/>
       <c r="J30" s="48">
-        <f>IF(OR(C30="",D30=""),"",IF(LEFT(D30,LEN(LEFT(C30,FIND(" ·",C30&amp;" ·")-1))+1)&lt;&gt;LEFT(C30,FIND(" ·",C30&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F30&lt;&gt;"",G30&lt;&gt;"",G30&lt;F30),"⚠ Fin avant début",IF(AND(F30&lt;&gt;"",IFERROR(F30&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C30,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G30&lt;&gt;"",IFERROR(G30&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C30,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C30="",D30=""),"",IF(LEFT(D30,LEN(LEFT(C30,FIND(" ·",C30&amp;" ·")-1))+1)&lt;&gt;LEFT(C30,FIND(" ·",C30&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F30&lt;&gt;"",G30&lt;&gt;"",G30&lt;F30),"⚠ Fin avant début",IF(AND(F30&lt;&gt;"",IFERROR(F30&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G30&lt;&gt;"",IFERROR(G30&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       <c r="H31" s="46" t="n"/>
       <c r="I31" s="46" t="n"/>
       <c r="J31" s="48">
-        <f>IF(OR(C31="",D31=""),"",IF(LEFT(D31,LEN(LEFT(C31,FIND(" ·",C31&amp;" ·")-1))+1)&lt;&gt;LEFT(C31,FIND(" ·",C31&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F31&lt;&gt;"",G31&lt;&gt;"",G31&lt;F31),"⚠ Fin avant début",IF(AND(F31&lt;&gt;"",IFERROR(F31&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C31,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G31&lt;&gt;"",IFERROR(G31&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C31,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C31="",D31=""),"",IF(LEFT(D31,LEN(LEFT(C31,FIND(" ·",C31&amp;" ·")-1))+1)&lt;&gt;LEFT(C31,FIND(" ·",C31&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F31&lt;&gt;"",G31&lt;&gt;"",G31&lt;F31),"⚠ Fin avant début",IF(AND(F31&lt;&gt;"",IFERROR(F31&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G31&lt;&gt;"",IFERROR(G31&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       <c r="H32" s="46" t="n"/>
       <c r="I32" s="46" t="n"/>
       <c r="J32" s="48">
-        <f>IF(OR(C32="",D32=""),"",IF(LEFT(D32,LEN(LEFT(C32,FIND(" ·",C32&amp;" ·")-1))+1)&lt;&gt;LEFT(C32,FIND(" ·",C32&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F32&lt;&gt;"",G32&lt;&gt;"",G32&lt;F32),"⚠ Fin avant début",IF(AND(F32&lt;&gt;"",IFERROR(F32&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C32,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G32&lt;&gt;"",IFERROR(G32&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C32,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C32="",D32=""),"",IF(LEFT(D32,LEN(LEFT(C32,FIND(" ·",C32&amp;" ·")-1))+1)&lt;&gt;LEFT(C32,FIND(" ·",C32&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F32&lt;&gt;"",G32&lt;&gt;"",G32&lt;F32),"⚠ Fin avant début",IF(AND(F32&lt;&gt;"",IFERROR(F32&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G32&lt;&gt;"",IFERROR(G32&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       <c r="H33" s="46" t="n"/>
       <c r="I33" s="46" t="n"/>
       <c r="J33" s="48">
-        <f>IF(OR(C33="",D33=""),"",IF(LEFT(D33,LEN(LEFT(C33,FIND(" ·",C33&amp;" ·")-1))+1)&lt;&gt;LEFT(C33,FIND(" ·",C33&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F33&lt;&gt;"",G33&lt;&gt;"",G33&lt;F33),"⚠ Fin avant début",IF(AND(F33&lt;&gt;"",IFERROR(F33&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C33,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G33&lt;&gt;"",IFERROR(G33&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C33,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C33="",D33=""),"",IF(LEFT(D33,LEN(LEFT(C33,FIND(" ·",C33&amp;" ·")-1))+1)&lt;&gt;LEFT(C33,FIND(" ·",C33&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F33&lt;&gt;"",G33&lt;&gt;"",G33&lt;F33),"⚠ Fin avant début",IF(AND(F33&lt;&gt;"",IFERROR(F33&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G33&lt;&gt;"",IFERROR(G33&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       <c r="H34" s="46" t="n"/>
       <c r="I34" s="46" t="n"/>
       <c r="J34" s="48">
-        <f>IF(OR(C34="",D34=""),"",IF(LEFT(D34,LEN(LEFT(C34,FIND(" ·",C34&amp;" ·")-1))+1)&lt;&gt;LEFT(C34,FIND(" ·",C34&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F34&lt;&gt;"",G34&lt;&gt;"",G34&lt;F34),"⚠ Fin avant début",IF(AND(F34&lt;&gt;"",IFERROR(F34&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C34,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G34&lt;&gt;"",IFERROR(G34&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C34,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C34="",D34=""),"",IF(LEFT(D34,LEN(LEFT(C34,FIND(" ·",C34&amp;" ·")-1))+1)&lt;&gt;LEFT(C34,FIND(" ·",C34&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F34&lt;&gt;"",G34&lt;&gt;"",G34&lt;F34),"⚠ Fin avant début",IF(AND(F34&lt;&gt;"",IFERROR(F34&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G34&lt;&gt;"",IFERROR(G34&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       <c r="H35" s="46" t="n"/>
       <c r="I35" s="46" t="n"/>
       <c r="J35" s="48">
-        <f>IF(OR(C35="",D35=""),"",IF(LEFT(D35,LEN(LEFT(C35,FIND(" ·",C35&amp;" ·")-1))+1)&lt;&gt;LEFT(C35,FIND(" ·",C35&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F35&lt;&gt;"",G35&lt;&gt;"",G35&lt;F35),"⚠ Fin avant début",IF(AND(F35&lt;&gt;"",IFERROR(F35&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C35,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G35&lt;&gt;"",IFERROR(G35&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C35,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C35="",D35=""),"",IF(LEFT(D35,LEN(LEFT(C35,FIND(" ·",C35&amp;" ·")-1))+1)&lt;&gt;LEFT(C35,FIND(" ·",C35&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F35&lt;&gt;"",G35&lt;&gt;"",G35&lt;F35),"⚠ Fin avant début",IF(AND(F35&lt;&gt;"",IFERROR(F35&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G35&lt;&gt;"",IFERROR(G35&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
       <c r="H36" s="46" t="n"/>
       <c r="I36" s="46" t="n"/>
       <c r="J36" s="48">
-        <f>IF(OR(C36="",D36=""),"",IF(LEFT(D36,LEN(LEFT(C36,FIND(" ·",C36&amp;" ·")-1))+1)&lt;&gt;LEFT(C36,FIND(" ·",C36&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F36&lt;&gt;"",G36&lt;&gt;"",G36&lt;F36),"⚠ Fin avant début",IF(AND(F36&lt;&gt;"",IFERROR(F36&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C36,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G36&lt;&gt;"",IFERROR(G36&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C36,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C36="",D36=""),"",IF(LEFT(D36,LEN(LEFT(C36,FIND(" ·",C36&amp;" ·")-1))+1)&lt;&gt;LEFT(C36,FIND(" ·",C36&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F36&lt;&gt;"",G36&lt;&gt;"",G36&lt;F36),"⚠ Fin avant début",IF(AND(F36&lt;&gt;"",IFERROR(F36&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G36&lt;&gt;"",IFERROR(G36&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4622,7 +4622,7 @@
       <c r="H37" s="46" t="n"/>
       <c r="I37" s="46" t="n"/>
       <c r="J37" s="48">
-        <f>IF(OR(C37="",D37=""),"",IF(LEFT(D37,LEN(LEFT(C37,FIND(" ·",C37&amp;" ·")-1))+1)&lt;&gt;LEFT(C37,FIND(" ·",C37&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F37&lt;&gt;"",G37&lt;&gt;"",G37&lt;F37),"⚠ Fin avant début",IF(AND(F37&lt;&gt;"",IFERROR(F37&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C37,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G37&lt;&gt;"",IFERROR(G37&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C37,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C37="",D37=""),"",IF(LEFT(D37,LEN(LEFT(C37,FIND(" ·",C37&amp;" ·")-1))+1)&lt;&gt;LEFT(C37,FIND(" ·",C37&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F37&lt;&gt;"",G37&lt;&gt;"",G37&lt;F37),"⚠ Fin avant début",IF(AND(F37&lt;&gt;"",IFERROR(F37&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G37&lt;&gt;"",IFERROR(G37&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4639,7 +4639,7 @@
       <c r="H38" s="46" t="n"/>
       <c r="I38" s="46" t="n"/>
       <c r="J38" s="48">
-        <f>IF(OR(C38="",D38=""),"",IF(LEFT(D38,LEN(LEFT(C38,FIND(" ·",C38&amp;" ·")-1))+1)&lt;&gt;LEFT(C38,FIND(" ·",C38&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F38&lt;&gt;"",G38&lt;&gt;"",G38&lt;F38),"⚠ Fin avant début",IF(AND(F38&lt;&gt;"",IFERROR(F38&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C38,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G38&lt;&gt;"",IFERROR(G38&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C38,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C38="",D38=""),"",IF(LEFT(D38,LEN(LEFT(C38,FIND(" ·",C38&amp;" ·")-1))+1)&lt;&gt;LEFT(C38,FIND(" ·",C38&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F38&lt;&gt;"",G38&lt;&gt;"",G38&lt;F38),"⚠ Fin avant début",IF(AND(F38&lt;&gt;"",IFERROR(F38&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G38&lt;&gt;"",IFERROR(G38&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
       <c r="H39" s="46" t="n"/>
       <c r="I39" s="46" t="n"/>
       <c r="J39" s="48">
-        <f>IF(OR(C39="",D39=""),"",IF(LEFT(D39,LEN(LEFT(C39,FIND(" ·",C39&amp;" ·")-1))+1)&lt;&gt;LEFT(C39,FIND(" ·",C39&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F39&lt;&gt;"",G39&lt;&gt;"",G39&lt;F39),"⚠ Fin avant début",IF(AND(F39&lt;&gt;"",IFERROR(F39&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C39,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G39&lt;&gt;"",IFERROR(G39&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C39,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C39="",D39=""),"",IF(LEFT(D39,LEN(LEFT(C39,FIND(" ·",C39&amp;" ·")-1))+1)&lt;&gt;LEFT(C39,FIND(" ·",C39&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F39&lt;&gt;"",G39&lt;&gt;"",G39&lt;F39),"⚠ Fin avant début",IF(AND(F39&lt;&gt;"",IFERROR(F39&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G39&lt;&gt;"",IFERROR(G39&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       <c r="H40" s="46" t="n"/>
       <c r="I40" s="46" t="n"/>
       <c r="J40" s="48">
-        <f>IF(OR(C40="",D40=""),"",IF(LEFT(D40,LEN(LEFT(C40,FIND(" ·",C40&amp;" ·")-1))+1)&lt;&gt;LEFT(C40,FIND(" ·",C40&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F40&lt;&gt;"",G40&lt;&gt;"",G40&lt;F40),"⚠ Fin avant début",IF(AND(F40&lt;&gt;"",IFERROR(F40&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C40,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G40&lt;&gt;"",IFERROR(G40&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C40,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C40="",D40=""),"",IF(LEFT(D40,LEN(LEFT(C40,FIND(" ·",C40&amp;" ·")-1))+1)&lt;&gt;LEFT(C40,FIND(" ·",C40&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F40&lt;&gt;"",G40&lt;&gt;"",G40&lt;F40),"⚠ Fin avant début",IF(AND(F40&lt;&gt;"",IFERROR(F40&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G40&lt;&gt;"",IFERROR(G40&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       <c r="H41" s="46" t="n"/>
       <c r="I41" s="46" t="n"/>
       <c r="J41" s="48">
-        <f>IF(OR(C41="",D41=""),"",IF(LEFT(D41,LEN(LEFT(C41,FIND(" ·",C41&amp;" ·")-1))+1)&lt;&gt;LEFT(C41,FIND(" ·",C41&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F41&lt;&gt;"",G41&lt;&gt;"",G41&lt;F41),"⚠ Fin avant début",IF(AND(F41&lt;&gt;"",IFERROR(F41&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C41,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G41&lt;&gt;"",IFERROR(G41&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C41,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C41="",D41=""),"",IF(LEFT(D41,LEN(LEFT(C41,FIND(" ·",C41&amp;" ·")-1))+1)&lt;&gt;LEFT(C41,FIND(" ·",C41&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F41&lt;&gt;"",G41&lt;&gt;"",G41&lt;F41),"⚠ Fin avant début",IF(AND(F41&lt;&gt;"",IFERROR(F41&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G41&lt;&gt;"",IFERROR(G41&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4707,7 +4707,7 @@
       <c r="H42" s="46" t="n"/>
       <c r="I42" s="46" t="n"/>
       <c r="J42" s="48">
-        <f>IF(OR(C42="",D42=""),"",IF(LEFT(D42,LEN(LEFT(C42,FIND(" ·",C42&amp;" ·")-1))+1)&lt;&gt;LEFT(C42,FIND(" ·",C42&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F42&lt;&gt;"",G42&lt;&gt;"",G42&lt;F42),"⚠ Fin avant début",IF(AND(F42&lt;&gt;"",IFERROR(F42&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C42,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G42&lt;&gt;"",IFERROR(G42&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C42,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C42="",D42=""),"",IF(LEFT(D42,LEN(LEFT(C42,FIND(" ·",C42&amp;" ·")-1))+1)&lt;&gt;LEFT(C42,FIND(" ·",C42&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F42&lt;&gt;"",G42&lt;&gt;"",G42&lt;F42),"⚠ Fin avant début",IF(AND(F42&lt;&gt;"",IFERROR(F42&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G42&lt;&gt;"",IFERROR(G42&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       <c r="H43" s="46" t="n"/>
       <c r="I43" s="46" t="n"/>
       <c r="J43" s="48">
-        <f>IF(OR(C43="",D43=""),"",IF(LEFT(D43,LEN(LEFT(C43,FIND(" ·",C43&amp;" ·")-1))+1)&lt;&gt;LEFT(C43,FIND(" ·",C43&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F43&lt;&gt;"",G43&lt;&gt;"",G43&lt;F43),"⚠ Fin avant début",IF(AND(F43&lt;&gt;"",IFERROR(F43&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C43,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G43&lt;&gt;"",IFERROR(G43&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C43,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C43="",D43=""),"",IF(LEFT(D43,LEN(LEFT(C43,FIND(" ·",C43&amp;" ·")-1))+1)&lt;&gt;LEFT(C43,FIND(" ·",C43&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F43&lt;&gt;"",G43&lt;&gt;"",G43&lt;F43),"⚠ Fin avant début",IF(AND(F43&lt;&gt;"",IFERROR(F43&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G43&lt;&gt;"",IFERROR(G43&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       <c r="H44" s="46" t="n"/>
       <c r="I44" s="46" t="n"/>
       <c r="J44" s="48">
-        <f>IF(OR(C44="",D44=""),"",IF(LEFT(D44,LEN(LEFT(C44,FIND(" ·",C44&amp;" ·")-1))+1)&lt;&gt;LEFT(C44,FIND(" ·",C44&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F44&lt;&gt;"",G44&lt;&gt;"",G44&lt;F44),"⚠ Fin avant début",IF(AND(F44&lt;&gt;"",IFERROR(F44&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C44,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G44&lt;&gt;"",IFERROR(G44&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C44,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C44="",D44=""),"",IF(LEFT(D44,LEN(LEFT(C44,FIND(" ·",C44&amp;" ·")-1))+1)&lt;&gt;LEFT(C44,FIND(" ·",C44&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F44&lt;&gt;"",G44&lt;&gt;"",G44&lt;F44),"⚠ Fin avant début",IF(AND(F44&lt;&gt;"",IFERROR(F44&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G44&lt;&gt;"",IFERROR(G44&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       <c r="H45" s="46" t="n"/>
       <c r="I45" s="46" t="n"/>
       <c r="J45" s="48">
-        <f>IF(OR(C45="",D45=""),"",IF(LEFT(D45,LEN(LEFT(C45,FIND(" ·",C45&amp;" ·")-1))+1)&lt;&gt;LEFT(C45,FIND(" ·",C45&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F45&lt;&gt;"",G45&lt;&gt;"",G45&lt;F45),"⚠ Fin avant début",IF(AND(F45&lt;&gt;"",IFERROR(F45&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C45,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G45&lt;&gt;"",IFERROR(G45&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C45,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C45="",D45=""),"",IF(LEFT(D45,LEN(LEFT(C45,FIND(" ·",C45&amp;" ·")-1))+1)&lt;&gt;LEFT(C45,FIND(" ·",C45&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F45&lt;&gt;"",G45&lt;&gt;"",G45&lt;F45),"⚠ Fin avant début",IF(AND(F45&lt;&gt;"",IFERROR(F45&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G45&lt;&gt;"",IFERROR(G45&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4775,7 +4775,7 @@
       <c r="H46" s="46" t="n"/>
       <c r="I46" s="46" t="n"/>
       <c r="J46" s="48">
-        <f>IF(OR(C46="",D46=""),"",IF(LEFT(D46,LEN(LEFT(C46,FIND(" ·",C46&amp;" ·")-1))+1)&lt;&gt;LEFT(C46,FIND(" ·",C46&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F46&lt;&gt;"",G46&lt;&gt;"",G46&lt;F46),"⚠ Fin avant début",IF(AND(F46&lt;&gt;"",IFERROR(F46&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C46,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G46&lt;&gt;"",IFERROR(G46&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C46,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C46="",D46=""),"",IF(LEFT(D46,LEN(LEFT(C46,FIND(" ·",C46&amp;" ·")-1))+1)&lt;&gt;LEFT(C46,FIND(" ·",C46&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F46&lt;&gt;"",G46&lt;&gt;"",G46&lt;F46),"⚠ Fin avant début",IF(AND(F46&lt;&gt;"",IFERROR(F46&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G46&lt;&gt;"",IFERROR(G46&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
       <c r="H47" s="46" t="n"/>
       <c r="I47" s="46" t="n"/>
       <c r="J47" s="48">
-        <f>IF(OR(C47="",D47=""),"",IF(LEFT(D47,LEN(LEFT(C47,FIND(" ·",C47&amp;" ·")-1))+1)&lt;&gt;LEFT(C47,FIND(" ·",C47&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F47&lt;&gt;"",G47&lt;&gt;"",G47&lt;F47),"⚠ Fin avant début",IF(AND(F47&lt;&gt;"",IFERROR(F47&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C47,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G47&lt;&gt;"",IFERROR(G47&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C47,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C47="",D47=""),"",IF(LEFT(D47,LEN(LEFT(C47,FIND(" ·",C47&amp;" ·")-1))+1)&lt;&gt;LEFT(C47,FIND(" ·",C47&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F47&lt;&gt;"",G47&lt;&gt;"",G47&lt;F47),"⚠ Fin avant début",IF(AND(F47&lt;&gt;"",IFERROR(F47&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G47&lt;&gt;"",IFERROR(G47&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4809,7 +4809,7 @@
       <c r="H48" s="46" t="n"/>
       <c r="I48" s="46" t="n"/>
       <c r="J48" s="48">
-        <f>IF(OR(C48="",D48=""),"",IF(LEFT(D48,LEN(LEFT(C48,FIND(" ·",C48&amp;" ·")-1))+1)&lt;&gt;LEFT(C48,FIND(" ·",C48&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F48&lt;&gt;"",G48&lt;&gt;"",G48&lt;F48),"⚠ Fin avant début",IF(AND(F48&lt;&gt;"",IFERROR(F48&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C48,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G48&lt;&gt;"",IFERROR(G48&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C48,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C48="",D48=""),"",IF(LEFT(D48,LEN(LEFT(C48,FIND(" ·",C48&amp;" ·")-1))+1)&lt;&gt;LEFT(C48,FIND(" ·",C48&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F48&lt;&gt;"",G48&lt;&gt;"",G48&lt;F48),"⚠ Fin avant début",IF(AND(F48&lt;&gt;"",IFERROR(F48&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G48&lt;&gt;"",IFERROR(G48&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       <c r="H49" s="46" t="n"/>
       <c r="I49" s="46" t="n"/>
       <c r="J49" s="48">
-        <f>IF(OR(C49="",D49=""),"",IF(LEFT(D49,LEN(LEFT(C49,FIND(" ·",C49&amp;" ·")-1))+1)&lt;&gt;LEFT(C49,FIND(" ·",C49&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F49&lt;&gt;"",G49&lt;&gt;"",G49&lt;F49),"⚠ Fin avant début",IF(AND(F49&lt;&gt;"",IFERROR(F49&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C49,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G49&lt;&gt;"",IFERROR(G49&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C49,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C49="",D49=""),"",IF(LEFT(D49,LEN(LEFT(C49,FIND(" ·",C49&amp;" ·")-1))+1)&lt;&gt;LEFT(C49,FIND(" ·",C49&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F49&lt;&gt;"",G49&lt;&gt;"",G49&lt;F49),"⚠ Fin avant début",IF(AND(F49&lt;&gt;"",IFERROR(F49&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G49&lt;&gt;"",IFERROR(G49&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       <c r="H50" s="46" t="n"/>
       <c r="I50" s="46" t="n"/>
       <c r="J50" s="48">
-        <f>IF(OR(C50="",D50=""),"",IF(LEFT(D50,LEN(LEFT(C50,FIND(" ·",C50&amp;" ·")-1))+1)&lt;&gt;LEFT(C50,FIND(" ·",C50&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F50&lt;&gt;"",G50&lt;&gt;"",G50&lt;F50),"⚠ Fin avant début",IF(AND(F50&lt;&gt;"",IFERROR(F50&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C50,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G50&lt;&gt;"",IFERROR(G50&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C50,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C50="",D50=""),"",IF(LEFT(D50,LEN(LEFT(C50,FIND(" ·",C50&amp;" ·")-1))+1)&lt;&gt;LEFT(C50,FIND(" ·",C50&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F50&lt;&gt;"",G50&lt;&gt;"",G50&lt;F50),"⚠ Fin avant début",IF(AND(F50&lt;&gt;"",IFERROR(F50&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G50&lt;&gt;"",IFERROR(G50&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       <c r="H51" s="46" t="n"/>
       <c r="I51" s="46" t="n"/>
       <c r="J51" s="48">
-        <f>IF(OR(C51="",D51=""),"",IF(LEFT(D51,LEN(LEFT(C51,FIND(" ·",C51&amp;" ·")-1))+1)&lt;&gt;LEFT(C51,FIND(" ·",C51&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F51&lt;&gt;"",G51&lt;&gt;"",G51&lt;F51),"⚠ Fin avant début",IF(AND(F51&lt;&gt;"",IFERROR(F51&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C51,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G51&lt;&gt;"",IFERROR(G51&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C51,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C51="",D51=""),"",IF(LEFT(D51,LEN(LEFT(C51,FIND(" ·",C51&amp;" ·")-1))+1)&lt;&gt;LEFT(C51,FIND(" ·",C51&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F51&lt;&gt;"",G51&lt;&gt;"",G51&lt;F51),"⚠ Fin avant début",IF(AND(F51&lt;&gt;"",IFERROR(F51&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G51&lt;&gt;"",IFERROR(G51&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       <c r="H52" s="46" t="n"/>
       <c r="I52" s="46" t="n"/>
       <c r="J52" s="48">
-        <f>IF(OR(C52="",D52=""),"",IF(LEFT(D52,LEN(LEFT(C52,FIND(" ·",C52&amp;" ·")-1))+1)&lt;&gt;LEFT(C52,FIND(" ·",C52&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F52&lt;&gt;"",G52&lt;&gt;"",G52&lt;F52),"⚠ Fin avant début",IF(AND(F52&lt;&gt;"",IFERROR(F52&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C52,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G52&lt;&gt;"",IFERROR(G52&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C52,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C52="",D52=""),"",IF(LEFT(D52,LEN(LEFT(C52,FIND(" ·",C52&amp;" ·")-1))+1)&lt;&gt;LEFT(C52,FIND(" ·",C52&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F52&lt;&gt;"",G52&lt;&gt;"",G52&lt;F52),"⚠ Fin avant début",IF(AND(F52&lt;&gt;"",IFERROR(F52&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G52&lt;&gt;"",IFERROR(G52&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       <c r="H53" s="46" t="n"/>
       <c r="I53" s="46" t="n"/>
       <c r="J53" s="48">
-        <f>IF(OR(C53="",D53=""),"",IF(LEFT(D53,LEN(LEFT(C53,FIND(" ·",C53&amp;" ·")-1))+1)&lt;&gt;LEFT(C53,FIND(" ·",C53&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F53&lt;&gt;"",G53&lt;&gt;"",G53&lt;F53),"⚠ Fin avant début",IF(AND(F53&lt;&gt;"",IFERROR(F53&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C53,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G53&lt;&gt;"",IFERROR(G53&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C53,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C53="",D53=""),"",IF(LEFT(D53,LEN(LEFT(C53,FIND(" ·",C53&amp;" ·")-1))+1)&lt;&gt;LEFT(C53,FIND(" ·",C53&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F53&lt;&gt;"",G53&lt;&gt;"",G53&lt;F53),"⚠ Fin avant début",IF(AND(F53&lt;&gt;"",IFERROR(F53&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G53&lt;&gt;"",IFERROR(G53&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       <c r="H54" s="46" t="n"/>
       <c r="I54" s="46" t="n"/>
       <c r="J54" s="48">
-        <f>IF(OR(C54="",D54=""),"",IF(LEFT(D54,LEN(LEFT(C54,FIND(" ·",C54&amp;" ·")-1))+1)&lt;&gt;LEFT(C54,FIND(" ·",C54&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F54&lt;&gt;"",G54&lt;&gt;"",G54&lt;F54),"⚠ Fin avant début",IF(AND(F54&lt;&gt;"",IFERROR(F54&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C54,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G54&lt;&gt;"",IFERROR(G54&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C54,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C54="",D54=""),"",IF(LEFT(D54,LEN(LEFT(C54,FIND(" ·",C54&amp;" ·")-1))+1)&lt;&gt;LEFT(C54,FIND(" ·",C54&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F54&lt;&gt;"",G54&lt;&gt;"",G54&lt;F54),"⚠ Fin avant début",IF(AND(F54&lt;&gt;"",IFERROR(F54&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G54&lt;&gt;"",IFERROR(G54&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4928,7 +4928,7 @@
       <c r="H55" s="46" t="n"/>
       <c r="I55" s="46" t="n"/>
       <c r="J55" s="48">
-        <f>IF(OR(C55="",D55=""),"",IF(LEFT(D55,LEN(LEFT(C55,FIND(" ·",C55&amp;" ·")-1))+1)&lt;&gt;LEFT(C55,FIND(" ·",C55&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F55&lt;&gt;"",G55&lt;&gt;"",G55&lt;F55),"⚠ Fin avant début",IF(AND(F55&lt;&gt;"",IFERROR(F55&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C55,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G55&lt;&gt;"",IFERROR(G55&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C55,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C55="",D55=""),"",IF(LEFT(D55,LEN(LEFT(C55,FIND(" ·",C55&amp;" ·")-1))+1)&lt;&gt;LEFT(C55,FIND(" ·",C55&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F55&lt;&gt;"",G55&lt;&gt;"",G55&lt;F55),"⚠ Fin avant début",IF(AND(F55&lt;&gt;"",IFERROR(F55&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G55&lt;&gt;"",IFERROR(G55&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       <c r="H56" s="46" t="n"/>
       <c r="I56" s="46" t="n"/>
       <c r="J56" s="48">
-        <f>IF(OR(C56="",D56=""),"",IF(LEFT(D56,LEN(LEFT(C56,FIND(" ·",C56&amp;" ·")-1))+1)&lt;&gt;LEFT(C56,FIND(" ·",C56&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F56&lt;&gt;"",G56&lt;&gt;"",G56&lt;F56),"⚠ Fin avant début",IF(AND(F56&lt;&gt;"",IFERROR(F56&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C56,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G56&lt;&gt;"",IFERROR(G56&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C56,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C56="",D56=""),"",IF(LEFT(D56,LEN(LEFT(C56,FIND(" ·",C56&amp;" ·")-1))+1)&lt;&gt;LEFT(C56,FIND(" ·",C56&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F56&lt;&gt;"",G56&lt;&gt;"",G56&lt;F56),"⚠ Fin avant début",IF(AND(F56&lt;&gt;"",IFERROR(F56&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G56&lt;&gt;"",IFERROR(G56&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4962,7 +4962,7 @@
       <c r="H57" s="46" t="n"/>
       <c r="I57" s="46" t="n"/>
       <c r="J57" s="48">
-        <f>IF(OR(C57="",D57=""),"",IF(LEFT(D57,LEN(LEFT(C57,FIND(" ·",C57&amp;" ·")-1))+1)&lt;&gt;LEFT(C57,FIND(" ·",C57&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F57&lt;&gt;"",G57&lt;&gt;"",G57&lt;F57),"⚠ Fin avant début",IF(AND(F57&lt;&gt;"",IFERROR(F57&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C57,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G57&lt;&gt;"",IFERROR(G57&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C57,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C57="",D57=""),"",IF(LEFT(D57,LEN(LEFT(C57,FIND(" ·",C57&amp;" ·")-1))+1)&lt;&gt;LEFT(C57,FIND(" ·",C57&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F57&lt;&gt;"",G57&lt;&gt;"",G57&lt;F57),"⚠ Fin avant début",IF(AND(F57&lt;&gt;"",IFERROR(F57&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G57&lt;&gt;"",IFERROR(G57&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       <c r="H58" s="46" t="n"/>
       <c r="I58" s="46" t="n"/>
       <c r="J58" s="48">
-        <f>IF(OR(C58="",D58=""),"",IF(LEFT(D58,LEN(LEFT(C58,FIND(" ·",C58&amp;" ·")-1))+1)&lt;&gt;LEFT(C58,FIND(" ·",C58&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F58&lt;&gt;"",G58&lt;&gt;"",G58&lt;F58),"⚠ Fin avant début",IF(AND(F58&lt;&gt;"",IFERROR(F58&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C58,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G58&lt;&gt;"",IFERROR(G58&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C58,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C58="",D58=""),"",IF(LEFT(D58,LEN(LEFT(C58,FIND(" ·",C58&amp;" ·")-1))+1)&lt;&gt;LEFT(C58,FIND(" ·",C58&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F58&lt;&gt;"",G58&lt;&gt;"",G58&lt;F58),"⚠ Fin avant début",IF(AND(F58&lt;&gt;"",IFERROR(F58&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G58&lt;&gt;"",IFERROR(G58&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       <c r="H59" s="46" t="n"/>
       <c r="I59" s="46" t="n"/>
       <c r="J59" s="48">
-        <f>IF(OR(C59="",D59=""),"",IF(LEFT(D59,LEN(LEFT(C59,FIND(" ·",C59&amp;" ·")-1))+1)&lt;&gt;LEFT(C59,FIND(" ·",C59&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F59&lt;&gt;"",G59&lt;&gt;"",G59&lt;F59),"⚠ Fin avant début",IF(AND(F59&lt;&gt;"",IFERROR(F59&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C59,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G59&lt;&gt;"",IFERROR(G59&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C59,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C59="",D59=""),"",IF(LEFT(D59,LEN(LEFT(C59,FIND(" ·",C59&amp;" ·")-1))+1)&lt;&gt;LEFT(C59,FIND(" ·",C59&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F59&lt;&gt;"",G59&lt;&gt;"",G59&lt;F59),"⚠ Fin avant début",IF(AND(F59&lt;&gt;"",IFERROR(F59&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G59&lt;&gt;"",IFERROR(G59&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       <c r="H60" s="46" t="n"/>
       <c r="I60" s="46" t="n"/>
       <c r="J60" s="48">
-        <f>IF(OR(C60="",D60=""),"",IF(LEFT(D60,LEN(LEFT(C60,FIND(" ·",C60&amp;" ·")-1))+1)&lt;&gt;LEFT(C60,FIND(" ·",C60&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F60&lt;&gt;"",G60&lt;&gt;"",G60&lt;F60),"⚠ Fin avant début",IF(AND(F60&lt;&gt;"",IFERROR(F60&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C60,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G60&lt;&gt;"",IFERROR(G60&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C60,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C60="",D60=""),"",IF(LEFT(D60,LEN(LEFT(C60,FIND(" ·",C60&amp;" ·")-1))+1)&lt;&gt;LEFT(C60,FIND(" ·",C60&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F60&lt;&gt;"",G60&lt;&gt;"",G60&lt;F60),"⚠ Fin avant début",IF(AND(F60&lt;&gt;"",IFERROR(F60&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G60&lt;&gt;"",IFERROR(G60&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       <c r="H61" s="46" t="n"/>
       <c r="I61" s="46" t="n"/>
       <c r="J61" s="48">
-        <f>IF(OR(C61="",D61=""),"",IF(LEFT(D61,LEN(LEFT(C61,FIND(" ·",C61&amp;" ·")-1))+1)&lt;&gt;LEFT(C61,FIND(" ·",C61&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F61&lt;&gt;"",G61&lt;&gt;"",G61&lt;F61),"⚠ Fin avant début",IF(AND(F61&lt;&gt;"",IFERROR(F61&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C61,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G61&lt;&gt;"",IFERROR(G61&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C61,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C61="",D61=""),"",IF(LEFT(D61,LEN(LEFT(C61,FIND(" ·",C61&amp;" ·")-1))+1)&lt;&gt;LEFT(C61,FIND(" ·",C61&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F61&lt;&gt;"",G61&lt;&gt;"",G61&lt;F61),"⚠ Fin avant début",IF(AND(F61&lt;&gt;"",IFERROR(F61&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G61&lt;&gt;"",IFERROR(G61&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       <c r="H62" s="46" t="n"/>
       <c r="I62" s="46" t="n"/>
       <c r="J62" s="48">
-        <f>IF(OR(C62="",D62=""),"",IF(LEFT(D62,LEN(LEFT(C62,FIND(" ·",C62&amp;" ·")-1))+1)&lt;&gt;LEFT(C62,FIND(" ·",C62&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F62&lt;&gt;"",G62&lt;&gt;"",G62&lt;F62),"⚠ Fin avant début",IF(AND(F62&lt;&gt;"",IFERROR(F62&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C62,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G62&lt;&gt;"",IFERROR(G62&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C62,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C62="",D62=""),"",IF(LEFT(D62,LEN(LEFT(C62,FIND(" ·",C62&amp;" ·")-1))+1)&lt;&gt;LEFT(C62,FIND(" ·",C62&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F62&lt;&gt;"",G62&lt;&gt;"",G62&lt;F62),"⚠ Fin avant début",IF(AND(F62&lt;&gt;"",IFERROR(F62&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G62&lt;&gt;"",IFERROR(G62&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       <c r="H63" s="46" t="n"/>
       <c r="I63" s="46" t="n"/>
       <c r="J63" s="48">
-        <f>IF(OR(C63="",D63=""),"",IF(LEFT(D63,LEN(LEFT(C63,FIND(" ·",C63&amp;" ·")-1))+1)&lt;&gt;LEFT(C63,FIND(" ·",C63&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F63&lt;&gt;"",G63&lt;&gt;"",G63&lt;F63),"⚠ Fin avant début",IF(AND(F63&lt;&gt;"",IFERROR(F63&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C63,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G63&lt;&gt;"",IFERROR(G63&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C63,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C63="",D63=""),"",IF(LEFT(D63,LEN(LEFT(C63,FIND(" ·",C63&amp;" ·")-1))+1)&lt;&gt;LEFT(C63,FIND(" ·",C63&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F63&lt;&gt;"",G63&lt;&gt;"",G63&lt;F63),"⚠ Fin avant début",IF(AND(F63&lt;&gt;"",IFERROR(F63&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G63&lt;&gt;"",IFERROR(G63&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       <c r="H64" s="46" t="n"/>
       <c r="I64" s="46" t="n"/>
       <c r="J64" s="48">
-        <f>IF(OR(C64="",D64=""),"",IF(LEFT(D64,LEN(LEFT(C64,FIND(" ·",C64&amp;" ·")-1))+1)&lt;&gt;LEFT(C64,FIND(" ·",C64&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F64&lt;&gt;"",G64&lt;&gt;"",G64&lt;F64),"⚠ Fin avant début",IF(AND(F64&lt;&gt;"",IFERROR(F64&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C64,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G64&lt;&gt;"",IFERROR(G64&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C64,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C64="",D64=""),"",IF(LEFT(D64,LEN(LEFT(C64,FIND(" ·",C64&amp;" ·")-1))+1)&lt;&gt;LEFT(C64,FIND(" ·",C64&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F64&lt;&gt;"",G64&lt;&gt;"",G64&lt;F64),"⚠ Fin avant début",IF(AND(F64&lt;&gt;"",IFERROR(F64&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G64&lt;&gt;"",IFERROR(G64&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5098,7 +5098,7 @@
       <c r="H65" s="46" t="n"/>
       <c r="I65" s="46" t="n"/>
       <c r="J65" s="48">
-        <f>IF(OR(C65="",D65=""),"",IF(LEFT(D65,LEN(LEFT(C65,FIND(" ·",C65&amp;" ·")-1))+1)&lt;&gt;LEFT(C65,FIND(" ·",C65&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F65&lt;&gt;"",G65&lt;&gt;"",G65&lt;F65),"⚠ Fin avant début",IF(AND(F65&lt;&gt;"",IFERROR(F65&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C65,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G65&lt;&gt;"",IFERROR(G65&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C65,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C65="",D65=""),"",IF(LEFT(D65,LEN(LEFT(C65,FIND(" ·",C65&amp;" ·")-1))+1)&lt;&gt;LEFT(C65,FIND(" ·",C65&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F65&lt;&gt;"",G65&lt;&gt;"",G65&lt;F65),"⚠ Fin avant début",IF(AND(F65&lt;&gt;"",IFERROR(F65&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G65&lt;&gt;"",IFERROR(G65&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       <c r="H66" s="46" t="n"/>
       <c r="I66" s="46" t="n"/>
       <c r="J66" s="48">
-        <f>IF(OR(C66="",D66=""),"",IF(LEFT(D66,LEN(LEFT(C66,FIND(" ·",C66&amp;" ·")-1))+1)&lt;&gt;LEFT(C66,FIND(" ·",C66&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F66&lt;&gt;"",G66&lt;&gt;"",G66&lt;F66),"⚠ Fin avant début",IF(AND(F66&lt;&gt;"",IFERROR(F66&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C66,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G66&lt;&gt;"",IFERROR(G66&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C66,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C66="",D66=""),"",IF(LEFT(D66,LEN(LEFT(C66,FIND(" ·",C66&amp;" ·")-1))+1)&lt;&gt;LEFT(C66,FIND(" ·",C66&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F66&lt;&gt;"",G66&lt;&gt;"",G66&lt;F66),"⚠ Fin avant début",IF(AND(F66&lt;&gt;"",IFERROR(F66&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G66&lt;&gt;"",IFERROR(G66&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       <c r="H67" s="46" t="n"/>
       <c r="I67" s="46" t="n"/>
       <c r="J67" s="48">
-        <f>IF(OR(C67="",D67=""),"",IF(LEFT(D67,LEN(LEFT(C67,FIND(" ·",C67&amp;" ·")-1))+1)&lt;&gt;LEFT(C67,FIND(" ·",C67&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F67&lt;&gt;"",G67&lt;&gt;"",G67&lt;F67),"⚠ Fin avant début",IF(AND(F67&lt;&gt;"",IFERROR(F67&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C67,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G67&lt;&gt;"",IFERROR(G67&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C67,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C67="",D67=""),"",IF(LEFT(D67,LEN(LEFT(C67,FIND(" ·",C67&amp;" ·")-1))+1)&lt;&gt;LEFT(C67,FIND(" ·",C67&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F67&lt;&gt;"",G67&lt;&gt;"",G67&lt;F67),"⚠ Fin avant début",IF(AND(F67&lt;&gt;"",IFERROR(F67&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G67&lt;&gt;"",IFERROR(G67&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5149,7 +5149,7 @@
       <c r="H68" s="46" t="n"/>
       <c r="I68" s="46" t="n"/>
       <c r="J68" s="48">
-        <f>IF(OR(C68="",D68=""),"",IF(LEFT(D68,LEN(LEFT(C68,FIND(" ·",C68&amp;" ·")-1))+1)&lt;&gt;LEFT(C68,FIND(" ·",C68&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F68&lt;&gt;"",G68&lt;&gt;"",G68&lt;F68),"⚠ Fin avant début",IF(AND(F68&lt;&gt;"",IFERROR(F68&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C68,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G68&lt;&gt;"",IFERROR(G68&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C68,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C68="",D68=""),"",IF(LEFT(D68,LEN(LEFT(C68,FIND(" ·",C68&amp;" ·")-1))+1)&lt;&gt;LEFT(C68,FIND(" ·",C68&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F68&lt;&gt;"",G68&lt;&gt;"",G68&lt;F68),"⚠ Fin avant début",IF(AND(F68&lt;&gt;"",IFERROR(F68&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G68&lt;&gt;"",IFERROR(G68&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       <c r="H69" s="46" t="n"/>
       <c r="I69" s="46" t="n"/>
       <c r="J69" s="48">
-        <f>IF(OR(C69="",D69=""),"",IF(LEFT(D69,LEN(LEFT(C69,FIND(" ·",C69&amp;" ·")-1))+1)&lt;&gt;LEFT(C69,FIND(" ·",C69&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F69&lt;&gt;"",G69&lt;&gt;"",G69&lt;F69),"⚠ Fin avant début",IF(AND(F69&lt;&gt;"",IFERROR(F69&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C69,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G69&lt;&gt;"",IFERROR(G69&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C69,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C69="",D69=""),"",IF(LEFT(D69,LEN(LEFT(C69,FIND(" ·",C69&amp;" ·")-1))+1)&lt;&gt;LEFT(C69,FIND(" ·",C69&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F69&lt;&gt;"",G69&lt;&gt;"",G69&lt;F69),"⚠ Fin avant début",IF(AND(F69&lt;&gt;"",IFERROR(F69&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G69&lt;&gt;"",IFERROR(G69&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       <c r="H70" s="46" t="n"/>
       <c r="I70" s="46" t="n"/>
       <c r="J70" s="48">
-        <f>IF(OR(C70="",D70=""),"",IF(LEFT(D70,LEN(LEFT(C70,FIND(" ·",C70&amp;" ·")-1))+1)&lt;&gt;LEFT(C70,FIND(" ·",C70&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F70&lt;&gt;"",G70&lt;&gt;"",G70&lt;F70),"⚠ Fin avant début",IF(AND(F70&lt;&gt;"",IFERROR(F70&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C70,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G70&lt;&gt;"",IFERROR(G70&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C70,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C70="",D70=""),"",IF(LEFT(D70,LEN(LEFT(C70,FIND(" ·",C70&amp;" ·")-1))+1)&lt;&gt;LEFT(C70,FIND(" ·",C70&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F70&lt;&gt;"",G70&lt;&gt;"",G70&lt;F70),"⚠ Fin avant début",IF(AND(F70&lt;&gt;"",IFERROR(F70&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G70&lt;&gt;"",IFERROR(G70&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       <c r="H71" s="46" t="n"/>
       <c r="I71" s="46" t="n"/>
       <c r="J71" s="48">
-        <f>IF(OR(C71="",D71=""),"",IF(LEFT(D71,LEN(LEFT(C71,FIND(" ·",C71&amp;" ·")-1))+1)&lt;&gt;LEFT(C71,FIND(" ·",C71&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F71&lt;&gt;"",G71&lt;&gt;"",G71&lt;F71),"⚠ Fin avant début",IF(AND(F71&lt;&gt;"",IFERROR(F71&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C71,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G71&lt;&gt;"",IFERROR(G71&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C71,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C71="",D71=""),"",IF(LEFT(D71,LEN(LEFT(C71,FIND(" ·",C71&amp;" ·")-1))+1)&lt;&gt;LEFT(C71,FIND(" ·",C71&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F71&lt;&gt;"",G71&lt;&gt;"",G71&lt;F71),"⚠ Fin avant début",IF(AND(F71&lt;&gt;"",IFERROR(F71&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G71&lt;&gt;"",IFERROR(G71&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       <c r="H72" s="46" t="n"/>
       <c r="I72" s="46" t="n"/>
       <c r="J72" s="48">
-        <f>IF(OR(C72="",D72=""),"",IF(LEFT(D72,LEN(LEFT(C72,FIND(" ·",C72&amp;" ·")-1))+1)&lt;&gt;LEFT(C72,FIND(" ·",C72&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F72&lt;&gt;"",G72&lt;&gt;"",G72&lt;F72),"⚠ Fin avant début",IF(AND(F72&lt;&gt;"",IFERROR(F72&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C72,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G72&lt;&gt;"",IFERROR(G72&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C72,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C72="",D72=""),"",IF(LEFT(D72,LEN(LEFT(C72,FIND(" ·",C72&amp;" ·")-1))+1)&lt;&gt;LEFT(C72,FIND(" ·",C72&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F72&lt;&gt;"",G72&lt;&gt;"",G72&lt;F72),"⚠ Fin avant début",IF(AND(F72&lt;&gt;"",IFERROR(F72&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G72&lt;&gt;"",IFERROR(G72&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       <c r="H73" s="46" t="n"/>
       <c r="I73" s="46" t="n"/>
       <c r="J73" s="48">
-        <f>IF(OR(C73="",D73=""),"",IF(LEFT(D73,LEN(LEFT(C73,FIND(" ·",C73&amp;" ·")-1))+1)&lt;&gt;LEFT(C73,FIND(" ·",C73&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F73&lt;&gt;"",G73&lt;&gt;"",G73&lt;F73),"⚠ Fin avant début",IF(AND(F73&lt;&gt;"",IFERROR(F73&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C73,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G73&lt;&gt;"",IFERROR(G73&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C73,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C73="",D73=""),"",IF(LEFT(D73,LEN(LEFT(C73,FIND(" ·",C73&amp;" ·")-1))+1)&lt;&gt;LEFT(C73,FIND(" ·",C73&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F73&lt;&gt;"",G73&lt;&gt;"",G73&lt;F73),"⚠ Fin avant début",IF(AND(F73&lt;&gt;"",IFERROR(F73&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G73&lt;&gt;"",IFERROR(G73&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       <c r="H74" s="46" t="n"/>
       <c r="I74" s="46" t="n"/>
       <c r="J74" s="48">
-        <f>IF(OR(C74="",D74=""),"",IF(LEFT(D74,LEN(LEFT(C74,FIND(" ·",C74&amp;" ·")-1))+1)&lt;&gt;LEFT(C74,FIND(" ·",C74&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F74&lt;&gt;"",G74&lt;&gt;"",G74&lt;F74),"⚠ Fin avant début",IF(AND(F74&lt;&gt;"",IFERROR(F74&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C74,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G74&lt;&gt;"",IFERROR(G74&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C74,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C74="",D74=""),"",IF(LEFT(D74,LEN(LEFT(C74,FIND(" ·",C74&amp;" ·")-1))+1)&lt;&gt;LEFT(C74,FIND(" ·",C74&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F74&lt;&gt;"",G74&lt;&gt;"",G74&lt;F74),"⚠ Fin avant début",IF(AND(F74&lt;&gt;"",IFERROR(F74&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G74&lt;&gt;"",IFERROR(G74&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5268,7 +5268,7 @@
       <c r="H75" s="46" t="n"/>
       <c r="I75" s="46" t="n"/>
       <c r="J75" s="48">
-        <f>IF(OR(C75="",D75=""),"",IF(LEFT(D75,LEN(LEFT(C75,FIND(" ·",C75&amp;" ·")-1))+1)&lt;&gt;LEFT(C75,FIND(" ·",C75&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F75&lt;&gt;"",G75&lt;&gt;"",G75&lt;F75),"⚠ Fin avant début",IF(AND(F75&lt;&gt;"",IFERROR(F75&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C75,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G75&lt;&gt;"",IFERROR(G75&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C75,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C75="",D75=""),"",IF(LEFT(D75,LEN(LEFT(C75,FIND(" ·",C75&amp;" ·")-1))+1)&lt;&gt;LEFT(C75,FIND(" ·",C75&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F75&lt;&gt;"",G75&lt;&gt;"",G75&lt;F75),"⚠ Fin avant début",IF(AND(F75&lt;&gt;"",IFERROR(F75&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G75&lt;&gt;"",IFERROR(G75&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
       <c r="H76" s="46" t="n"/>
       <c r="I76" s="46" t="n"/>
       <c r="J76" s="48">
-        <f>IF(OR(C76="",D76=""),"",IF(LEFT(D76,LEN(LEFT(C76,FIND(" ·",C76&amp;" ·")-1))+1)&lt;&gt;LEFT(C76,FIND(" ·",C76&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F76&lt;&gt;"",G76&lt;&gt;"",G76&lt;F76),"⚠ Fin avant début",IF(AND(F76&lt;&gt;"",IFERROR(F76&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C76,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G76&lt;&gt;"",IFERROR(G76&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C76,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C76="",D76=""),"",IF(LEFT(D76,LEN(LEFT(C76,FIND(" ·",C76&amp;" ·")-1))+1)&lt;&gt;LEFT(C76,FIND(" ·",C76&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F76&lt;&gt;"",G76&lt;&gt;"",G76&lt;F76),"⚠ Fin avant début",IF(AND(F76&lt;&gt;"",IFERROR(F76&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G76&lt;&gt;"",IFERROR(G76&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       <c r="H77" s="46" t="n"/>
       <c r="I77" s="46" t="n"/>
       <c r="J77" s="48">
-        <f>IF(OR(C77="",D77=""),"",IF(LEFT(D77,LEN(LEFT(C77,FIND(" ·",C77&amp;" ·")-1))+1)&lt;&gt;LEFT(C77,FIND(" ·",C77&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F77&lt;&gt;"",G77&lt;&gt;"",G77&lt;F77),"⚠ Fin avant début",IF(AND(F77&lt;&gt;"",IFERROR(F77&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C77,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G77&lt;&gt;"",IFERROR(G77&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C77,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C77="",D77=""),"",IF(LEFT(D77,LEN(LEFT(C77,FIND(" ·",C77&amp;" ·")-1))+1)&lt;&gt;LEFT(C77,FIND(" ·",C77&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F77&lt;&gt;"",G77&lt;&gt;"",G77&lt;F77),"⚠ Fin avant début",IF(AND(F77&lt;&gt;"",IFERROR(F77&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G77&lt;&gt;"",IFERROR(G77&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5319,7 +5319,7 @@
       <c r="H78" s="46" t="n"/>
       <c r="I78" s="46" t="n"/>
       <c r="J78" s="48">
-        <f>IF(OR(C78="",D78=""),"",IF(LEFT(D78,LEN(LEFT(C78,FIND(" ·",C78&amp;" ·")-1))+1)&lt;&gt;LEFT(C78,FIND(" ·",C78&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F78&lt;&gt;"",G78&lt;&gt;"",G78&lt;F78),"⚠ Fin avant début",IF(AND(F78&lt;&gt;"",IFERROR(F78&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C78,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G78&lt;&gt;"",IFERROR(G78&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C78,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C78="",D78=""),"",IF(LEFT(D78,LEN(LEFT(C78,FIND(" ·",C78&amp;" ·")-1))+1)&lt;&gt;LEFT(C78,FIND(" ·",C78&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F78&lt;&gt;"",G78&lt;&gt;"",G78&lt;F78),"⚠ Fin avant début",IF(AND(F78&lt;&gt;"",IFERROR(F78&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G78&lt;&gt;"",IFERROR(G78&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       <c r="H79" s="46" t="n"/>
       <c r="I79" s="46" t="n"/>
       <c r="J79" s="48">
-        <f>IF(OR(C79="",D79=""),"",IF(LEFT(D79,LEN(LEFT(C79,FIND(" ·",C79&amp;" ·")-1))+1)&lt;&gt;LEFT(C79,FIND(" ·",C79&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F79&lt;&gt;"",G79&lt;&gt;"",G79&lt;F79),"⚠ Fin avant début",IF(AND(F79&lt;&gt;"",IFERROR(F79&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C79,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G79&lt;&gt;"",IFERROR(G79&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C79,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C79="",D79=""),"",IF(LEFT(D79,LEN(LEFT(C79,FIND(" ·",C79&amp;" ·")-1))+1)&lt;&gt;LEFT(C79,FIND(" ·",C79&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F79&lt;&gt;"",G79&lt;&gt;"",G79&lt;F79),"⚠ Fin avant début",IF(AND(F79&lt;&gt;"",IFERROR(F79&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G79&lt;&gt;"",IFERROR(G79&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       <c r="H80" s="46" t="n"/>
       <c r="I80" s="46" t="n"/>
       <c r="J80" s="48">
-        <f>IF(OR(C80="",D80=""),"",IF(LEFT(D80,LEN(LEFT(C80,FIND(" ·",C80&amp;" ·")-1))+1)&lt;&gt;LEFT(C80,FIND(" ·",C80&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F80&lt;&gt;"",G80&lt;&gt;"",G80&lt;F80),"⚠ Fin avant début",IF(AND(F80&lt;&gt;"",IFERROR(F80&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C80,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G80&lt;&gt;"",IFERROR(G80&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C80,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C80="",D80=""),"",IF(LEFT(D80,LEN(LEFT(C80,FIND(" ·",C80&amp;" ·")-1))+1)&lt;&gt;LEFT(C80,FIND(" ·",C80&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F80&lt;&gt;"",G80&lt;&gt;"",G80&lt;F80),"⚠ Fin avant début",IF(AND(F80&lt;&gt;"",IFERROR(F80&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G80&lt;&gt;"",IFERROR(G80&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5370,7 +5370,7 @@
       <c r="H81" s="46" t="n"/>
       <c r="I81" s="46" t="n"/>
       <c r="J81" s="48">
-        <f>IF(OR(C81="",D81=""),"",IF(LEFT(D81,LEN(LEFT(C81,FIND(" ·",C81&amp;" ·")-1))+1)&lt;&gt;LEFT(C81,FIND(" ·",C81&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F81&lt;&gt;"",G81&lt;&gt;"",G81&lt;F81),"⚠ Fin avant début",IF(AND(F81&lt;&gt;"",IFERROR(F81&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C81,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G81&lt;&gt;"",IFERROR(G81&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C81,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C81="",D81=""),"",IF(LEFT(D81,LEN(LEFT(C81,FIND(" ·",C81&amp;" ·")-1))+1)&lt;&gt;LEFT(C81,FIND(" ·",C81&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F81&lt;&gt;"",G81&lt;&gt;"",G81&lt;F81),"⚠ Fin avant début",IF(AND(F81&lt;&gt;"",IFERROR(F81&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G81&lt;&gt;"",IFERROR(G81&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5387,7 +5387,7 @@
       <c r="H82" s="46" t="n"/>
       <c r="I82" s="46" t="n"/>
       <c r="J82" s="48">
-        <f>IF(OR(C82="",D82=""),"",IF(LEFT(D82,LEN(LEFT(C82,FIND(" ·",C82&amp;" ·")-1))+1)&lt;&gt;LEFT(C82,FIND(" ·",C82&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F82&lt;&gt;"",G82&lt;&gt;"",G82&lt;F82),"⚠ Fin avant début",IF(AND(F82&lt;&gt;"",IFERROR(F82&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C82,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G82&lt;&gt;"",IFERROR(G82&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C82,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C82="",D82=""),"",IF(LEFT(D82,LEN(LEFT(C82,FIND(" ·",C82&amp;" ·")-1))+1)&lt;&gt;LEFT(C82,FIND(" ·",C82&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F82&lt;&gt;"",G82&lt;&gt;"",G82&lt;F82),"⚠ Fin avant début",IF(AND(F82&lt;&gt;"",IFERROR(F82&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G82&lt;&gt;"",IFERROR(G82&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5404,7 +5404,7 @@
       <c r="H83" s="46" t="n"/>
       <c r="I83" s="46" t="n"/>
       <c r="J83" s="48">
-        <f>IF(OR(C83="",D83=""),"",IF(LEFT(D83,LEN(LEFT(C83,FIND(" ·",C83&amp;" ·")-1))+1)&lt;&gt;LEFT(C83,FIND(" ·",C83&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F83&lt;&gt;"",G83&lt;&gt;"",G83&lt;F83),"⚠ Fin avant début",IF(AND(F83&lt;&gt;"",IFERROR(F83&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C83,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G83&lt;&gt;"",IFERROR(G83&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C83,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C83="",D83=""),"",IF(LEFT(D83,LEN(LEFT(C83,FIND(" ·",C83&amp;" ·")-1))+1)&lt;&gt;LEFT(C83,FIND(" ·",C83&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F83&lt;&gt;"",G83&lt;&gt;"",G83&lt;F83),"⚠ Fin avant début",IF(AND(F83&lt;&gt;"",IFERROR(F83&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G83&lt;&gt;"",IFERROR(G83&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       <c r="H84" s="46" t="n"/>
       <c r="I84" s="46" t="n"/>
       <c r="J84" s="48">
-        <f>IF(OR(C84="",D84=""),"",IF(LEFT(D84,LEN(LEFT(C84,FIND(" ·",C84&amp;" ·")-1))+1)&lt;&gt;LEFT(C84,FIND(" ·",C84&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F84&lt;&gt;"",G84&lt;&gt;"",G84&lt;F84),"⚠ Fin avant début",IF(AND(F84&lt;&gt;"",IFERROR(F84&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C84,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G84&lt;&gt;"",IFERROR(G84&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C84,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C84="",D84=""),"",IF(LEFT(D84,LEN(LEFT(C84,FIND(" ·",C84&amp;" ·")-1))+1)&lt;&gt;LEFT(C84,FIND(" ·",C84&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F84&lt;&gt;"",G84&lt;&gt;"",G84&lt;F84),"⚠ Fin avant début",IF(AND(F84&lt;&gt;"",IFERROR(F84&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G84&lt;&gt;"",IFERROR(G84&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       <c r="H85" s="46" t="n"/>
       <c r="I85" s="46" t="n"/>
       <c r="J85" s="48">
-        <f>IF(OR(C85="",D85=""),"",IF(LEFT(D85,LEN(LEFT(C85,FIND(" ·",C85&amp;" ·")-1))+1)&lt;&gt;LEFT(C85,FIND(" ·",C85&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F85&lt;&gt;"",G85&lt;&gt;"",G85&lt;F85),"⚠ Fin avant début",IF(AND(F85&lt;&gt;"",IFERROR(F85&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C85,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G85&lt;&gt;"",IFERROR(G85&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C85,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C85="",D85=""),"",IF(LEFT(D85,LEN(LEFT(C85,FIND(" ·",C85&amp;" ·")-1))+1)&lt;&gt;LEFT(C85,FIND(" ·",C85&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F85&lt;&gt;"",G85&lt;&gt;"",G85&lt;F85),"⚠ Fin avant début",IF(AND(F85&lt;&gt;"",IFERROR(F85&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G85&lt;&gt;"",IFERROR(G85&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5455,7 +5455,7 @@
       <c r="H86" s="46" t="n"/>
       <c r="I86" s="46" t="n"/>
       <c r="J86" s="48">
-        <f>IF(OR(C86="",D86=""),"",IF(LEFT(D86,LEN(LEFT(C86,FIND(" ·",C86&amp;" ·")-1))+1)&lt;&gt;LEFT(C86,FIND(" ·",C86&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F86&lt;&gt;"",G86&lt;&gt;"",G86&lt;F86),"⚠ Fin avant début",IF(AND(F86&lt;&gt;"",IFERROR(F86&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C86,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G86&lt;&gt;"",IFERROR(G86&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C86,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C86="",D86=""),"",IF(LEFT(D86,LEN(LEFT(C86,FIND(" ·",C86&amp;" ·")-1))+1)&lt;&gt;LEFT(C86,FIND(" ·",C86&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F86&lt;&gt;"",G86&lt;&gt;"",G86&lt;F86),"⚠ Fin avant début",IF(AND(F86&lt;&gt;"",IFERROR(F86&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G86&lt;&gt;"",IFERROR(G86&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5472,7 +5472,7 @@
       <c r="H87" s="46" t="n"/>
       <c r="I87" s="46" t="n"/>
       <c r="J87" s="48">
-        <f>IF(OR(C87="",D87=""),"",IF(LEFT(D87,LEN(LEFT(C87,FIND(" ·",C87&amp;" ·")-1))+1)&lt;&gt;LEFT(C87,FIND(" ·",C87&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F87&lt;&gt;"",G87&lt;&gt;"",G87&lt;F87),"⚠ Fin avant début",IF(AND(F87&lt;&gt;"",IFERROR(F87&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C87,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G87&lt;&gt;"",IFERROR(G87&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C87,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C87="",D87=""),"",IF(LEFT(D87,LEN(LEFT(C87,FIND(" ·",C87&amp;" ·")-1))+1)&lt;&gt;LEFT(C87,FIND(" ·",C87&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F87&lt;&gt;"",G87&lt;&gt;"",G87&lt;F87),"⚠ Fin avant début",IF(AND(F87&lt;&gt;"",IFERROR(F87&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G87&lt;&gt;"",IFERROR(G87&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       <c r="H88" s="46" t="n"/>
       <c r="I88" s="46" t="n"/>
       <c r="J88" s="48">
-        <f>IF(OR(C88="",D88=""),"",IF(LEFT(D88,LEN(LEFT(C88,FIND(" ·",C88&amp;" ·")-1))+1)&lt;&gt;LEFT(C88,FIND(" ·",C88&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F88&lt;&gt;"",G88&lt;&gt;"",G88&lt;F88),"⚠ Fin avant début",IF(AND(F88&lt;&gt;"",IFERROR(F88&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(C88,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G88&lt;&gt;"",IFERROR(G88&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(C88,'07 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C88="",D88=""),"",IF(LEFT(D88,LEN(LEFT(C88,FIND(" ·",C88&amp;" ·")-1))+1)&lt;&gt;LEFT(C88,FIND(" ·",C88&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F88&lt;&gt;"",G88&lt;&gt;"",G88&lt;F88),"⚠ Fin avant début",IF(AND(F88&lt;&gt;"",IFERROR(F88&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G88&lt;&gt;"",IFERROR(G88&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="J3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5612,7 +5612,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 09    </t>
+            <t xml:space="preserve">Étape 10    </t>
           </r>
           <r>
             <rPr>
@@ -6336,7 +6336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:J28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6394,7 +6394,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 10    </t>
+            <t xml:space="preserve">Étape 11    </t>
           </r>
           <r>
             <rPr>
@@ -6513,7 +6513,7 @@
       <c r="G9" s="46" t="n"/>
       <c r="H9" s="46" t="n"/>
       <c r="I9" s="47">
-        <f>IF(B9="","",COUNTIF('11 Membres'!$B$9:$B$208,B9))</f>
+        <f>IF(B9="","",COUNTIF('12 Membres'!$B$9:$B$208,B9))</f>
         <v/>
       </c>
       <c r="J9" s="48">
@@ -6533,7 +6533,7 @@
       <c r="G10" s="46" t="n"/>
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="47">
-        <f>IF(B10="","",COUNTIF('11 Membres'!$B$9:$B$208,B10))</f>
+        <f>IF(B10="","",COUNTIF('12 Membres'!$B$9:$B$208,B10))</f>
         <v/>
       </c>
       <c r="J10" s="48">
@@ -6553,7 +6553,7 @@
       <c r="G11" s="46" t="n"/>
       <c r="H11" s="46" t="n"/>
       <c r="I11" s="47">
-        <f>IF(B11="","",COUNTIF('11 Membres'!$B$9:$B$208,B11))</f>
+        <f>IF(B11="","",COUNTIF('12 Membres'!$B$9:$B$208,B11))</f>
         <v/>
       </c>
       <c r="J11" s="48">
@@ -6573,7 +6573,7 @@
       <c r="G12" s="46" t="n"/>
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="47">
-        <f>IF(B12="","",COUNTIF('11 Membres'!$B$9:$B$208,B12))</f>
+        <f>IF(B12="","",COUNTIF('12 Membres'!$B$9:$B$208,B12))</f>
         <v/>
       </c>
       <c r="J12" s="48">
@@ -6593,7 +6593,7 @@
       <c r="G13" s="46" t="n"/>
       <c r="H13" s="46" t="n"/>
       <c r="I13" s="47">
-        <f>IF(B13="","",COUNTIF('11 Membres'!$B$9:$B$208,B13))</f>
+        <f>IF(B13="","",COUNTIF('12 Membres'!$B$9:$B$208,B13))</f>
         <v/>
       </c>
       <c r="J13" s="48">
@@ -6613,7 +6613,7 @@
       <c r="G14" s="46" t="n"/>
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="47">
-        <f>IF(B14="","",COUNTIF('11 Membres'!$B$9:$B$208,B14))</f>
+        <f>IF(B14="","",COUNTIF('12 Membres'!$B$9:$B$208,B14))</f>
         <v/>
       </c>
       <c r="J14" s="48">
@@ -6633,7 +6633,7 @@
       <c r="G15" s="46" t="n"/>
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="47">
-        <f>IF(B15="","",COUNTIF('11 Membres'!$B$9:$B$208,B15))</f>
+        <f>IF(B15="","",COUNTIF('12 Membres'!$B$9:$B$208,B15))</f>
         <v/>
       </c>
       <c r="J15" s="48">
@@ -6653,7 +6653,7 @@
       <c r="G16" s="46" t="n"/>
       <c r="H16" s="46" t="n"/>
       <c r="I16" s="47">
-        <f>IF(B16="","",COUNTIF('11 Membres'!$B$9:$B$208,B16))</f>
+        <f>IF(B16="","",COUNTIF('12 Membres'!$B$9:$B$208,B16))</f>
         <v/>
       </c>
       <c r="J16" s="48">
@@ -6673,7 +6673,7 @@
       <c r="G17" s="46" t="n"/>
       <c r="H17" s="46" t="n"/>
       <c r="I17" s="47">
-        <f>IF(B17="","",COUNTIF('11 Membres'!$B$9:$B$208,B17))</f>
+        <f>IF(B17="","",COUNTIF('12 Membres'!$B$9:$B$208,B17))</f>
         <v/>
       </c>
       <c r="J17" s="48">
@@ -6693,7 +6693,7 @@
       <c r="G18" s="46" t="n"/>
       <c r="H18" s="46" t="n"/>
       <c r="I18" s="47">
-        <f>IF(B18="","",COUNTIF('11 Membres'!$B$9:$B$208,B18))</f>
+        <f>IF(B18="","",COUNTIF('12 Membres'!$B$9:$B$208,B18))</f>
         <v/>
       </c>
       <c r="J18" s="48">
@@ -6713,7 +6713,7 @@
       <c r="G19" s="46" t="n"/>
       <c r="H19" s="46" t="n"/>
       <c r="I19" s="47">
-        <f>IF(B19="","",COUNTIF('11 Membres'!$B$9:$B$208,B19))</f>
+        <f>IF(B19="","",COUNTIF('12 Membres'!$B$9:$B$208,B19))</f>
         <v/>
       </c>
       <c r="J19" s="48">
@@ -6733,7 +6733,7 @@
       <c r="G20" s="46" t="n"/>
       <c r="H20" s="46" t="n"/>
       <c r="I20" s="47">
-        <f>IF(B20="","",COUNTIF('11 Membres'!$B$9:$B$208,B20))</f>
+        <f>IF(B20="","",COUNTIF('12 Membres'!$B$9:$B$208,B20))</f>
         <v/>
       </c>
       <c r="J20" s="48">
@@ -6753,7 +6753,7 @@
       <c r="G21" s="46" t="n"/>
       <c r="H21" s="46" t="n"/>
       <c r="I21" s="47">
-        <f>IF(B21="","",COUNTIF('11 Membres'!$B$9:$B$208,B21))</f>
+        <f>IF(B21="","",COUNTIF('12 Membres'!$B$9:$B$208,B21))</f>
         <v/>
       </c>
       <c r="J21" s="48">
@@ -6773,7 +6773,7 @@
       <c r="G22" s="46" t="n"/>
       <c r="H22" s="46" t="n"/>
       <c r="I22" s="47">
-        <f>IF(B22="","",COUNTIF('11 Membres'!$B$9:$B$208,B22))</f>
+        <f>IF(B22="","",COUNTIF('12 Membres'!$B$9:$B$208,B22))</f>
         <v/>
       </c>
       <c r="J22" s="48">
@@ -6793,7 +6793,7 @@
       <c r="G23" s="46" t="n"/>
       <c r="H23" s="46" t="n"/>
       <c r="I23" s="47">
-        <f>IF(B23="","",COUNTIF('11 Membres'!$B$9:$B$208,B23))</f>
+        <f>IF(B23="","",COUNTIF('12 Membres'!$B$9:$B$208,B23))</f>
         <v/>
       </c>
       <c r="J23" s="48">
@@ -6813,7 +6813,7 @@
       <c r="G24" s="46" t="n"/>
       <c r="H24" s="46" t="n"/>
       <c r="I24" s="47">
-        <f>IF(B24="","",COUNTIF('11 Membres'!$B$9:$B$208,B24))</f>
+        <f>IF(B24="","",COUNTIF('12 Membres'!$B$9:$B$208,B24))</f>
         <v/>
       </c>
       <c r="J24" s="48">
@@ -6833,7 +6833,7 @@
       <c r="G25" s="46" t="n"/>
       <c r="H25" s="46" t="n"/>
       <c r="I25" s="47">
-        <f>IF(B25="","",COUNTIF('11 Membres'!$B$9:$B$208,B25))</f>
+        <f>IF(B25="","",COUNTIF('12 Membres'!$B$9:$B$208,B25))</f>
         <v/>
       </c>
       <c r="J25" s="48">
@@ -6853,7 +6853,7 @@
       <c r="G26" s="46" t="n"/>
       <c r="H26" s="46" t="n"/>
       <c r="I26" s="47">
-        <f>IF(B26="","",COUNTIF('11 Membres'!$B$9:$B$208,B26))</f>
+        <f>IF(B26="","",COUNTIF('12 Membres'!$B$9:$B$208,B26))</f>
         <v/>
       </c>
       <c r="J26" s="48">
@@ -6873,7 +6873,7 @@
       <c r="G27" s="46" t="n"/>
       <c r="H27" s="46" t="n"/>
       <c r="I27" s="47">
-        <f>IF(B27="","",COUNTIF('11 Membres'!$B$9:$B$208,B27))</f>
+        <f>IF(B27="","",COUNTIF('12 Membres'!$B$9:$B$208,B27))</f>
         <v/>
       </c>
       <c r="J27" s="48">
@@ -6893,7 +6893,7 @@
       <c r="G28" s="46" t="n"/>
       <c r="H28" s="46" t="n"/>
       <c r="I28" s="47">
-        <f>IF(B28="","",COUNTIF('11 Membres'!$B$9:$B$208,B28))</f>
+        <f>IF(B28="","",COUNTIF('12 Membres'!$B$9:$B$208,B28))</f>
         <v/>
       </c>
       <c r="J28" s="48">
@@ -6979,7 +6979,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="J3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -6993,7 +6993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E208"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7046,7 +7046,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 11    </t>
+            <t xml:space="preserve">Étape 12    </t>
           </r>
           <r>
             <rPr>
@@ -8953,7 +8953,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="E3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -8967,7 +8967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K108"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -9026,7 +9026,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 12    </t>
+            <t xml:space="preserve">Étape 13    </t>
           </r>
           <r>
             <rPr>
@@ -9165,7 +9165,7 @@
       <c r="I9" s="49" t="n"/>
       <c r="J9" s="49" t="n"/>
       <c r="K9" s="48">
-        <f>IF(C9="","",IF(D9="","⚠ Phase manquante",IF(AND(E9&lt;&gt;"",LEFT(E9,LEN(LEFT(D9,FIND(" ·",D9&amp;" ·")-1))+1)&lt;&gt;LEFT(D9,FIND(" ·",D9&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I9&lt;&gt;"",IFERROR(OR(I9&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D9,'07 Phases'!$B$9:$B$38,0)),I9&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D9,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C9="","",IF(D9="","⚠ Phase manquante",IF(AND(E9&lt;&gt;"",LEFT(E9,LEN(LEFT(D9,FIND(" ·",D9&amp;" ·")-1))+1)&lt;&gt;LEFT(D9,FIND(" ·",D9&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I9&lt;&gt;"",IFERROR(OR(I9&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D9,'08 Phases'!$B$9:$B$38,0)),I9&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D9,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9183,7 +9183,7 @@
       <c r="I10" s="49" t="n"/>
       <c r="J10" s="49" t="n"/>
       <c r="K10" s="48">
-        <f>IF(C10="","",IF(D10="","⚠ Phase manquante",IF(AND(E10&lt;&gt;"",LEFT(E10,LEN(LEFT(D10,FIND(" ·",D10&amp;" ·")-1))+1)&lt;&gt;LEFT(D10,FIND(" ·",D10&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I10&lt;&gt;"",IFERROR(OR(I10&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D10,'07 Phases'!$B$9:$B$38,0)),I10&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D10,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C10="","",IF(D10="","⚠ Phase manquante",IF(AND(E10&lt;&gt;"",LEFT(E10,LEN(LEFT(D10,FIND(" ·",D10&amp;" ·")-1))+1)&lt;&gt;LEFT(D10,FIND(" ·",D10&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I10&lt;&gt;"",IFERROR(OR(I10&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D10,'08 Phases'!$B$9:$B$38,0)),I10&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D10,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       <c r="I11" s="49" t="n"/>
       <c r="J11" s="49" t="n"/>
       <c r="K11" s="48">
-        <f>IF(C11="","",IF(D11="","⚠ Phase manquante",IF(AND(E11&lt;&gt;"",LEFT(E11,LEN(LEFT(D11,FIND(" ·",D11&amp;" ·")-1))+1)&lt;&gt;LEFT(D11,FIND(" ·",D11&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I11&lt;&gt;"",IFERROR(OR(I11&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D11,'07 Phases'!$B$9:$B$38,0)),I11&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D11,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C11="","",IF(D11="","⚠ Phase manquante",IF(AND(E11&lt;&gt;"",LEFT(E11,LEN(LEFT(D11,FIND(" ·",D11&amp;" ·")-1))+1)&lt;&gt;LEFT(D11,FIND(" ·",D11&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I11&lt;&gt;"",IFERROR(OR(I11&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D11,'08 Phases'!$B$9:$B$38,0)),I11&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D11,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9219,7 +9219,7 @@
       <c r="I12" s="49" t="n"/>
       <c r="J12" s="49" t="n"/>
       <c r="K12" s="48">
-        <f>IF(C12="","",IF(D12="","⚠ Phase manquante",IF(AND(E12&lt;&gt;"",LEFT(E12,LEN(LEFT(D12,FIND(" ·",D12&amp;" ·")-1))+1)&lt;&gt;LEFT(D12,FIND(" ·",D12&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I12&lt;&gt;"",IFERROR(OR(I12&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D12,'07 Phases'!$B$9:$B$38,0)),I12&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D12,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C12="","",IF(D12="","⚠ Phase manquante",IF(AND(E12&lt;&gt;"",LEFT(E12,LEN(LEFT(D12,FIND(" ·",D12&amp;" ·")-1))+1)&lt;&gt;LEFT(D12,FIND(" ·",D12&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I12&lt;&gt;"",IFERROR(OR(I12&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D12,'08 Phases'!$B$9:$B$38,0)),I12&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D12,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9237,7 +9237,7 @@
       <c r="I13" s="49" t="n"/>
       <c r="J13" s="49" t="n"/>
       <c r="K13" s="48">
-        <f>IF(C13="","",IF(D13="","⚠ Phase manquante",IF(AND(E13&lt;&gt;"",LEFT(E13,LEN(LEFT(D13,FIND(" ·",D13&amp;" ·")-1))+1)&lt;&gt;LEFT(D13,FIND(" ·",D13&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I13&lt;&gt;"",IFERROR(OR(I13&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D13,'07 Phases'!$B$9:$B$38,0)),I13&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D13,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C13="","",IF(D13="","⚠ Phase manquante",IF(AND(E13&lt;&gt;"",LEFT(E13,LEN(LEFT(D13,FIND(" ·",D13&amp;" ·")-1))+1)&lt;&gt;LEFT(D13,FIND(" ·",D13&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I13&lt;&gt;"",IFERROR(OR(I13&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D13,'08 Phases'!$B$9:$B$38,0)),I13&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D13,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9255,7 +9255,7 @@
       <c r="I14" s="49" t="n"/>
       <c r="J14" s="49" t="n"/>
       <c r="K14" s="48">
-        <f>IF(C14="","",IF(D14="","⚠ Phase manquante",IF(AND(E14&lt;&gt;"",LEFT(E14,LEN(LEFT(D14,FIND(" ·",D14&amp;" ·")-1))+1)&lt;&gt;LEFT(D14,FIND(" ·",D14&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I14&lt;&gt;"",IFERROR(OR(I14&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D14,'07 Phases'!$B$9:$B$38,0)),I14&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D14,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C14="","",IF(D14="","⚠ Phase manquante",IF(AND(E14&lt;&gt;"",LEFT(E14,LEN(LEFT(D14,FIND(" ·",D14&amp;" ·")-1))+1)&lt;&gt;LEFT(D14,FIND(" ·",D14&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I14&lt;&gt;"",IFERROR(OR(I14&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D14,'08 Phases'!$B$9:$B$38,0)),I14&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D14,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9273,7 +9273,7 @@
       <c r="I15" s="49" t="n"/>
       <c r="J15" s="49" t="n"/>
       <c r="K15" s="48">
-        <f>IF(C15="","",IF(D15="","⚠ Phase manquante",IF(AND(E15&lt;&gt;"",LEFT(E15,LEN(LEFT(D15,FIND(" ·",D15&amp;" ·")-1))+1)&lt;&gt;LEFT(D15,FIND(" ·",D15&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I15&lt;&gt;"",IFERROR(OR(I15&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D15,'07 Phases'!$B$9:$B$38,0)),I15&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D15,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C15="","",IF(D15="","⚠ Phase manquante",IF(AND(E15&lt;&gt;"",LEFT(E15,LEN(LEFT(D15,FIND(" ·",D15&amp;" ·")-1))+1)&lt;&gt;LEFT(D15,FIND(" ·",D15&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I15&lt;&gt;"",IFERROR(OR(I15&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D15,'08 Phases'!$B$9:$B$38,0)),I15&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D15,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9291,7 +9291,7 @@
       <c r="I16" s="49" t="n"/>
       <c r="J16" s="49" t="n"/>
       <c r="K16" s="48">
-        <f>IF(C16="","",IF(D16="","⚠ Phase manquante",IF(AND(E16&lt;&gt;"",LEFT(E16,LEN(LEFT(D16,FIND(" ·",D16&amp;" ·")-1))+1)&lt;&gt;LEFT(D16,FIND(" ·",D16&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I16&lt;&gt;"",IFERROR(OR(I16&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D16,'07 Phases'!$B$9:$B$38,0)),I16&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D16,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C16="","",IF(D16="","⚠ Phase manquante",IF(AND(E16&lt;&gt;"",LEFT(E16,LEN(LEFT(D16,FIND(" ·",D16&amp;" ·")-1))+1)&lt;&gt;LEFT(D16,FIND(" ·",D16&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I16&lt;&gt;"",IFERROR(OR(I16&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D16,'08 Phases'!$B$9:$B$38,0)),I16&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D16,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9309,7 +9309,7 @@
       <c r="I17" s="49" t="n"/>
       <c r="J17" s="49" t="n"/>
       <c r="K17" s="48">
-        <f>IF(C17="","",IF(D17="","⚠ Phase manquante",IF(AND(E17&lt;&gt;"",LEFT(E17,LEN(LEFT(D17,FIND(" ·",D17&amp;" ·")-1))+1)&lt;&gt;LEFT(D17,FIND(" ·",D17&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I17&lt;&gt;"",IFERROR(OR(I17&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D17,'07 Phases'!$B$9:$B$38,0)),I17&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D17,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C17="","",IF(D17="","⚠ Phase manquante",IF(AND(E17&lt;&gt;"",LEFT(E17,LEN(LEFT(D17,FIND(" ·",D17&amp;" ·")-1))+1)&lt;&gt;LEFT(D17,FIND(" ·",D17&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I17&lt;&gt;"",IFERROR(OR(I17&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D17,'08 Phases'!$B$9:$B$38,0)),I17&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D17,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9327,7 +9327,7 @@
       <c r="I18" s="49" t="n"/>
       <c r="J18" s="49" t="n"/>
       <c r="K18" s="48">
-        <f>IF(C18="","",IF(D18="","⚠ Phase manquante",IF(AND(E18&lt;&gt;"",LEFT(E18,LEN(LEFT(D18,FIND(" ·",D18&amp;" ·")-1))+1)&lt;&gt;LEFT(D18,FIND(" ·",D18&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I18&lt;&gt;"",IFERROR(OR(I18&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D18,'07 Phases'!$B$9:$B$38,0)),I18&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D18,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C18="","",IF(D18="","⚠ Phase manquante",IF(AND(E18&lt;&gt;"",LEFT(E18,LEN(LEFT(D18,FIND(" ·",D18&amp;" ·")-1))+1)&lt;&gt;LEFT(D18,FIND(" ·",D18&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I18&lt;&gt;"",IFERROR(OR(I18&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D18,'08 Phases'!$B$9:$B$38,0)),I18&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D18,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9345,7 +9345,7 @@
       <c r="I19" s="49" t="n"/>
       <c r="J19" s="49" t="n"/>
       <c r="K19" s="48">
-        <f>IF(C19="","",IF(D19="","⚠ Phase manquante",IF(AND(E19&lt;&gt;"",LEFT(E19,LEN(LEFT(D19,FIND(" ·",D19&amp;" ·")-1))+1)&lt;&gt;LEFT(D19,FIND(" ·",D19&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I19&lt;&gt;"",IFERROR(OR(I19&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D19,'07 Phases'!$B$9:$B$38,0)),I19&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D19,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C19="","",IF(D19="","⚠ Phase manquante",IF(AND(E19&lt;&gt;"",LEFT(E19,LEN(LEFT(D19,FIND(" ·",D19&amp;" ·")-1))+1)&lt;&gt;LEFT(D19,FIND(" ·",D19&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I19&lt;&gt;"",IFERROR(OR(I19&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D19,'08 Phases'!$B$9:$B$38,0)),I19&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D19,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9363,7 +9363,7 @@
       <c r="I20" s="49" t="n"/>
       <c r="J20" s="49" t="n"/>
       <c r="K20" s="48">
-        <f>IF(C20="","",IF(D20="","⚠ Phase manquante",IF(AND(E20&lt;&gt;"",LEFT(E20,LEN(LEFT(D20,FIND(" ·",D20&amp;" ·")-1))+1)&lt;&gt;LEFT(D20,FIND(" ·",D20&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I20&lt;&gt;"",IFERROR(OR(I20&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D20,'07 Phases'!$B$9:$B$38,0)),I20&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D20,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C20="","",IF(D20="","⚠ Phase manquante",IF(AND(E20&lt;&gt;"",LEFT(E20,LEN(LEFT(D20,FIND(" ·",D20&amp;" ·")-1))+1)&lt;&gt;LEFT(D20,FIND(" ·",D20&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I20&lt;&gt;"",IFERROR(OR(I20&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D20,'08 Phases'!$B$9:$B$38,0)),I20&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D20,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9381,7 +9381,7 @@
       <c r="I21" s="49" t="n"/>
       <c r="J21" s="49" t="n"/>
       <c r="K21" s="48">
-        <f>IF(C21="","",IF(D21="","⚠ Phase manquante",IF(AND(E21&lt;&gt;"",LEFT(E21,LEN(LEFT(D21,FIND(" ·",D21&amp;" ·")-1))+1)&lt;&gt;LEFT(D21,FIND(" ·",D21&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I21&lt;&gt;"",IFERROR(OR(I21&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D21,'07 Phases'!$B$9:$B$38,0)),I21&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D21,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C21="","",IF(D21="","⚠ Phase manquante",IF(AND(E21&lt;&gt;"",LEFT(E21,LEN(LEFT(D21,FIND(" ·",D21&amp;" ·")-1))+1)&lt;&gt;LEFT(D21,FIND(" ·",D21&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I21&lt;&gt;"",IFERROR(OR(I21&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D21,'08 Phases'!$B$9:$B$38,0)),I21&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D21,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9399,7 +9399,7 @@
       <c r="I22" s="49" t="n"/>
       <c r="J22" s="49" t="n"/>
       <c r="K22" s="48">
-        <f>IF(C22="","",IF(D22="","⚠ Phase manquante",IF(AND(E22&lt;&gt;"",LEFT(E22,LEN(LEFT(D22,FIND(" ·",D22&amp;" ·")-1))+1)&lt;&gt;LEFT(D22,FIND(" ·",D22&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I22&lt;&gt;"",IFERROR(OR(I22&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D22,'07 Phases'!$B$9:$B$38,0)),I22&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D22,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C22="","",IF(D22="","⚠ Phase manquante",IF(AND(E22&lt;&gt;"",LEFT(E22,LEN(LEFT(D22,FIND(" ·",D22&amp;" ·")-1))+1)&lt;&gt;LEFT(D22,FIND(" ·",D22&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I22&lt;&gt;"",IFERROR(OR(I22&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D22,'08 Phases'!$B$9:$B$38,0)),I22&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D22,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9417,7 +9417,7 @@
       <c r="I23" s="49" t="n"/>
       <c r="J23" s="49" t="n"/>
       <c r="K23" s="48">
-        <f>IF(C23="","",IF(D23="","⚠ Phase manquante",IF(AND(E23&lt;&gt;"",LEFT(E23,LEN(LEFT(D23,FIND(" ·",D23&amp;" ·")-1))+1)&lt;&gt;LEFT(D23,FIND(" ·",D23&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I23&lt;&gt;"",IFERROR(OR(I23&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D23,'07 Phases'!$B$9:$B$38,0)),I23&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D23,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C23="","",IF(D23="","⚠ Phase manquante",IF(AND(E23&lt;&gt;"",LEFT(E23,LEN(LEFT(D23,FIND(" ·",D23&amp;" ·")-1))+1)&lt;&gt;LEFT(D23,FIND(" ·",D23&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I23&lt;&gt;"",IFERROR(OR(I23&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D23,'08 Phases'!$B$9:$B$38,0)),I23&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D23,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       <c r="I24" s="49" t="n"/>
       <c r="J24" s="49" t="n"/>
       <c r="K24" s="48">
-        <f>IF(C24="","",IF(D24="","⚠ Phase manquante",IF(AND(E24&lt;&gt;"",LEFT(E24,LEN(LEFT(D24,FIND(" ·",D24&amp;" ·")-1))+1)&lt;&gt;LEFT(D24,FIND(" ·",D24&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I24&lt;&gt;"",IFERROR(OR(I24&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D24,'07 Phases'!$B$9:$B$38,0)),I24&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D24,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C24="","",IF(D24="","⚠ Phase manquante",IF(AND(E24&lt;&gt;"",LEFT(E24,LEN(LEFT(D24,FIND(" ·",D24&amp;" ·")-1))+1)&lt;&gt;LEFT(D24,FIND(" ·",D24&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I24&lt;&gt;"",IFERROR(OR(I24&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D24,'08 Phases'!$B$9:$B$38,0)),I24&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D24,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9453,7 +9453,7 @@
       <c r="I25" s="49" t="n"/>
       <c r="J25" s="49" t="n"/>
       <c r="K25" s="48">
-        <f>IF(C25="","",IF(D25="","⚠ Phase manquante",IF(AND(E25&lt;&gt;"",LEFT(E25,LEN(LEFT(D25,FIND(" ·",D25&amp;" ·")-1))+1)&lt;&gt;LEFT(D25,FIND(" ·",D25&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I25&lt;&gt;"",IFERROR(OR(I25&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D25,'07 Phases'!$B$9:$B$38,0)),I25&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D25,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C25="","",IF(D25="","⚠ Phase manquante",IF(AND(E25&lt;&gt;"",LEFT(E25,LEN(LEFT(D25,FIND(" ·",D25&amp;" ·")-1))+1)&lt;&gt;LEFT(D25,FIND(" ·",D25&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I25&lt;&gt;"",IFERROR(OR(I25&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D25,'08 Phases'!$B$9:$B$38,0)),I25&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D25,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9471,7 +9471,7 @@
       <c r="I26" s="49" t="n"/>
       <c r="J26" s="49" t="n"/>
       <c r="K26" s="48">
-        <f>IF(C26="","",IF(D26="","⚠ Phase manquante",IF(AND(E26&lt;&gt;"",LEFT(E26,LEN(LEFT(D26,FIND(" ·",D26&amp;" ·")-1))+1)&lt;&gt;LEFT(D26,FIND(" ·",D26&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I26&lt;&gt;"",IFERROR(OR(I26&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D26,'07 Phases'!$B$9:$B$38,0)),I26&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D26,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C26="","",IF(D26="","⚠ Phase manquante",IF(AND(E26&lt;&gt;"",LEFT(E26,LEN(LEFT(D26,FIND(" ·",D26&amp;" ·")-1))+1)&lt;&gt;LEFT(D26,FIND(" ·",D26&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I26&lt;&gt;"",IFERROR(OR(I26&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D26,'08 Phases'!$B$9:$B$38,0)),I26&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D26,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9489,7 +9489,7 @@
       <c r="I27" s="49" t="n"/>
       <c r="J27" s="49" t="n"/>
       <c r="K27" s="48">
-        <f>IF(C27="","",IF(D27="","⚠ Phase manquante",IF(AND(E27&lt;&gt;"",LEFT(E27,LEN(LEFT(D27,FIND(" ·",D27&amp;" ·")-1))+1)&lt;&gt;LEFT(D27,FIND(" ·",D27&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I27&lt;&gt;"",IFERROR(OR(I27&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D27,'07 Phases'!$B$9:$B$38,0)),I27&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D27,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C27="","",IF(D27="","⚠ Phase manquante",IF(AND(E27&lt;&gt;"",LEFT(E27,LEN(LEFT(D27,FIND(" ·",D27&amp;" ·")-1))+1)&lt;&gt;LEFT(D27,FIND(" ·",D27&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I27&lt;&gt;"",IFERROR(OR(I27&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D27,'08 Phases'!$B$9:$B$38,0)),I27&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D27,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9507,7 +9507,7 @@
       <c r="I28" s="49" t="n"/>
       <c r="J28" s="49" t="n"/>
       <c r="K28" s="48">
-        <f>IF(C28="","",IF(D28="","⚠ Phase manquante",IF(AND(E28&lt;&gt;"",LEFT(E28,LEN(LEFT(D28,FIND(" ·",D28&amp;" ·")-1))+1)&lt;&gt;LEFT(D28,FIND(" ·",D28&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I28&lt;&gt;"",IFERROR(OR(I28&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D28,'07 Phases'!$B$9:$B$38,0)),I28&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D28,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C28="","",IF(D28="","⚠ Phase manquante",IF(AND(E28&lt;&gt;"",LEFT(E28,LEN(LEFT(D28,FIND(" ·",D28&amp;" ·")-1))+1)&lt;&gt;LEFT(D28,FIND(" ·",D28&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I28&lt;&gt;"",IFERROR(OR(I28&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D28,'08 Phases'!$B$9:$B$38,0)),I28&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D28,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9525,7 +9525,7 @@
       <c r="I29" s="49" t="n"/>
       <c r="J29" s="49" t="n"/>
       <c r="K29" s="48">
-        <f>IF(C29="","",IF(D29="","⚠ Phase manquante",IF(AND(E29&lt;&gt;"",LEFT(E29,LEN(LEFT(D29,FIND(" ·",D29&amp;" ·")-1))+1)&lt;&gt;LEFT(D29,FIND(" ·",D29&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I29&lt;&gt;"",IFERROR(OR(I29&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D29,'07 Phases'!$B$9:$B$38,0)),I29&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D29,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C29="","",IF(D29="","⚠ Phase manquante",IF(AND(E29&lt;&gt;"",LEFT(E29,LEN(LEFT(D29,FIND(" ·",D29&amp;" ·")-1))+1)&lt;&gt;LEFT(D29,FIND(" ·",D29&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I29&lt;&gt;"",IFERROR(OR(I29&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D29,'08 Phases'!$B$9:$B$38,0)),I29&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D29,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9543,7 +9543,7 @@
       <c r="I30" s="49" t="n"/>
       <c r="J30" s="49" t="n"/>
       <c r="K30" s="48">
-        <f>IF(C30="","",IF(D30="","⚠ Phase manquante",IF(AND(E30&lt;&gt;"",LEFT(E30,LEN(LEFT(D30,FIND(" ·",D30&amp;" ·")-1))+1)&lt;&gt;LEFT(D30,FIND(" ·",D30&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I30&lt;&gt;"",IFERROR(OR(I30&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D30,'07 Phases'!$B$9:$B$38,0)),I30&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D30,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C30="","",IF(D30="","⚠ Phase manquante",IF(AND(E30&lt;&gt;"",LEFT(E30,LEN(LEFT(D30,FIND(" ·",D30&amp;" ·")-1))+1)&lt;&gt;LEFT(D30,FIND(" ·",D30&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I30&lt;&gt;"",IFERROR(OR(I30&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D30,'08 Phases'!$B$9:$B$38,0)),I30&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D30,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9561,7 +9561,7 @@
       <c r="I31" s="49" t="n"/>
       <c r="J31" s="49" t="n"/>
       <c r="K31" s="48">
-        <f>IF(C31="","",IF(D31="","⚠ Phase manquante",IF(AND(E31&lt;&gt;"",LEFT(E31,LEN(LEFT(D31,FIND(" ·",D31&amp;" ·")-1))+1)&lt;&gt;LEFT(D31,FIND(" ·",D31&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I31&lt;&gt;"",IFERROR(OR(I31&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D31,'07 Phases'!$B$9:$B$38,0)),I31&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D31,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C31="","",IF(D31="","⚠ Phase manquante",IF(AND(E31&lt;&gt;"",LEFT(E31,LEN(LEFT(D31,FIND(" ·",D31&amp;" ·")-1))+1)&lt;&gt;LEFT(D31,FIND(" ·",D31&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I31&lt;&gt;"",IFERROR(OR(I31&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D31,'08 Phases'!$B$9:$B$38,0)),I31&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D31,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9579,7 +9579,7 @@
       <c r="I32" s="49" t="n"/>
       <c r="J32" s="49" t="n"/>
       <c r="K32" s="48">
-        <f>IF(C32="","",IF(D32="","⚠ Phase manquante",IF(AND(E32&lt;&gt;"",LEFT(E32,LEN(LEFT(D32,FIND(" ·",D32&amp;" ·")-1))+1)&lt;&gt;LEFT(D32,FIND(" ·",D32&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I32&lt;&gt;"",IFERROR(OR(I32&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D32,'07 Phases'!$B$9:$B$38,0)),I32&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D32,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C32="","",IF(D32="","⚠ Phase manquante",IF(AND(E32&lt;&gt;"",LEFT(E32,LEN(LEFT(D32,FIND(" ·",D32&amp;" ·")-1))+1)&lt;&gt;LEFT(D32,FIND(" ·",D32&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I32&lt;&gt;"",IFERROR(OR(I32&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D32,'08 Phases'!$B$9:$B$38,0)),I32&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D32,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9597,7 +9597,7 @@
       <c r="I33" s="49" t="n"/>
       <c r="J33" s="49" t="n"/>
       <c r="K33" s="48">
-        <f>IF(C33="","",IF(D33="","⚠ Phase manquante",IF(AND(E33&lt;&gt;"",LEFT(E33,LEN(LEFT(D33,FIND(" ·",D33&amp;" ·")-1))+1)&lt;&gt;LEFT(D33,FIND(" ·",D33&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I33&lt;&gt;"",IFERROR(OR(I33&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D33,'07 Phases'!$B$9:$B$38,0)),I33&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D33,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C33="","",IF(D33="","⚠ Phase manquante",IF(AND(E33&lt;&gt;"",LEFT(E33,LEN(LEFT(D33,FIND(" ·",D33&amp;" ·")-1))+1)&lt;&gt;LEFT(D33,FIND(" ·",D33&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I33&lt;&gt;"",IFERROR(OR(I33&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D33,'08 Phases'!$B$9:$B$38,0)),I33&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D33,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9615,7 +9615,7 @@
       <c r="I34" s="49" t="n"/>
       <c r="J34" s="49" t="n"/>
       <c r="K34" s="48">
-        <f>IF(C34="","",IF(D34="","⚠ Phase manquante",IF(AND(E34&lt;&gt;"",LEFT(E34,LEN(LEFT(D34,FIND(" ·",D34&amp;" ·")-1))+1)&lt;&gt;LEFT(D34,FIND(" ·",D34&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I34&lt;&gt;"",IFERROR(OR(I34&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D34,'07 Phases'!$B$9:$B$38,0)),I34&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D34,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C34="","",IF(D34="","⚠ Phase manquante",IF(AND(E34&lt;&gt;"",LEFT(E34,LEN(LEFT(D34,FIND(" ·",D34&amp;" ·")-1))+1)&lt;&gt;LEFT(D34,FIND(" ·",D34&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I34&lt;&gt;"",IFERROR(OR(I34&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D34,'08 Phases'!$B$9:$B$38,0)),I34&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D34,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
       <c r="I35" s="49" t="n"/>
       <c r="J35" s="49" t="n"/>
       <c r="K35" s="48">
-        <f>IF(C35="","",IF(D35="","⚠ Phase manquante",IF(AND(E35&lt;&gt;"",LEFT(E35,LEN(LEFT(D35,FIND(" ·",D35&amp;" ·")-1))+1)&lt;&gt;LEFT(D35,FIND(" ·",D35&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I35&lt;&gt;"",IFERROR(OR(I35&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D35,'07 Phases'!$B$9:$B$38,0)),I35&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D35,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C35="","",IF(D35="","⚠ Phase manquante",IF(AND(E35&lt;&gt;"",LEFT(E35,LEN(LEFT(D35,FIND(" ·",D35&amp;" ·")-1))+1)&lt;&gt;LEFT(D35,FIND(" ·",D35&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I35&lt;&gt;"",IFERROR(OR(I35&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D35,'08 Phases'!$B$9:$B$38,0)),I35&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D35,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9651,7 +9651,7 @@
       <c r="I36" s="49" t="n"/>
       <c r="J36" s="49" t="n"/>
       <c r="K36" s="48">
-        <f>IF(C36="","",IF(D36="","⚠ Phase manquante",IF(AND(E36&lt;&gt;"",LEFT(E36,LEN(LEFT(D36,FIND(" ·",D36&amp;" ·")-1))+1)&lt;&gt;LEFT(D36,FIND(" ·",D36&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I36&lt;&gt;"",IFERROR(OR(I36&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D36,'07 Phases'!$B$9:$B$38,0)),I36&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D36,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C36="","",IF(D36="","⚠ Phase manquante",IF(AND(E36&lt;&gt;"",LEFT(E36,LEN(LEFT(D36,FIND(" ·",D36&amp;" ·")-1))+1)&lt;&gt;LEFT(D36,FIND(" ·",D36&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I36&lt;&gt;"",IFERROR(OR(I36&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D36,'08 Phases'!$B$9:$B$38,0)),I36&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D36,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9669,7 +9669,7 @@
       <c r="I37" s="49" t="n"/>
       <c r="J37" s="49" t="n"/>
       <c r="K37" s="48">
-        <f>IF(C37="","",IF(D37="","⚠ Phase manquante",IF(AND(E37&lt;&gt;"",LEFT(E37,LEN(LEFT(D37,FIND(" ·",D37&amp;" ·")-1))+1)&lt;&gt;LEFT(D37,FIND(" ·",D37&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I37&lt;&gt;"",IFERROR(OR(I37&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D37,'07 Phases'!$B$9:$B$38,0)),I37&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D37,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C37="","",IF(D37="","⚠ Phase manquante",IF(AND(E37&lt;&gt;"",LEFT(E37,LEN(LEFT(D37,FIND(" ·",D37&amp;" ·")-1))+1)&lt;&gt;LEFT(D37,FIND(" ·",D37&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I37&lt;&gt;"",IFERROR(OR(I37&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D37,'08 Phases'!$B$9:$B$38,0)),I37&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D37,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       <c r="I38" s="49" t="n"/>
       <c r="J38" s="49" t="n"/>
       <c r="K38" s="48">
-        <f>IF(C38="","",IF(D38="","⚠ Phase manquante",IF(AND(E38&lt;&gt;"",LEFT(E38,LEN(LEFT(D38,FIND(" ·",D38&amp;" ·")-1))+1)&lt;&gt;LEFT(D38,FIND(" ·",D38&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I38&lt;&gt;"",IFERROR(OR(I38&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D38,'07 Phases'!$B$9:$B$38,0)),I38&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D38,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C38="","",IF(D38="","⚠ Phase manquante",IF(AND(E38&lt;&gt;"",LEFT(E38,LEN(LEFT(D38,FIND(" ·",D38&amp;" ·")-1))+1)&lt;&gt;LEFT(D38,FIND(" ·",D38&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I38&lt;&gt;"",IFERROR(OR(I38&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D38,'08 Phases'!$B$9:$B$38,0)),I38&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D38,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9705,7 +9705,7 @@
       <c r="I39" s="49" t="n"/>
       <c r="J39" s="49" t="n"/>
       <c r="K39" s="48">
-        <f>IF(C39="","",IF(D39="","⚠ Phase manquante",IF(AND(E39&lt;&gt;"",LEFT(E39,LEN(LEFT(D39,FIND(" ·",D39&amp;" ·")-1))+1)&lt;&gt;LEFT(D39,FIND(" ·",D39&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I39&lt;&gt;"",IFERROR(OR(I39&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D39,'07 Phases'!$B$9:$B$38,0)),I39&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D39,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C39="","",IF(D39="","⚠ Phase manquante",IF(AND(E39&lt;&gt;"",LEFT(E39,LEN(LEFT(D39,FIND(" ·",D39&amp;" ·")-1))+1)&lt;&gt;LEFT(D39,FIND(" ·",D39&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I39&lt;&gt;"",IFERROR(OR(I39&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D39,'08 Phases'!$B$9:$B$38,0)),I39&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D39,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9723,7 +9723,7 @@
       <c r="I40" s="49" t="n"/>
       <c r="J40" s="49" t="n"/>
       <c r="K40" s="48">
-        <f>IF(C40="","",IF(D40="","⚠ Phase manquante",IF(AND(E40&lt;&gt;"",LEFT(E40,LEN(LEFT(D40,FIND(" ·",D40&amp;" ·")-1))+1)&lt;&gt;LEFT(D40,FIND(" ·",D40&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I40&lt;&gt;"",IFERROR(OR(I40&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D40,'07 Phases'!$B$9:$B$38,0)),I40&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D40,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C40="","",IF(D40="","⚠ Phase manquante",IF(AND(E40&lt;&gt;"",LEFT(E40,LEN(LEFT(D40,FIND(" ·",D40&amp;" ·")-1))+1)&lt;&gt;LEFT(D40,FIND(" ·",D40&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I40&lt;&gt;"",IFERROR(OR(I40&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D40,'08 Phases'!$B$9:$B$38,0)),I40&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D40,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       <c r="I41" s="49" t="n"/>
       <c r="J41" s="49" t="n"/>
       <c r="K41" s="48">
-        <f>IF(C41="","",IF(D41="","⚠ Phase manquante",IF(AND(E41&lt;&gt;"",LEFT(E41,LEN(LEFT(D41,FIND(" ·",D41&amp;" ·")-1))+1)&lt;&gt;LEFT(D41,FIND(" ·",D41&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I41&lt;&gt;"",IFERROR(OR(I41&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D41,'07 Phases'!$B$9:$B$38,0)),I41&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D41,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C41="","",IF(D41="","⚠ Phase manquante",IF(AND(E41&lt;&gt;"",LEFT(E41,LEN(LEFT(D41,FIND(" ·",D41&amp;" ·")-1))+1)&lt;&gt;LEFT(D41,FIND(" ·",D41&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I41&lt;&gt;"",IFERROR(OR(I41&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D41,'08 Phases'!$B$9:$B$38,0)),I41&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D41,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9759,7 +9759,7 @@
       <c r="I42" s="49" t="n"/>
       <c r="J42" s="49" t="n"/>
       <c r="K42" s="48">
-        <f>IF(C42="","",IF(D42="","⚠ Phase manquante",IF(AND(E42&lt;&gt;"",LEFT(E42,LEN(LEFT(D42,FIND(" ·",D42&amp;" ·")-1))+1)&lt;&gt;LEFT(D42,FIND(" ·",D42&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I42&lt;&gt;"",IFERROR(OR(I42&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D42,'07 Phases'!$B$9:$B$38,0)),I42&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D42,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C42="","",IF(D42="","⚠ Phase manquante",IF(AND(E42&lt;&gt;"",LEFT(E42,LEN(LEFT(D42,FIND(" ·",D42&amp;" ·")-1))+1)&lt;&gt;LEFT(D42,FIND(" ·",D42&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I42&lt;&gt;"",IFERROR(OR(I42&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D42,'08 Phases'!$B$9:$B$38,0)),I42&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D42,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9777,7 +9777,7 @@
       <c r="I43" s="49" t="n"/>
       <c r="J43" s="49" t="n"/>
       <c r="K43" s="48">
-        <f>IF(C43="","",IF(D43="","⚠ Phase manquante",IF(AND(E43&lt;&gt;"",LEFT(E43,LEN(LEFT(D43,FIND(" ·",D43&amp;" ·")-1))+1)&lt;&gt;LEFT(D43,FIND(" ·",D43&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I43&lt;&gt;"",IFERROR(OR(I43&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D43,'07 Phases'!$B$9:$B$38,0)),I43&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D43,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C43="","",IF(D43="","⚠ Phase manquante",IF(AND(E43&lt;&gt;"",LEFT(E43,LEN(LEFT(D43,FIND(" ·",D43&amp;" ·")-1))+1)&lt;&gt;LEFT(D43,FIND(" ·",D43&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I43&lt;&gt;"",IFERROR(OR(I43&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D43,'08 Phases'!$B$9:$B$38,0)),I43&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D43,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9795,7 +9795,7 @@
       <c r="I44" s="49" t="n"/>
       <c r="J44" s="49" t="n"/>
       <c r="K44" s="48">
-        <f>IF(C44="","",IF(D44="","⚠ Phase manquante",IF(AND(E44&lt;&gt;"",LEFT(E44,LEN(LEFT(D44,FIND(" ·",D44&amp;" ·")-1))+1)&lt;&gt;LEFT(D44,FIND(" ·",D44&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I44&lt;&gt;"",IFERROR(OR(I44&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D44,'07 Phases'!$B$9:$B$38,0)),I44&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D44,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C44="","",IF(D44="","⚠ Phase manquante",IF(AND(E44&lt;&gt;"",LEFT(E44,LEN(LEFT(D44,FIND(" ·",D44&amp;" ·")-1))+1)&lt;&gt;LEFT(D44,FIND(" ·",D44&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I44&lt;&gt;"",IFERROR(OR(I44&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D44,'08 Phases'!$B$9:$B$38,0)),I44&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D44,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9813,7 +9813,7 @@
       <c r="I45" s="49" t="n"/>
       <c r="J45" s="49" t="n"/>
       <c r="K45" s="48">
-        <f>IF(C45="","",IF(D45="","⚠ Phase manquante",IF(AND(E45&lt;&gt;"",LEFT(E45,LEN(LEFT(D45,FIND(" ·",D45&amp;" ·")-1))+1)&lt;&gt;LEFT(D45,FIND(" ·",D45&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I45&lt;&gt;"",IFERROR(OR(I45&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D45,'07 Phases'!$B$9:$B$38,0)),I45&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D45,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C45="","",IF(D45="","⚠ Phase manquante",IF(AND(E45&lt;&gt;"",LEFT(E45,LEN(LEFT(D45,FIND(" ·",D45&amp;" ·")-1))+1)&lt;&gt;LEFT(D45,FIND(" ·",D45&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I45&lt;&gt;"",IFERROR(OR(I45&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D45,'08 Phases'!$B$9:$B$38,0)),I45&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D45,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9831,7 +9831,7 @@
       <c r="I46" s="49" t="n"/>
       <c r="J46" s="49" t="n"/>
       <c r="K46" s="48">
-        <f>IF(C46="","",IF(D46="","⚠ Phase manquante",IF(AND(E46&lt;&gt;"",LEFT(E46,LEN(LEFT(D46,FIND(" ·",D46&amp;" ·")-1))+1)&lt;&gt;LEFT(D46,FIND(" ·",D46&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I46&lt;&gt;"",IFERROR(OR(I46&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D46,'07 Phases'!$B$9:$B$38,0)),I46&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D46,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C46="","",IF(D46="","⚠ Phase manquante",IF(AND(E46&lt;&gt;"",LEFT(E46,LEN(LEFT(D46,FIND(" ·",D46&amp;" ·")-1))+1)&lt;&gt;LEFT(D46,FIND(" ·",D46&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I46&lt;&gt;"",IFERROR(OR(I46&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D46,'08 Phases'!$B$9:$B$38,0)),I46&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D46,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9849,7 +9849,7 @@
       <c r="I47" s="49" t="n"/>
       <c r="J47" s="49" t="n"/>
       <c r="K47" s="48">
-        <f>IF(C47="","",IF(D47="","⚠ Phase manquante",IF(AND(E47&lt;&gt;"",LEFT(E47,LEN(LEFT(D47,FIND(" ·",D47&amp;" ·")-1))+1)&lt;&gt;LEFT(D47,FIND(" ·",D47&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I47&lt;&gt;"",IFERROR(OR(I47&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D47,'07 Phases'!$B$9:$B$38,0)),I47&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D47,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C47="","",IF(D47="","⚠ Phase manquante",IF(AND(E47&lt;&gt;"",LEFT(E47,LEN(LEFT(D47,FIND(" ·",D47&amp;" ·")-1))+1)&lt;&gt;LEFT(D47,FIND(" ·",D47&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I47&lt;&gt;"",IFERROR(OR(I47&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D47,'08 Phases'!$B$9:$B$38,0)),I47&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D47,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       <c r="I48" s="49" t="n"/>
       <c r="J48" s="49" t="n"/>
       <c r="K48" s="48">
-        <f>IF(C48="","",IF(D48="","⚠ Phase manquante",IF(AND(E48&lt;&gt;"",LEFT(E48,LEN(LEFT(D48,FIND(" ·",D48&amp;" ·")-1))+1)&lt;&gt;LEFT(D48,FIND(" ·",D48&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I48&lt;&gt;"",IFERROR(OR(I48&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D48,'07 Phases'!$B$9:$B$38,0)),I48&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D48,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C48="","",IF(D48="","⚠ Phase manquante",IF(AND(E48&lt;&gt;"",LEFT(E48,LEN(LEFT(D48,FIND(" ·",D48&amp;" ·")-1))+1)&lt;&gt;LEFT(D48,FIND(" ·",D48&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I48&lt;&gt;"",IFERROR(OR(I48&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D48,'08 Phases'!$B$9:$B$38,0)),I48&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D48,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9885,7 +9885,7 @@
       <c r="I49" s="49" t="n"/>
       <c r="J49" s="49" t="n"/>
       <c r="K49" s="48">
-        <f>IF(C49="","",IF(D49="","⚠ Phase manquante",IF(AND(E49&lt;&gt;"",LEFT(E49,LEN(LEFT(D49,FIND(" ·",D49&amp;" ·")-1))+1)&lt;&gt;LEFT(D49,FIND(" ·",D49&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I49&lt;&gt;"",IFERROR(OR(I49&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D49,'07 Phases'!$B$9:$B$38,0)),I49&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D49,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C49="","",IF(D49="","⚠ Phase manquante",IF(AND(E49&lt;&gt;"",LEFT(E49,LEN(LEFT(D49,FIND(" ·",D49&amp;" ·")-1))+1)&lt;&gt;LEFT(D49,FIND(" ·",D49&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I49&lt;&gt;"",IFERROR(OR(I49&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D49,'08 Phases'!$B$9:$B$38,0)),I49&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D49,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9903,7 +9903,7 @@
       <c r="I50" s="49" t="n"/>
       <c r="J50" s="49" t="n"/>
       <c r="K50" s="48">
-        <f>IF(C50="","",IF(D50="","⚠ Phase manquante",IF(AND(E50&lt;&gt;"",LEFT(E50,LEN(LEFT(D50,FIND(" ·",D50&amp;" ·")-1))+1)&lt;&gt;LEFT(D50,FIND(" ·",D50&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I50&lt;&gt;"",IFERROR(OR(I50&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D50,'07 Phases'!$B$9:$B$38,0)),I50&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D50,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C50="","",IF(D50="","⚠ Phase manquante",IF(AND(E50&lt;&gt;"",LEFT(E50,LEN(LEFT(D50,FIND(" ·",D50&amp;" ·")-1))+1)&lt;&gt;LEFT(D50,FIND(" ·",D50&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I50&lt;&gt;"",IFERROR(OR(I50&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D50,'08 Phases'!$B$9:$B$38,0)),I50&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D50,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9921,7 +9921,7 @@
       <c r="I51" s="49" t="n"/>
       <c r="J51" s="49" t="n"/>
       <c r="K51" s="48">
-        <f>IF(C51="","",IF(D51="","⚠ Phase manquante",IF(AND(E51&lt;&gt;"",LEFT(E51,LEN(LEFT(D51,FIND(" ·",D51&amp;" ·")-1))+1)&lt;&gt;LEFT(D51,FIND(" ·",D51&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I51&lt;&gt;"",IFERROR(OR(I51&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D51,'07 Phases'!$B$9:$B$38,0)),I51&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D51,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C51="","",IF(D51="","⚠ Phase manquante",IF(AND(E51&lt;&gt;"",LEFT(E51,LEN(LEFT(D51,FIND(" ·",D51&amp;" ·")-1))+1)&lt;&gt;LEFT(D51,FIND(" ·",D51&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I51&lt;&gt;"",IFERROR(OR(I51&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D51,'08 Phases'!$B$9:$B$38,0)),I51&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D51,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9939,7 +9939,7 @@
       <c r="I52" s="49" t="n"/>
       <c r="J52" s="49" t="n"/>
       <c r="K52" s="48">
-        <f>IF(C52="","",IF(D52="","⚠ Phase manquante",IF(AND(E52&lt;&gt;"",LEFT(E52,LEN(LEFT(D52,FIND(" ·",D52&amp;" ·")-1))+1)&lt;&gt;LEFT(D52,FIND(" ·",D52&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I52&lt;&gt;"",IFERROR(OR(I52&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D52,'07 Phases'!$B$9:$B$38,0)),I52&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D52,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C52="","",IF(D52="","⚠ Phase manquante",IF(AND(E52&lt;&gt;"",LEFT(E52,LEN(LEFT(D52,FIND(" ·",D52&amp;" ·")-1))+1)&lt;&gt;LEFT(D52,FIND(" ·",D52&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I52&lt;&gt;"",IFERROR(OR(I52&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D52,'08 Phases'!$B$9:$B$38,0)),I52&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D52,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9957,7 +9957,7 @@
       <c r="I53" s="49" t="n"/>
       <c r="J53" s="49" t="n"/>
       <c r="K53" s="48">
-        <f>IF(C53="","",IF(D53="","⚠ Phase manquante",IF(AND(E53&lt;&gt;"",LEFT(E53,LEN(LEFT(D53,FIND(" ·",D53&amp;" ·")-1))+1)&lt;&gt;LEFT(D53,FIND(" ·",D53&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I53&lt;&gt;"",IFERROR(OR(I53&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D53,'07 Phases'!$B$9:$B$38,0)),I53&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D53,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C53="","",IF(D53="","⚠ Phase manquante",IF(AND(E53&lt;&gt;"",LEFT(E53,LEN(LEFT(D53,FIND(" ·",D53&amp;" ·")-1))+1)&lt;&gt;LEFT(D53,FIND(" ·",D53&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I53&lt;&gt;"",IFERROR(OR(I53&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D53,'08 Phases'!$B$9:$B$38,0)),I53&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D53,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9975,7 +9975,7 @@
       <c r="I54" s="49" t="n"/>
       <c r="J54" s="49" t="n"/>
       <c r="K54" s="48">
-        <f>IF(C54="","",IF(D54="","⚠ Phase manquante",IF(AND(E54&lt;&gt;"",LEFT(E54,LEN(LEFT(D54,FIND(" ·",D54&amp;" ·")-1))+1)&lt;&gt;LEFT(D54,FIND(" ·",D54&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I54&lt;&gt;"",IFERROR(OR(I54&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D54,'07 Phases'!$B$9:$B$38,0)),I54&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D54,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C54="","",IF(D54="","⚠ Phase manquante",IF(AND(E54&lt;&gt;"",LEFT(E54,LEN(LEFT(D54,FIND(" ·",D54&amp;" ·")-1))+1)&lt;&gt;LEFT(D54,FIND(" ·",D54&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I54&lt;&gt;"",IFERROR(OR(I54&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D54,'08 Phases'!$B$9:$B$38,0)),I54&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D54,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -9993,7 +9993,7 @@
       <c r="I55" s="49" t="n"/>
       <c r="J55" s="49" t="n"/>
       <c r="K55" s="48">
-        <f>IF(C55="","",IF(D55="","⚠ Phase manquante",IF(AND(E55&lt;&gt;"",LEFT(E55,LEN(LEFT(D55,FIND(" ·",D55&amp;" ·")-1))+1)&lt;&gt;LEFT(D55,FIND(" ·",D55&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I55&lt;&gt;"",IFERROR(OR(I55&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D55,'07 Phases'!$B$9:$B$38,0)),I55&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D55,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C55="","",IF(D55="","⚠ Phase manquante",IF(AND(E55&lt;&gt;"",LEFT(E55,LEN(LEFT(D55,FIND(" ·",D55&amp;" ·")-1))+1)&lt;&gt;LEFT(D55,FIND(" ·",D55&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I55&lt;&gt;"",IFERROR(OR(I55&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D55,'08 Phases'!$B$9:$B$38,0)),I55&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D55,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10011,7 +10011,7 @@
       <c r="I56" s="49" t="n"/>
       <c r="J56" s="49" t="n"/>
       <c r="K56" s="48">
-        <f>IF(C56="","",IF(D56="","⚠ Phase manquante",IF(AND(E56&lt;&gt;"",LEFT(E56,LEN(LEFT(D56,FIND(" ·",D56&amp;" ·")-1))+1)&lt;&gt;LEFT(D56,FIND(" ·",D56&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I56&lt;&gt;"",IFERROR(OR(I56&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D56,'07 Phases'!$B$9:$B$38,0)),I56&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D56,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C56="","",IF(D56="","⚠ Phase manquante",IF(AND(E56&lt;&gt;"",LEFT(E56,LEN(LEFT(D56,FIND(" ·",D56&amp;" ·")-1))+1)&lt;&gt;LEFT(D56,FIND(" ·",D56&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I56&lt;&gt;"",IFERROR(OR(I56&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D56,'08 Phases'!$B$9:$B$38,0)),I56&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D56,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10029,7 +10029,7 @@
       <c r="I57" s="49" t="n"/>
       <c r="J57" s="49" t="n"/>
       <c r="K57" s="48">
-        <f>IF(C57="","",IF(D57="","⚠ Phase manquante",IF(AND(E57&lt;&gt;"",LEFT(E57,LEN(LEFT(D57,FIND(" ·",D57&amp;" ·")-1))+1)&lt;&gt;LEFT(D57,FIND(" ·",D57&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I57&lt;&gt;"",IFERROR(OR(I57&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D57,'07 Phases'!$B$9:$B$38,0)),I57&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D57,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C57="","",IF(D57="","⚠ Phase manquante",IF(AND(E57&lt;&gt;"",LEFT(E57,LEN(LEFT(D57,FIND(" ·",D57&amp;" ·")-1))+1)&lt;&gt;LEFT(D57,FIND(" ·",D57&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I57&lt;&gt;"",IFERROR(OR(I57&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D57,'08 Phases'!$B$9:$B$38,0)),I57&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D57,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
       <c r="I58" s="49" t="n"/>
       <c r="J58" s="49" t="n"/>
       <c r="K58" s="48">
-        <f>IF(C58="","",IF(D58="","⚠ Phase manquante",IF(AND(E58&lt;&gt;"",LEFT(E58,LEN(LEFT(D58,FIND(" ·",D58&amp;" ·")-1))+1)&lt;&gt;LEFT(D58,FIND(" ·",D58&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I58&lt;&gt;"",IFERROR(OR(I58&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D58,'07 Phases'!$B$9:$B$38,0)),I58&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D58,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C58="","",IF(D58="","⚠ Phase manquante",IF(AND(E58&lt;&gt;"",LEFT(E58,LEN(LEFT(D58,FIND(" ·",D58&amp;" ·")-1))+1)&lt;&gt;LEFT(D58,FIND(" ·",D58&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I58&lt;&gt;"",IFERROR(OR(I58&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D58,'08 Phases'!$B$9:$B$38,0)),I58&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D58,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
       <c r="I59" s="49" t="n"/>
       <c r="J59" s="49" t="n"/>
       <c r="K59" s="48">
-        <f>IF(C59="","",IF(D59="","⚠ Phase manquante",IF(AND(E59&lt;&gt;"",LEFT(E59,LEN(LEFT(D59,FIND(" ·",D59&amp;" ·")-1))+1)&lt;&gt;LEFT(D59,FIND(" ·",D59&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I59&lt;&gt;"",IFERROR(OR(I59&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D59,'07 Phases'!$B$9:$B$38,0)),I59&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D59,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C59="","",IF(D59="","⚠ Phase manquante",IF(AND(E59&lt;&gt;"",LEFT(E59,LEN(LEFT(D59,FIND(" ·",D59&amp;" ·")-1))+1)&lt;&gt;LEFT(D59,FIND(" ·",D59&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I59&lt;&gt;"",IFERROR(OR(I59&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D59,'08 Phases'!$B$9:$B$38,0)),I59&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D59,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10083,7 +10083,7 @@
       <c r="I60" s="49" t="n"/>
       <c r="J60" s="49" t="n"/>
       <c r="K60" s="48">
-        <f>IF(C60="","",IF(D60="","⚠ Phase manquante",IF(AND(E60&lt;&gt;"",LEFT(E60,LEN(LEFT(D60,FIND(" ·",D60&amp;" ·")-1))+1)&lt;&gt;LEFT(D60,FIND(" ·",D60&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I60&lt;&gt;"",IFERROR(OR(I60&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D60,'07 Phases'!$B$9:$B$38,0)),I60&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D60,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C60="","",IF(D60="","⚠ Phase manquante",IF(AND(E60&lt;&gt;"",LEFT(E60,LEN(LEFT(D60,FIND(" ·",D60&amp;" ·")-1))+1)&lt;&gt;LEFT(D60,FIND(" ·",D60&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I60&lt;&gt;"",IFERROR(OR(I60&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D60,'08 Phases'!$B$9:$B$38,0)),I60&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D60,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10101,7 +10101,7 @@
       <c r="I61" s="49" t="n"/>
       <c r="J61" s="49" t="n"/>
       <c r="K61" s="48">
-        <f>IF(C61="","",IF(D61="","⚠ Phase manquante",IF(AND(E61&lt;&gt;"",LEFT(E61,LEN(LEFT(D61,FIND(" ·",D61&amp;" ·")-1))+1)&lt;&gt;LEFT(D61,FIND(" ·",D61&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I61&lt;&gt;"",IFERROR(OR(I61&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D61,'07 Phases'!$B$9:$B$38,0)),I61&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D61,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C61="","",IF(D61="","⚠ Phase manquante",IF(AND(E61&lt;&gt;"",LEFT(E61,LEN(LEFT(D61,FIND(" ·",D61&amp;" ·")-1))+1)&lt;&gt;LEFT(D61,FIND(" ·",D61&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I61&lt;&gt;"",IFERROR(OR(I61&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D61,'08 Phases'!$B$9:$B$38,0)),I61&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D61,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10119,7 +10119,7 @@
       <c r="I62" s="49" t="n"/>
       <c r="J62" s="49" t="n"/>
       <c r="K62" s="48">
-        <f>IF(C62="","",IF(D62="","⚠ Phase manquante",IF(AND(E62&lt;&gt;"",LEFT(E62,LEN(LEFT(D62,FIND(" ·",D62&amp;" ·")-1))+1)&lt;&gt;LEFT(D62,FIND(" ·",D62&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I62&lt;&gt;"",IFERROR(OR(I62&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D62,'07 Phases'!$B$9:$B$38,0)),I62&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D62,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C62="","",IF(D62="","⚠ Phase manquante",IF(AND(E62&lt;&gt;"",LEFT(E62,LEN(LEFT(D62,FIND(" ·",D62&amp;" ·")-1))+1)&lt;&gt;LEFT(D62,FIND(" ·",D62&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I62&lt;&gt;"",IFERROR(OR(I62&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D62,'08 Phases'!$B$9:$B$38,0)),I62&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D62,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10137,7 +10137,7 @@
       <c r="I63" s="49" t="n"/>
       <c r="J63" s="49" t="n"/>
       <c r="K63" s="48">
-        <f>IF(C63="","",IF(D63="","⚠ Phase manquante",IF(AND(E63&lt;&gt;"",LEFT(E63,LEN(LEFT(D63,FIND(" ·",D63&amp;" ·")-1))+1)&lt;&gt;LEFT(D63,FIND(" ·",D63&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I63&lt;&gt;"",IFERROR(OR(I63&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D63,'07 Phases'!$B$9:$B$38,0)),I63&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D63,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C63="","",IF(D63="","⚠ Phase manquante",IF(AND(E63&lt;&gt;"",LEFT(E63,LEN(LEFT(D63,FIND(" ·",D63&amp;" ·")-1))+1)&lt;&gt;LEFT(D63,FIND(" ·",D63&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I63&lt;&gt;"",IFERROR(OR(I63&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D63,'08 Phases'!$B$9:$B$38,0)),I63&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D63,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       <c r="I64" s="49" t="n"/>
       <c r="J64" s="49" t="n"/>
       <c r="K64" s="48">
-        <f>IF(C64="","",IF(D64="","⚠ Phase manquante",IF(AND(E64&lt;&gt;"",LEFT(E64,LEN(LEFT(D64,FIND(" ·",D64&amp;" ·")-1))+1)&lt;&gt;LEFT(D64,FIND(" ·",D64&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I64&lt;&gt;"",IFERROR(OR(I64&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D64,'07 Phases'!$B$9:$B$38,0)),I64&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D64,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C64="","",IF(D64="","⚠ Phase manquante",IF(AND(E64&lt;&gt;"",LEFT(E64,LEN(LEFT(D64,FIND(" ·",D64&amp;" ·")-1))+1)&lt;&gt;LEFT(D64,FIND(" ·",D64&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I64&lt;&gt;"",IFERROR(OR(I64&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D64,'08 Phases'!$B$9:$B$38,0)),I64&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D64,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10173,7 +10173,7 @@
       <c r="I65" s="49" t="n"/>
       <c r="J65" s="49" t="n"/>
       <c r="K65" s="48">
-        <f>IF(C65="","",IF(D65="","⚠ Phase manquante",IF(AND(E65&lt;&gt;"",LEFT(E65,LEN(LEFT(D65,FIND(" ·",D65&amp;" ·")-1))+1)&lt;&gt;LEFT(D65,FIND(" ·",D65&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I65&lt;&gt;"",IFERROR(OR(I65&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D65,'07 Phases'!$B$9:$B$38,0)),I65&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D65,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C65="","",IF(D65="","⚠ Phase manquante",IF(AND(E65&lt;&gt;"",LEFT(E65,LEN(LEFT(D65,FIND(" ·",D65&amp;" ·")-1))+1)&lt;&gt;LEFT(D65,FIND(" ·",D65&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I65&lt;&gt;"",IFERROR(OR(I65&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D65,'08 Phases'!$B$9:$B$38,0)),I65&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D65,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10191,7 +10191,7 @@
       <c r="I66" s="49" t="n"/>
       <c r="J66" s="49" t="n"/>
       <c r="K66" s="48">
-        <f>IF(C66="","",IF(D66="","⚠ Phase manquante",IF(AND(E66&lt;&gt;"",LEFT(E66,LEN(LEFT(D66,FIND(" ·",D66&amp;" ·")-1))+1)&lt;&gt;LEFT(D66,FIND(" ·",D66&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I66&lt;&gt;"",IFERROR(OR(I66&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D66,'07 Phases'!$B$9:$B$38,0)),I66&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D66,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C66="","",IF(D66="","⚠ Phase manquante",IF(AND(E66&lt;&gt;"",LEFT(E66,LEN(LEFT(D66,FIND(" ·",D66&amp;" ·")-1))+1)&lt;&gt;LEFT(D66,FIND(" ·",D66&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I66&lt;&gt;"",IFERROR(OR(I66&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D66,'08 Phases'!$B$9:$B$38,0)),I66&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D66,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10209,7 +10209,7 @@
       <c r="I67" s="49" t="n"/>
       <c r="J67" s="49" t="n"/>
       <c r="K67" s="48">
-        <f>IF(C67="","",IF(D67="","⚠ Phase manquante",IF(AND(E67&lt;&gt;"",LEFT(E67,LEN(LEFT(D67,FIND(" ·",D67&amp;" ·")-1))+1)&lt;&gt;LEFT(D67,FIND(" ·",D67&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I67&lt;&gt;"",IFERROR(OR(I67&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D67,'07 Phases'!$B$9:$B$38,0)),I67&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D67,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C67="","",IF(D67="","⚠ Phase manquante",IF(AND(E67&lt;&gt;"",LEFT(E67,LEN(LEFT(D67,FIND(" ·",D67&amp;" ·")-1))+1)&lt;&gt;LEFT(D67,FIND(" ·",D67&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I67&lt;&gt;"",IFERROR(OR(I67&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D67,'08 Phases'!$B$9:$B$38,0)),I67&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D67,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10227,7 +10227,7 @@
       <c r="I68" s="49" t="n"/>
       <c r="J68" s="49" t="n"/>
       <c r="K68" s="48">
-        <f>IF(C68="","",IF(D68="","⚠ Phase manquante",IF(AND(E68&lt;&gt;"",LEFT(E68,LEN(LEFT(D68,FIND(" ·",D68&amp;" ·")-1))+1)&lt;&gt;LEFT(D68,FIND(" ·",D68&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I68&lt;&gt;"",IFERROR(OR(I68&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D68,'07 Phases'!$B$9:$B$38,0)),I68&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D68,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C68="","",IF(D68="","⚠ Phase manquante",IF(AND(E68&lt;&gt;"",LEFT(E68,LEN(LEFT(D68,FIND(" ·",D68&amp;" ·")-1))+1)&lt;&gt;LEFT(D68,FIND(" ·",D68&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I68&lt;&gt;"",IFERROR(OR(I68&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D68,'08 Phases'!$B$9:$B$38,0)),I68&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D68,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
       <c r="I69" s="49" t="n"/>
       <c r="J69" s="49" t="n"/>
       <c r="K69" s="48">
-        <f>IF(C69="","",IF(D69="","⚠ Phase manquante",IF(AND(E69&lt;&gt;"",LEFT(E69,LEN(LEFT(D69,FIND(" ·",D69&amp;" ·")-1))+1)&lt;&gt;LEFT(D69,FIND(" ·",D69&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I69&lt;&gt;"",IFERROR(OR(I69&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D69,'07 Phases'!$B$9:$B$38,0)),I69&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D69,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C69="","",IF(D69="","⚠ Phase manquante",IF(AND(E69&lt;&gt;"",LEFT(E69,LEN(LEFT(D69,FIND(" ·",D69&amp;" ·")-1))+1)&lt;&gt;LEFT(D69,FIND(" ·",D69&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I69&lt;&gt;"",IFERROR(OR(I69&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D69,'08 Phases'!$B$9:$B$38,0)),I69&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D69,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       <c r="I70" s="49" t="n"/>
       <c r="J70" s="49" t="n"/>
       <c r="K70" s="48">
-        <f>IF(C70="","",IF(D70="","⚠ Phase manquante",IF(AND(E70&lt;&gt;"",LEFT(E70,LEN(LEFT(D70,FIND(" ·",D70&amp;" ·")-1))+1)&lt;&gt;LEFT(D70,FIND(" ·",D70&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I70&lt;&gt;"",IFERROR(OR(I70&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D70,'07 Phases'!$B$9:$B$38,0)),I70&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D70,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C70="","",IF(D70="","⚠ Phase manquante",IF(AND(E70&lt;&gt;"",LEFT(E70,LEN(LEFT(D70,FIND(" ·",D70&amp;" ·")-1))+1)&lt;&gt;LEFT(D70,FIND(" ·",D70&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I70&lt;&gt;"",IFERROR(OR(I70&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D70,'08 Phases'!$B$9:$B$38,0)),I70&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D70,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       <c r="I71" s="49" t="n"/>
       <c r="J71" s="49" t="n"/>
       <c r="K71" s="48">
-        <f>IF(C71="","",IF(D71="","⚠ Phase manquante",IF(AND(E71&lt;&gt;"",LEFT(E71,LEN(LEFT(D71,FIND(" ·",D71&amp;" ·")-1))+1)&lt;&gt;LEFT(D71,FIND(" ·",D71&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I71&lt;&gt;"",IFERROR(OR(I71&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D71,'07 Phases'!$B$9:$B$38,0)),I71&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D71,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C71="","",IF(D71="","⚠ Phase manquante",IF(AND(E71&lt;&gt;"",LEFT(E71,LEN(LEFT(D71,FIND(" ·",D71&amp;" ·")-1))+1)&lt;&gt;LEFT(D71,FIND(" ·",D71&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I71&lt;&gt;"",IFERROR(OR(I71&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D71,'08 Phases'!$B$9:$B$38,0)),I71&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D71,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10299,7 +10299,7 @@
       <c r="I72" s="49" t="n"/>
       <c r="J72" s="49" t="n"/>
       <c r="K72" s="48">
-        <f>IF(C72="","",IF(D72="","⚠ Phase manquante",IF(AND(E72&lt;&gt;"",LEFT(E72,LEN(LEFT(D72,FIND(" ·",D72&amp;" ·")-1))+1)&lt;&gt;LEFT(D72,FIND(" ·",D72&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I72&lt;&gt;"",IFERROR(OR(I72&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D72,'07 Phases'!$B$9:$B$38,0)),I72&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D72,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C72="","",IF(D72="","⚠ Phase manquante",IF(AND(E72&lt;&gt;"",LEFT(E72,LEN(LEFT(D72,FIND(" ·",D72&amp;" ·")-1))+1)&lt;&gt;LEFT(D72,FIND(" ·",D72&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I72&lt;&gt;"",IFERROR(OR(I72&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D72,'08 Phases'!$B$9:$B$38,0)),I72&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D72,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10317,7 +10317,7 @@
       <c r="I73" s="49" t="n"/>
       <c r="J73" s="49" t="n"/>
       <c r="K73" s="48">
-        <f>IF(C73="","",IF(D73="","⚠ Phase manquante",IF(AND(E73&lt;&gt;"",LEFT(E73,LEN(LEFT(D73,FIND(" ·",D73&amp;" ·")-1))+1)&lt;&gt;LEFT(D73,FIND(" ·",D73&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I73&lt;&gt;"",IFERROR(OR(I73&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D73,'07 Phases'!$B$9:$B$38,0)),I73&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D73,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C73="","",IF(D73="","⚠ Phase manquante",IF(AND(E73&lt;&gt;"",LEFT(E73,LEN(LEFT(D73,FIND(" ·",D73&amp;" ·")-1))+1)&lt;&gt;LEFT(D73,FIND(" ·",D73&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I73&lt;&gt;"",IFERROR(OR(I73&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D73,'08 Phases'!$B$9:$B$38,0)),I73&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D73,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10335,7 +10335,7 @@
       <c r="I74" s="49" t="n"/>
       <c r="J74" s="49" t="n"/>
       <c r="K74" s="48">
-        <f>IF(C74="","",IF(D74="","⚠ Phase manquante",IF(AND(E74&lt;&gt;"",LEFT(E74,LEN(LEFT(D74,FIND(" ·",D74&amp;" ·")-1))+1)&lt;&gt;LEFT(D74,FIND(" ·",D74&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I74&lt;&gt;"",IFERROR(OR(I74&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D74,'07 Phases'!$B$9:$B$38,0)),I74&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D74,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C74="","",IF(D74="","⚠ Phase manquante",IF(AND(E74&lt;&gt;"",LEFT(E74,LEN(LEFT(D74,FIND(" ·",D74&amp;" ·")-1))+1)&lt;&gt;LEFT(D74,FIND(" ·",D74&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I74&lt;&gt;"",IFERROR(OR(I74&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D74,'08 Phases'!$B$9:$B$38,0)),I74&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D74,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10353,7 +10353,7 @@
       <c r="I75" s="49" t="n"/>
       <c r="J75" s="49" t="n"/>
       <c r="K75" s="48">
-        <f>IF(C75="","",IF(D75="","⚠ Phase manquante",IF(AND(E75&lt;&gt;"",LEFT(E75,LEN(LEFT(D75,FIND(" ·",D75&amp;" ·")-1))+1)&lt;&gt;LEFT(D75,FIND(" ·",D75&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I75&lt;&gt;"",IFERROR(OR(I75&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D75,'07 Phases'!$B$9:$B$38,0)),I75&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D75,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C75="","",IF(D75="","⚠ Phase manquante",IF(AND(E75&lt;&gt;"",LEFT(E75,LEN(LEFT(D75,FIND(" ·",D75&amp;" ·")-1))+1)&lt;&gt;LEFT(D75,FIND(" ·",D75&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I75&lt;&gt;"",IFERROR(OR(I75&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D75,'08 Phases'!$B$9:$B$38,0)),I75&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D75,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10371,7 +10371,7 @@
       <c r="I76" s="49" t="n"/>
       <c r="J76" s="49" t="n"/>
       <c r="K76" s="48">
-        <f>IF(C76="","",IF(D76="","⚠ Phase manquante",IF(AND(E76&lt;&gt;"",LEFT(E76,LEN(LEFT(D76,FIND(" ·",D76&amp;" ·")-1))+1)&lt;&gt;LEFT(D76,FIND(" ·",D76&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I76&lt;&gt;"",IFERROR(OR(I76&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D76,'07 Phases'!$B$9:$B$38,0)),I76&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D76,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C76="","",IF(D76="","⚠ Phase manquante",IF(AND(E76&lt;&gt;"",LEFT(E76,LEN(LEFT(D76,FIND(" ·",D76&amp;" ·")-1))+1)&lt;&gt;LEFT(D76,FIND(" ·",D76&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I76&lt;&gt;"",IFERROR(OR(I76&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D76,'08 Phases'!$B$9:$B$38,0)),I76&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D76,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10389,7 +10389,7 @@
       <c r="I77" s="49" t="n"/>
       <c r="J77" s="49" t="n"/>
       <c r="K77" s="48">
-        <f>IF(C77="","",IF(D77="","⚠ Phase manquante",IF(AND(E77&lt;&gt;"",LEFT(E77,LEN(LEFT(D77,FIND(" ·",D77&amp;" ·")-1))+1)&lt;&gt;LEFT(D77,FIND(" ·",D77&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I77&lt;&gt;"",IFERROR(OR(I77&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D77,'07 Phases'!$B$9:$B$38,0)),I77&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D77,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C77="","",IF(D77="","⚠ Phase manquante",IF(AND(E77&lt;&gt;"",LEFT(E77,LEN(LEFT(D77,FIND(" ·",D77&amp;" ·")-1))+1)&lt;&gt;LEFT(D77,FIND(" ·",D77&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I77&lt;&gt;"",IFERROR(OR(I77&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D77,'08 Phases'!$B$9:$B$38,0)),I77&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D77,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10407,7 +10407,7 @@
       <c r="I78" s="49" t="n"/>
       <c r="J78" s="49" t="n"/>
       <c r="K78" s="48">
-        <f>IF(C78="","",IF(D78="","⚠ Phase manquante",IF(AND(E78&lt;&gt;"",LEFT(E78,LEN(LEFT(D78,FIND(" ·",D78&amp;" ·")-1))+1)&lt;&gt;LEFT(D78,FIND(" ·",D78&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I78&lt;&gt;"",IFERROR(OR(I78&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D78,'07 Phases'!$B$9:$B$38,0)),I78&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D78,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C78="","",IF(D78="","⚠ Phase manquante",IF(AND(E78&lt;&gt;"",LEFT(E78,LEN(LEFT(D78,FIND(" ·",D78&amp;" ·")-1))+1)&lt;&gt;LEFT(D78,FIND(" ·",D78&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I78&lt;&gt;"",IFERROR(OR(I78&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D78,'08 Phases'!$B$9:$B$38,0)),I78&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D78,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10425,7 +10425,7 @@
       <c r="I79" s="49" t="n"/>
       <c r="J79" s="49" t="n"/>
       <c r="K79" s="48">
-        <f>IF(C79="","",IF(D79="","⚠ Phase manquante",IF(AND(E79&lt;&gt;"",LEFT(E79,LEN(LEFT(D79,FIND(" ·",D79&amp;" ·")-1))+1)&lt;&gt;LEFT(D79,FIND(" ·",D79&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I79&lt;&gt;"",IFERROR(OR(I79&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D79,'07 Phases'!$B$9:$B$38,0)),I79&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D79,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C79="","",IF(D79="","⚠ Phase manquante",IF(AND(E79&lt;&gt;"",LEFT(E79,LEN(LEFT(D79,FIND(" ·",D79&amp;" ·")-1))+1)&lt;&gt;LEFT(D79,FIND(" ·",D79&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I79&lt;&gt;"",IFERROR(OR(I79&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D79,'08 Phases'!$B$9:$B$38,0)),I79&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D79,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10443,7 +10443,7 @@
       <c r="I80" s="49" t="n"/>
       <c r="J80" s="49" t="n"/>
       <c r="K80" s="48">
-        <f>IF(C80="","",IF(D80="","⚠ Phase manquante",IF(AND(E80&lt;&gt;"",LEFT(E80,LEN(LEFT(D80,FIND(" ·",D80&amp;" ·")-1))+1)&lt;&gt;LEFT(D80,FIND(" ·",D80&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I80&lt;&gt;"",IFERROR(OR(I80&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D80,'07 Phases'!$B$9:$B$38,0)),I80&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D80,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C80="","",IF(D80="","⚠ Phase manquante",IF(AND(E80&lt;&gt;"",LEFT(E80,LEN(LEFT(D80,FIND(" ·",D80&amp;" ·")-1))+1)&lt;&gt;LEFT(D80,FIND(" ·",D80&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I80&lt;&gt;"",IFERROR(OR(I80&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D80,'08 Phases'!$B$9:$B$38,0)),I80&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D80,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10461,7 +10461,7 @@
       <c r="I81" s="49" t="n"/>
       <c r="J81" s="49" t="n"/>
       <c r="K81" s="48">
-        <f>IF(C81="","",IF(D81="","⚠ Phase manquante",IF(AND(E81&lt;&gt;"",LEFT(E81,LEN(LEFT(D81,FIND(" ·",D81&amp;" ·")-1))+1)&lt;&gt;LEFT(D81,FIND(" ·",D81&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I81&lt;&gt;"",IFERROR(OR(I81&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D81,'07 Phases'!$B$9:$B$38,0)),I81&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D81,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C81="","",IF(D81="","⚠ Phase manquante",IF(AND(E81&lt;&gt;"",LEFT(E81,LEN(LEFT(D81,FIND(" ·",D81&amp;" ·")-1))+1)&lt;&gt;LEFT(D81,FIND(" ·",D81&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I81&lt;&gt;"",IFERROR(OR(I81&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D81,'08 Phases'!$B$9:$B$38,0)),I81&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D81,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10479,7 +10479,7 @@
       <c r="I82" s="49" t="n"/>
       <c r="J82" s="49" t="n"/>
       <c r="K82" s="48">
-        <f>IF(C82="","",IF(D82="","⚠ Phase manquante",IF(AND(E82&lt;&gt;"",LEFT(E82,LEN(LEFT(D82,FIND(" ·",D82&amp;" ·")-1))+1)&lt;&gt;LEFT(D82,FIND(" ·",D82&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I82&lt;&gt;"",IFERROR(OR(I82&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D82,'07 Phases'!$B$9:$B$38,0)),I82&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D82,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C82="","",IF(D82="","⚠ Phase manquante",IF(AND(E82&lt;&gt;"",LEFT(E82,LEN(LEFT(D82,FIND(" ·",D82&amp;" ·")-1))+1)&lt;&gt;LEFT(D82,FIND(" ·",D82&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I82&lt;&gt;"",IFERROR(OR(I82&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D82,'08 Phases'!$B$9:$B$38,0)),I82&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D82,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10497,7 +10497,7 @@
       <c r="I83" s="49" t="n"/>
       <c r="J83" s="49" t="n"/>
       <c r="K83" s="48">
-        <f>IF(C83="","",IF(D83="","⚠ Phase manquante",IF(AND(E83&lt;&gt;"",LEFT(E83,LEN(LEFT(D83,FIND(" ·",D83&amp;" ·")-1))+1)&lt;&gt;LEFT(D83,FIND(" ·",D83&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I83&lt;&gt;"",IFERROR(OR(I83&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D83,'07 Phases'!$B$9:$B$38,0)),I83&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D83,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C83="","",IF(D83="","⚠ Phase manquante",IF(AND(E83&lt;&gt;"",LEFT(E83,LEN(LEFT(D83,FIND(" ·",D83&amp;" ·")-1))+1)&lt;&gt;LEFT(D83,FIND(" ·",D83&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I83&lt;&gt;"",IFERROR(OR(I83&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D83,'08 Phases'!$B$9:$B$38,0)),I83&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D83,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10515,7 +10515,7 @@
       <c r="I84" s="49" t="n"/>
       <c r="J84" s="49" t="n"/>
       <c r="K84" s="48">
-        <f>IF(C84="","",IF(D84="","⚠ Phase manquante",IF(AND(E84&lt;&gt;"",LEFT(E84,LEN(LEFT(D84,FIND(" ·",D84&amp;" ·")-1))+1)&lt;&gt;LEFT(D84,FIND(" ·",D84&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I84&lt;&gt;"",IFERROR(OR(I84&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D84,'07 Phases'!$B$9:$B$38,0)),I84&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D84,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C84="","",IF(D84="","⚠ Phase manquante",IF(AND(E84&lt;&gt;"",LEFT(E84,LEN(LEFT(D84,FIND(" ·",D84&amp;" ·")-1))+1)&lt;&gt;LEFT(D84,FIND(" ·",D84&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I84&lt;&gt;"",IFERROR(OR(I84&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D84,'08 Phases'!$B$9:$B$38,0)),I84&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D84,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10533,7 +10533,7 @@
       <c r="I85" s="49" t="n"/>
       <c r="J85" s="49" t="n"/>
       <c r="K85" s="48">
-        <f>IF(C85="","",IF(D85="","⚠ Phase manquante",IF(AND(E85&lt;&gt;"",LEFT(E85,LEN(LEFT(D85,FIND(" ·",D85&amp;" ·")-1))+1)&lt;&gt;LEFT(D85,FIND(" ·",D85&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I85&lt;&gt;"",IFERROR(OR(I85&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D85,'07 Phases'!$B$9:$B$38,0)),I85&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D85,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C85="","",IF(D85="","⚠ Phase manquante",IF(AND(E85&lt;&gt;"",LEFT(E85,LEN(LEFT(D85,FIND(" ·",D85&amp;" ·")-1))+1)&lt;&gt;LEFT(D85,FIND(" ·",D85&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I85&lt;&gt;"",IFERROR(OR(I85&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D85,'08 Phases'!$B$9:$B$38,0)),I85&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D85,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10551,7 +10551,7 @@
       <c r="I86" s="49" t="n"/>
       <c r="J86" s="49" t="n"/>
       <c r="K86" s="48">
-        <f>IF(C86="","",IF(D86="","⚠ Phase manquante",IF(AND(E86&lt;&gt;"",LEFT(E86,LEN(LEFT(D86,FIND(" ·",D86&amp;" ·")-1))+1)&lt;&gt;LEFT(D86,FIND(" ·",D86&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I86&lt;&gt;"",IFERROR(OR(I86&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D86,'07 Phases'!$B$9:$B$38,0)),I86&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D86,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C86="","",IF(D86="","⚠ Phase manquante",IF(AND(E86&lt;&gt;"",LEFT(E86,LEN(LEFT(D86,FIND(" ·",D86&amp;" ·")-1))+1)&lt;&gt;LEFT(D86,FIND(" ·",D86&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I86&lt;&gt;"",IFERROR(OR(I86&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D86,'08 Phases'!$B$9:$B$38,0)),I86&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D86,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10569,7 +10569,7 @@
       <c r="I87" s="49" t="n"/>
       <c r="J87" s="49" t="n"/>
       <c r="K87" s="48">
-        <f>IF(C87="","",IF(D87="","⚠ Phase manquante",IF(AND(E87&lt;&gt;"",LEFT(E87,LEN(LEFT(D87,FIND(" ·",D87&amp;" ·")-1))+1)&lt;&gt;LEFT(D87,FIND(" ·",D87&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I87&lt;&gt;"",IFERROR(OR(I87&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D87,'07 Phases'!$B$9:$B$38,0)),I87&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D87,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C87="","",IF(D87="","⚠ Phase manquante",IF(AND(E87&lt;&gt;"",LEFT(E87,LEN(LEFT(D87,FIND(" ·",D87&amp;" ·")-1))+1)&lt;&gt;LEFT(D87,FIND(" ·",D87&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I87&lt;&gt;"",IFERROR(OR(I87&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D87,'08 Phases'!$B$9:$B$38,0)),I87&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D87,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       <c r="I88" s="49" t="n"/>
       <c r="J88" s="49" t="n"/>
       <c r="K88" s="48">
-        <f>IF(C88="","",IF(D88="","⚠ Phase manquante",IF(AND(E88&lt;&gt;"",LEFT(E88,LEN(LEFT(D88,FIND(" ·",D88&amp;" ·")-1))+1)&lt;&gt;LEFT(D88,FIND(" ·",D88&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I88&lt;&gt;"",IFERROR(OR(I88&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D88,'07 Phases'!$B$9:$B$38,0)),I88&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D88,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C88="","",IF(D88="","⚠ Phase manquante",IF(AND(E88&lt;&gt;"",LEFT(E88,LEN(LEFT(D88,FIND(" ·",D88&amp;" ·")-1))+1)&lt;&gt;LEFT(D88,FIND(" ·",D88&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I88&lt;&gt;"",IFERROR(OR(I88&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D88,'08 Phases'!$B$9:$B$38,0)),I88&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D88,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10605,7 +10605,7 @@
       <c r="I89" s="49" t="n"/>
       <c r="J89" s="49" t="n"/>
       <c r="K89" s="48">
-        <f>IF(C89="","",IF(D89="","⚠ Phase manquante",IF(AND(E89&lt;&gt;"",LEFT(E89,LEN(LEFT(D89,FIND(" ·",D89&amp;" ·")-1))+1)&lt;&gt;LEFT(D89,FIND(" ·",D89&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I89&lt;&gt;"",IFERROR(OR(I89&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D89,'07 Phases'!$B$9:$B$38,0)),I89&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D89,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C89="","",IF(D89="","⚠ Phase manquante",IF(AND(E89&lt;&gt;"",LEFT(E89,LEN(LEFT(D89,FIND(" ·",D89&amp;" ·")-1))+1)&lt;&gt;LEFT(D89,FIND(" ·",D89&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I89&lt;&gt;"",IFERROR(OR(I89&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D89,'08 Phases'!$B$9:$B$38,0)),I89&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D89,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10623,7 +10623,7 @@
       <c r="I90" s="49" t="n"/>
       <c r="J90" s="49" t="n"/>
       <c r="K90" s="48">
-        <f>IF(C90="","",IF(D90="","⚠ Phase manquante",IF(AND(E90&lt;&gt;"",LEFT(E90,LEN(LEFT(D90,FIND(" ·",D90&amp;" ·")-1))+1)&lt;&gt;LEFT(D90,FIND(" ·",D90&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I90&lt;&gt;"",IFERROR(OR(I90&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D90,'07 Phases'!$B$9:$B$38,0)),I90&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D90,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C90="","",IF(D90="","⚠ Phase manquante",IF(AND(E90&lt;&gt;"",LEFT(E90,LEN(LEFT(D90,FIND(" ·",D90&amp;" ·")-1))+1)&lt;&gt;LEFT(D90,FIND(" ·",D90&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I90&lt;&gt;"",IFERROR(OR(I90&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D90,'08 Phases'!$B$9:$B$38,0)),I90&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D90,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10641,7 +10641,7 @@
       <c r="I91" s="49" t="n"/>
       <c r="J91" s="49" t="n"/>
       <c r="K91" s="48">
-        <f>IF(C91="","",IF(D91="","⚠ Phase manquante",IF(AND(E91&lt;&gt;"",LEFT(E91,LEN(LEFT(D91,FIND(" ·",D91&amp;" ·")-1))+1)&lt;&gt;LEFT(D91,FIND(" ·",D91&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I91&lt;&gt;"",IFERROR(OR(I91&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D91,'07 Phases'!$B$9:$B$38,0)),I91&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D91,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C91="","",IF(D91="","⚠ Phase manquante",IF(AND(E91&lt;&gt;"",LEFT(E91,LEN(LEFT(D91,FIND(" ·",D91&amp;" ·")-1))+1)&lt;&gt;LEFT(D91,FIND(" ·",D91&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I91&lt;&gt;"",IFERROR(OR(I91&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D91,'08 Phases'!$B$9:$B$38,0)),I91&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D91,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10659,7 +10659,7 @@
       <c r="I92" s="49" t="n"/>
       <c r="J92" s="49" t="n"/>
       <c r="K92" s="48">
-        <f>IF(C92="","",IF(D92="","⚠ Phase manquante",IF(AND(E92&lt;&gt;"",LEFT(E92,LEN(LEFT(D92,FIND(" ·",D92&amp;" ·")-1))+1)&lt;&gt;LEFT(D92,FIND(" ·",D92&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I92&lt;&gt;"",IFERROR(OR(I92&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D92,'07 Phases'!$B$9:$B$38,0)),I92&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D92,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C92="","",IF(D92="","⚠ Phase manquante",IF(AND(E92&lt;&gt;"",LEFT(E92,LEN(LEFT(D92,FIND(" ·",D92&amp;" ·")-1))+1)&lt;&gt;LEFT(D92,FIND(" ·",D92&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I92&lt;&gt;"",IFERROR(OR(I92&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D92,'08 Phases'!$B$9:$B$38,0)),I92&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D92,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10677,7 +10677,7 @@
       <c r="I93" s="49" t="n"/>
       <c r="J93" s="49" t="n"/>
       <c r="K93" s="48">
-        <f>IF(C93="","",IF(D93="","⚠ Phase manquante",IF(AND(E93&lt;&gt;"",LEFT(E93,LEN(LEFT(D93,FIND(" ·",D93&amp;" ·")-1))+1)&lt;&gt;LEFT(D93,FIND(" ·",D93&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I93&lt;&gt;"",IFERROR(OR(I93&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D93,'07 Phases'!$B$9:$B$38,0)),I93&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D93,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C93="","",IF(D93="","⚠ Phase manquante",IF(AND(E93&lt;&gt;"",LEFT(E93,LEN(LEFT(D93,FIND(" ·",D93&amp;" ·")-1))+1)&lt;&gt;LEFT(D93,FIND(" ·",D93&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I93&lt;&gt;"",IFERROR(OR(I93&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D93,'08 Phases'!$B$9:$B$38,0)),I93&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D93,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10695,7 +10695,7 @@
       <c r="I94" s="49" t="n"/>
       <c r="J94" s="49" t="n"/>
       <c r="K94" s="48">
-        <f>IF(C94="","",IF(D94="","⚠ Phase manquante",IF(AND(E94&lt;&gt;"",LEFT(E94,LEN(LEFT(D94,FIND(" ·",D94&amp;" ·")-1))+1)&lt;&gt;LEFT(D94,FIND(" ·",D94&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I94&lt;&gt;"",IFERROR(OR(I94&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D94,'07 Phases'!$B$9:$B$38,0)),I94&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D94,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C94="","",IF(D94="","⚠ Phase manquante",IF(AND(E94&lt;&gt;"",LEFT(E94,LEN(LEFT(D94,FIND(" ·",D94&amp;" ·")-1))+1)&lt;&gt;LEFT(D94,FIND(" ·",D94&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I94&lt;&gt;"",IFERROR(OR(I94&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D94,'08 Phases'!$B$9:$B$38,0)),I94&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D94,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10713,7 +10713,7 @@
       <c r="I95" s="49" t="n"/>
       <c r="J95" s="49" t="n"/>
       <c r="K95" s="48">
-        <f>IF(C95="","",IF(D95="","⚠ Phase manquante",IF(AND(E95&lt;&gt;"",LEFT(E95,LEN(LEFT(D95,FIND(" ·",D95&amp;" ·")-1))+1)&lt;&gt;LEFT(D95,FIND(" ·",D95&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I95&lt;&gt;"",IFERROR(OR(I95&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D95,'07 Phases'!$B$9:$B$38,0)),I95&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D95,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C95="","",IF(D95="","⚠ Phase manquante",IF(AND(E95&lt;&gt;"",LEFT(E95,LEN(LEFT(D95,FIND(" ·",D95&amp;" ·")-1))+1)&lt;&gt;LEFT(D95,FIND(" ·",D95&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I95&lt;&gt;"",IFERROR(OR(I95&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D95,'08 Phases'!$B$9:$B$38,0)),I95&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D95,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10731,7 +10731,7 @@
       <c r="I96" s="49" t="n"/>
       <c r="J96" s="49" t="n"/>
       <c r="K96" s="48">
-        <f>IF(C96="","",IF(D96="","⚠ Phase manquante",IF(AND(E96&lt;&gt;"",LEFT(E96,LEN(LEFT(D96,FIND(" ·",D96&amp;" ·")-1))+1)&lt;&gt;LEFT(D96,FIND(" ·",D96&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I96&lt;&gt;"",IFERROR(OR(I96&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D96,'07 Phases'!$B$9:$B$38,0)),I96&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D96,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C96="","",IF(D96="","⚠ Phase manquante",IF(AND(E96&lt;&gt;"",LEFT(E96,LEN(LEFT(D96,FIND(" ·",D96&amp;" ·")-1))+1)&lt;&gt;LEFT(D96,FIND(" ·",D96&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I96&lt;&gt;"",IFERROR(OR(I96&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D96,'08 Phases'!$B$9:$B$38,0)),I96&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D96,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10749,7 +10749,7 @@
       <c r="I97" s="49" t="n"/>
       <c r="J97" s="49" t="n"/>
       <c r="K97" s="48">
-        <f>IF(C97="","",IF(D97="","⚠ Phase manquante",IF(AND(E97&lt;&gt;"",LEFT(E97,LEN(LEFT(D97,FIND(" ·",D97&amp;" ·")-1))+1)&lt;&gt;LEFT(D97,FIND(" ·",D97&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I97&lt;&gt;"",IFERROR(OR(I97&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D97,'07 Phases'!$B$9:$B$38,0)),I97&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D97,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C97="","",IF(D97="","⚠ Phase manquante",IF(AND(E97&lt;&gt;"",LEFT(E97,LEN(LEFT(D97,FIND(" ·",D97&amp;" ·")-1))+1)&lt;&gt;LEFT(D97,FIND(" ·",D97&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I97&lt;&gt;"",IFERROR(OR(I97&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D97,'08 Phases'!$B$9:$B$38,0)),I97&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D97,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10767,7 +10767,7 @@
       <c r="I98" s="49" t="n"/>
       <c r="J98" s="49" t="n"/>
       <c r="K98" s="48">
-        <f>IF(C98="","",IF(D98="","⚠ Phase manquante",IF(AND(E98&lt;&gt;"",LEFT(E98,LEN(LEFT(D98,FIND(" ·",D98&amp;" ·")-1))+1)&lt;&gt;LEFT(D98,FIND(" ·",D98&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I98&lt;&gt;"",IFERROR(OR(I98&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D98,'07 Phases'!$B$9:$B$38,0)),I98&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D98,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C98="","",IF(D98="","⚠ Phase manquante",IF(AND(E98&lt;&gt;"",LEFT(E98,LEN(LEFT(D98,FIND(" ·",D98&amp;" ·")-1))+1)&lt;&gt;LEFT(D98,FIND(" ·",D98&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I98&lt;&gt;"",IFERROR(OR(I98&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D98,'08 Phases'!$B$9:$B$38,0)),I98&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D98,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10785,7 +10785,7 @@
       <c r="I99" s="49" t="n"/>
       <c r="J99" s="49" t="n"/>
       <c r="K99" s="48">
-        <f>IF(C99="","",IF(D99="","⚠ Phase manquante",IF(AND(E99&lt;&gt;"",LEFT(E99,LEN(LEFT(D99,FIND(" ·",D99&amp;" ·")-1))+1)&lt;&gt;LEFT(D99,FIND(" ·",D99&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I99&lt;&gt;"",IFERROR(OR(I99&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D99,'07 Phases'!$B$9:$B$38,0)),I99&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D99,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C99="","",IF(D99="","⚠ Phase manquante",IF(AND(E99&lt;&gt;"",LEFT(E99,LEN(LEFT(D99,FIND(" ·",D99&amp;" ·")-1))+1)&lt;&gt;LEFT(D99,FIND(" ·",D99&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I99&lt;&gt;"",IFERROR(OR(I99&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D99,'08 Phases'!$B$9:$B$38,0)),I99&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D99,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
       <c r="I100" s="49" t="n"/>
       <c r="J100" s="49" t="n"/>
       <c r="K100" s="48">
-        <f>IF(C100="","",IF(D100="","⚠ Phase manquante",IF(AND(E100&lt;&gt;"",LEFT(E100,LEN(LEFT(D100,FIND(" ·",D100&amp;" ·")-1))+1)&lt;&gt;LEFT(D100,FIND(" ·",D100&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I100&lt;&gt;"",IFERROR(OR(I100&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D100,'07 Phases'!$B$9:$B$38,0)),I100&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D100,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C100="","",IF(D100="","⚠ Phase manquante",IF(AND(E100&lt;&gt;"",LEFT(E100,LEN(LEFT(D100,FIND(" ·",D100&amp;" ·")-1))+1)&lt;&gt;LEFT(D100,FIND(" ·",D100&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I100&lt;&gt;"",IFERROR(OR(I100&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D100,'08 Phases'!$B$9:$B$38,0)),I100&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D100,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       <c r="I101" s="49" t="n"/>
       <c r="J101" s="49" t="n"/>
       <c r="K101" s="48">
-        <f>IF(C101="","",IF(D101="","⚠ Phase manquante",IF(AND(E101&lt;&gt;"",LEFT(E101,LEN(LEFT(D101,FIND(" ·",D101&amp;" ·")-1))+1)&lt;&gt;LEFT(D101,FIND(" ·",D101&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I101&lt;&gt;"",IFERROR(OR(I101&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D101,'07 Phases'!$B$9:$B$38,0)),I101&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D101,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C101="","",IF(D101="","⚠ Phase manquante",IF(AND(E101&lt;&gt;"",LEFT(E101,LEN(LEFT(D101,FIND(" ·",D101&amp;" ·")-1))+1)&lt;&gt;LEFT(D101,FIND(" ·",D101&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I101&lt;&gt;"",IFERROR(OR(I101&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D101,'08 Phases'!$B$9:$B$38,0)),I101&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D101,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10839,7 +10839,7 @@
       <c r="I102" s="49" t="n"/>
       <c r="J102" s="49" t="n"/>
       <c r="K102" s="48">
-        <f>IF(C102="","",IF(D102="","⚠ Phase manquante",IF(AND(E102&lt;&gt;"",LEFT(E102,LEN(LEFT(D102,FIND(" ·",D102&amp;" ·")-1))+1)&lt;&gt;LEFT(D102,FIND(" ·",D102&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I102&lt;&gt;"",IFERROR(OR(I102&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D102,'07 Phases'!$B$9:$B$38,0)),I102&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D102,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C102="","",IF(D102="","⚠ Phase manquante",IF(AND(E102&lt;&gt;"",LEFT(E102,LEN(LEFT(D102,FIND(" ·",D102&amp;" ·")-1))+1)&lt;&gt;LEFT(D102,FIND(" ·",D102&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I102&lt;&gt;"",IFERROR(OR(I102&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D102,'08 Phases'!$B$9:$B$38,0)),I102&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D102,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10857,7 +10857,7 @@
       <c r="I103" s="49" t="n"/>
       <c r="J103" s="49" t="n"/>
       <c r="K103" s="48">
-        <f>IF(C103="","",IF(D103="","⚠ Phase manquante",IF(AND(E103&lt;&gt;"",LEFT(E103,LEN(LEFT(D103,FIND(" ·",D103&amp;" ·")-1))+1)&lt;&gt;LEFT(D103,FIND(" ·",D103&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I103&lt;&gt;"",IFERROR(OR(I103&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D103,'07 Phases'!$B$9:$B$38,0)),I103&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D103,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C103="","",IF(D103="","⚠ Phase manquante",IF(AND(E103&lt;&gt;"",LEFT(E103,LEN(LEFT(D103,FIND(" ·",D103&amp;" ·")-1))+1)&lt;&gt;LEFT(D103,FIND(" ·",D103&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I103&lt;&gt;"",IFERROR(OR(I103&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D103,'08 Phases'!$B$9:$B$38,0)),I103&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D103,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
       <c r="I104" s="49" t="n"/>
       <c r="J104" s="49" t="n"/>
       <c r="K104" s="48">
-        <f>IF(C104="","",IF(D104="","⚠ Phase manquante",IF(AND(E104&lt;&gt;"",LEFT(E104,LEN(LEFT(D104,FIND(" ·",D104&amp;" ·")-1))+1)&lt;&gt;LEFT(D104,FIND(" ·",D104&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I104&lt;&gt;"",IFERROR(OR(I104&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D104,'07 Phases'!$B$9:$B$38,0)),I104&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D104,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C104="","",IF(D104="","⚠ Phase manquante",IF(AND(E104&lt;&gt;"",LEFT(E104,LEN(LEFT(D104,FIND(" ·",D104&amp;" ·")-1))+1)&lt;&gt;LEFT(D104,FIND(" ·",D104&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I104&lt;&gt;"",IFERROR(OR(I104&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D104,'08 Phases'!$B$9:$B$38,0)),I104&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D104,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10893,7 +10893,7 @@
       <c r="I105" s="49" t="n"/>
       <c r="J105" s="49" t="n"/>
       <c r="K105" s="48">
-        <f>IF(C105="","",IF(D105="","⚠ Phase manquante",IF(AND(E105&lt;&gt;"",LEFT(E105,LEN(LEFT(D105,FIND(" ·",D105&amp;" ·")-1))+1)&lt;&gt;LEFT(D105,FIND(" ·",D105&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I105&lt;&gt;"",IFERROR(OR(I105&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D105,'07 Phases'!$B$9:$B$38,0)),I105&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D105,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C105="","",IF(D105="","⚠ Phase manquante",IF(AND(E105&lt;&gt;"",LEFT(E105,LEN(LEFT(D105,FIND(" ·",D105&amp;" ·")-1))+1)&lt;&gt;LEFT(D105,FIND(" ·",D105&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I105&lt;&gt;"",IFERROR(OR(I105&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D105,'08 Phases'!$B$9:$B$38,0)),I105&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D105,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10911,7 +10911,7 @@
       <c r="I106" s="49" t="n"/>
       <c r="J106" s="49" t="n"/>
       <c r="K106" s="48">
-        <f>IF(C106="","",IF(D106="","⚠ Phase manquante",IF(AND(E106&lt;&gt;"",LEFT(E106,LEN(LEFT(D106,FIND(" ·",D106&amp;" ·")-1))+1)&lt;&gt;LEFT(D106,FIND(" ·",D106&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I106&lt;&gt;"",IFERROR(OR(I106&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D106,'07 Phases'!$B$9:$B$38,0)),I106&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D106,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C106="","",IF(D106="","⚠ Phase manquante",IF(AND(E106&lt;&gt;"",LEFT(E106,LEN(LEFT(D106,FIND(" ·",D106&amp;" ·")-1))+1)&lt;&gt;LEFT(D106,FIND(" ·",D106&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I106&lt;&gt;"",IFERROR(OR(I106&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D106,'08 Phases'!$B$9:$B$38,0)),I106&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D106,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       <c r="I107" s="49" t="n"/>
       <c r="J107" s="49" t="n"/>
       <c r="K107" s="48">
-        <f>IF(C107="","",IF(D107="","⚠ Phase manquante",IF(AND(E107&lt;&gt;"",LEFT(E107,LEN(LEFT(D107,FIND(" ·",D107&amp;" ·")-1))+1)&lt;&gt;LEFT(D107,FIND(" ·",D107&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I107&lt;&gt;"",IFERROR(OR(I107&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D107,'07 Phases'!$B$9:$B$38,0)),I107&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D107,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C107="","",IF(D107="","⚠ Phase manquante",IF(AND(E107&lt;&gt;"",LEFT(E107,LEN(LEFT(D107,FIND(" ·",D107&amp;" ·")-1))+1)&lt;&gt;LEFT(D107,FIND(" ·",D107&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I107&lt;&gt;"",IFERROR(OR(I107&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D107,'08 Phases'!$B$9:$B$38,0)),I107&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D107,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10947,7 +10947,7 @@
       <c r="I108" s="49" t="n"/>
       <c r="J108" s="49" t="n"/>
       <c r="K108" s="48">
-        <f>IF(C108="","",IF(D108="","⚠ Phase manquante",IF(AND(E108&lt;&gt;"",LEFT(E108,LEN(LEFT(D108,FIND(" ·",D108&amp;" ·")-1))+1)&lt;&gt;LEFT(D108,FIND(" ·",D108&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I108&lt;&gt;"",IFERROR(OR(I108&lt;INDEX('07 Phases'!$F$9:$F$38,MATCH(D108,'07 Phases'!$B$9:$B$38,0)),I108&gt;INDEX('07 Phases'!$G$9:$G$38,MATCH(D108,'07 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
+        <f>IF(C108="","",IF(D108="","⚠ Phase manquante",IF(AND(E108&lt;&gt;"",LEFT(E108,LEN(LEFT(D108,FIND(" ·",D108&amp;" ·")-1))+1)&lt;&gt;LEFT(D108,FIND(" ·",D108&amp;" ·")-1)&amp;"."),"⚠ Sous-phase hors phase",IF(AND(I108&lt;&gt;"",IFERROR(OR(I108&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(D108,'08 Phases'!$B$9:$B$38,0)),I108&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(D108,'08 Phases'!$B$9:$B$38,0))),FALSE)),"◔ Date hors période de la phase","✓"))))</f>
         <v/>
       </c>
     </row>
@@ -10988,7 +10988,7 @@
       <formula1>L_SousPhases</formula1>
     </dataValidation>
     <dataValidation sqref="E9:E108" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur hors liste" error="Choisissez une sous-phase de la phase de la colonne Phase (onglet 08 Sous-phases)." type="list" errorStyle="stop">
-      <formula1>IF($D9="",L_SousPhases,OFFSET('08 Sous-phases'!$B$9,IFERROR(MATCH(LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*",'08 Sous-phases'!$B$9:$B$88,0)-1,0),0,MAX(1,COUNTIF('08 Sous-phases'!$B$9:$B$88,LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*"))))</formula1>
+      <formula1>IF($D9="",L_SousPhases,OFFSET('09 Sous-phases'!$B$9,IFERROR(MATCH(LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*",'09 Sous-phases'!$B$9:$B$88,0)-1,0),0,MAX(1,COUNTIF('09 Sous-phases'!$B$9:$B$88,LEFT($D9,FIND(" ·",$D9&amp;" ·")-1)&amp;".*"))))</formula1>
     </dataValidation>
     <dataValidation sqref="F10:F108" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste. Elle se remplit à partir de l’onglet correspondant." type="list" errorStyle="stop">
       <formula1>L_Chantiers</formula1>
@@ -11016,7 +11016,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="K3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -11030,7 +11030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H158"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -11084,7 +11084,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 13    </t>
+            <t xml:space="preserve">Étape 14    </t>
           </r>
           <r>
             <rPr>
@@ -13037,7 +13037,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="H3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -13434,7 +13434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -13460,6 +13460,7 @@
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
+    <row r="5"/>
     <row r="6" ht="24" customHeight="1">
       <c r="B6" s="29" t="inlineStr">
         <is>
@@ -13624,7 +13625,7 @@
       </c>
       <c r="E14" s="34" t="inlineStr">
         <is>
-          <t>06 Lots</t>
+          <t>07 Lots</t>
         </is>
       </c>
     </row>
@@ -13646,7 +13647,7 @@
       </c>
       <c r="E15" s="34" t="inlineStr">
         <is>
-          <t>07 Phases</t>
+          <t>08 Phases</t>
         </is>
       </c>
     </row>
@@ -13668,7 +13669,7 @@
       </c>
       <c r="E16" s="34" t="inlineStr">
         <is>
-          <t>08 Sous-phases</t>
+          <t>09 Sous-phases</t>
         </is>
       </c>
     </row>
@@ -13690,7 +13691,7 @@
       </c>
       <c r="E17" s="34" t="inlineStr">
         <is>
-          <t>09 Chantiers</t>
+          <t>10 Chantiers</t>
         </is>
       </c>
     </row>
@@ -13719,7 +13720,7 @@
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>10 Instances</t>
+          <t>11 Instances</t>
         </is>
       </c>
     </row>
@@ -13741,7 +13742,7 @@
       </c>
       <c r="E20" s="34" t="inlineStr">
         <is>
-          <t>10 Instances</t>
+          <t>11 Instances</t>
         </is>
       </c>
     </row>
@@ -13763,7 +13764,7 @@
       </c>
       <c r="E21" s="34" t="inlineStr">
         <is>
-          <t>11 Membres</t>
+          <t>12 Membres</t>
         </is>
       </c>
     </row>
@@ -13792,7 +13793,7 @@
       </c>
       <c r="E23" s="34" t="inlineStr">
         <is>
-          <t>12 Jalons</t>
+          <t>13 Jalons</t>
         </is>
       </c>
     </row>
@@ -13814,7 +13815,7 @@
       </c>
       <c r="E24" s="34" t="inlineStr">
         <is>
-          <t>12 Jalons</t>
+          <t>13 Jalons</t>
         </is>
       </c>
     </row>
@@ -13836,7 +13837,7 @@
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>12 Jalons</t>
+          <t>13 Jalons</t>
         </is>
       </c>
     </row>
@@ -13858,7 +13859,7 @@
       </c>
       <c r="E26" s="34" t="inlineStr">
         <is>
-          <t>13 Livrables</t>
+          <t>14 Livrables</t>
         </is>
       </c>
     </row>
@@ -13887,7 +13888,7 @@
       </c>
       <c r="E28" s="34" t="inlineStr">
         <is>
-          <t>07 Phases</t>
+          <t>08 Phases</t>
         </is>
       </c>
     </row>
@@ -13909,7 +13910,7 @@
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
-          <t>12 Jalons</t>
+          <t>13 Jalons</t>
         </is>
       </c>
     </row>
@@ -13931,7 +13932,7 @@
       </c>
       <c r="E30" s="34" t="inlineStr">
         <is>
-          <t>12 Jalons</t>
+          <t>13 Jalons</t>
         </is>
       </c>
     </row>
@@ -13959,26 +13960,26 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" location="#'01 Équipes'!A1" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" location="#'02 Rôles'!A1" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" location="#'03 Personnes'!A1" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" location="#'04 Affectations'!A1" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" location="#'Complétude'!A1" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" location="#'06 Lots'!A1" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" location="#'07 Phases'!A1" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" location="#'08 Sous-phases'!A1" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" location="#'09 Chantiers'!A1" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" location="#'10 Instances'!A1" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" location="#'10 Instances'!A1" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" location="#'11 Membres'!A1" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" location="#'12 Jalons'!A1" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" location="#'12 Jalons'!A1" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" location="#'12 Jalons'!A1" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" location="#'13 Livrables'!A1" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" location="#'07 Phases'!A1" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" location="#'12 Jalons'!A1" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" location="#'12 Jalons'!A1" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" location="#'Complétude'!A1" r:id="rId20"/>
+    <hyperlink ref="E8" location="#'01 Équipes'!A1"/>
+    <hyperlink ref="E9" location="#'02 Rôles'!A1"/>
+    <hyperlink ref="E10" location="#'03 Personnes'!A1"/>
+    <hyperlink ref="E11" location="#'04 Affectations'!A1"/>
+    <hyperlink ref="E13" location="#'Complétude'!A1"/>
+    <hyperlink ref="E14" location="#'07 Lots'!A1"/>
+    <hyperlink ref="E15" location="#'08 Phases'!A1"/>
+    <hyperlink ref="E16" location="#'09 Sous-phases'!A1"/>
+    <hyperlink ref="E17" location="#'10 Chantiers'!A1"/>
+    <hyperlink ref="E19" location="#'11 Instances'!A1"/>
+    <hyperlink ref="E20" location="#'11 Instances'!A1"/>
+    <hyperlink ref="E21" location="#'12 Membres'!A1"/>
+    <hyperlink ref="E23" location="#'13 Jalons'!A1"/>
+    <hyperlink ref="E24" location="#'13 Jalons'!A1"/>
+    <hyperlink ref="E25" location="#'13 Jalons'!A1"/>
+    <hyperlink ref="E26" location="#'14 Livrables'!A1"/>
+    <hyperlink ref="E28" location="#'08 Phases'!A1"/>
+    <hyperlink ref="E29" location="#'13 Jalons'!A1"/>
+    <hyperlink ref="E30" location="#'13 Jalons'!A1"/>
+    <hyperlink ref="E31" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -13991,7 +13992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E102"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -14004,6 +14005,7 @@
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -14018,6 +14020,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
@@ -14043,10 +14046,11 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Colonnes concernées (09 Chantiers) : Phases (N° ou nom), Sous-phases (N°, ex. 3.1, dans une phase du chantier), Dépendances (noms ou codes des chantiers, ou Tous seul).</t>
-        </is>
-      </c>
-    </row>
+          <t>Colonnes concernées (10 Chantiers) : Phases (N° ou nom), Sous-phases (N°, ex. 3.1, dans une phase du chantier), Dépendances (noms ou codes des chantiers, ou Tous seul).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
@@ -14057,7 +14061,7 @@
               <color rgb="FF1D8F86"/>
               <sz val="8"/>
             </rPr>
-            <t>RUBRIQUES DE INFO PROJET  (onglet 05b)</t>
+            <t>RUBRIQUES DE INFO PROJET  (onglet 06)</t>
           </r>
         </is>
       </c>
@@ -14260,6 +14264,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
@@ -14294,428 +14300,428 @@
     </row>
     <row r="23">
       <c r="B23" s="47">
-        <f>IF('07 Phases'!$B$9="","",'07 Phases'!$B$9)</f>
+        <f>IF('08 Phases'!$B$9="","",'08 Phases'!$B$9)</f>
         <v/>
       </c>
       <c r="C23" s="47">
-        <f>IF('08 Sous-phases'!$B$9="","",'08 Sous-phases'!$B$9)</f>
+        <f>IF('09 Sous-phases'!$B$9="","",'09 Sous-phases'!$B$9)</f>
         <v/>
       </c>
       <c r="D23" s="47">
-        <f>IF('09 Chantiers'!$C$9="","",'09 Chantiers'!$B$9&amp;" · "&amp;'09 Chantiers'!$C$9)</f>
+        <f>IF('10 Chantiers'!$C$9="","",'10 Chantiers'!$B$9&amp;" · "&amp;'10 Chantiers'!$C$9)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="47">
-        <f>IF('07 Phases'!$B$10="","",'07 Phases'!$B$10)</f>
+        <f>IF('08 Phases'!$B$10="","",'08 Phases'!$B$10)</f>
         <v/>
       </c>
       <c r="C24" s="47">
-        <f>IF('08 Sous-phases'!$B$10="","",'08 Sous-phases'!$B$10)</f>
+        <f>IF('09 Sous-phases'!$B$10="","",'09 Sous-phases'!$B$10)</f>
         <v/>
       </c>
       <c r="D24" s="47">
-        <f>IF('09 Chantiers'!$C$10="","",'09 Chantiers'!$B$10&amp;" · "&amp;'09 Chantiers'!$C$10)</f>
+        <f>IF('10 Chantiers'!$C$10="","",'10 Chantiers'!$B$10&amp;" · "&amp;'10 Chantiers'!$C$10)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="47">
-        <f>IF('07 Phases'!$B$11="","",'07 Phases'!$B$11)</f>
+        <f>IF('08 Phases'!$B$11="","",'08 Phases'!$B$11)</f>
         <v/>
       </c>
       <c r="C25" s="47">
-        <f>IF('08 Sous-phases'!$B$11="","",'08 Sous-phases'!$B$11)</f>
+        <f>IF('09 Sous-phases'!$B$11="","",'09 Sous-phases'!$B$11)</f>
         <v/>
       </c>
       <c r="D25" s="47">
-        <f>IF('09 Chantiers'!$C$11="","",'09 Chantiers'!$B$11&amp;" · "&amp;'09 Chantiers'!$C$11)</f>
+        <f>IF('10 Chantiers'!$C$11="","",'10 Chantiers'!$B$11&amp;" · "&amp;'10 Chantiers'!$C$11)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="47">
-        <f>IF('07 Phases'!$B$12="","",'07 Phases'!$B$12)</f>
+        <f>IF('08 Phases'!$B$12="","",'08 Phases'!$B$12)</f>
         <v/>
       </c>
       <c r="C26" s="47">
-        <f>IF('08 Sous-phases'!$B$12="","",'08 Sous-phases'!$B$12)</f>
+        <f>IF('09 Sous-phases'!$B$12="","",'09 Sous-phases'!$B$12)</f>
         <v/>
       </c>
       <c r="D26" s="47">
-        <f>IF('09 Chantiers'!$C$12="","",'09 Chantiers'!$B$12&amp;" · "&amp;'09 Chantiers'!$C$12)</f>
+        <f>IF('10 Chantiers'!$C$12="","",'10 Chantiers'!$B$12&amp;" · "&amp;'10 Chantiers'!$C$12)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="47">
-        <f>IF('07 Phases'!$B$13="","",'07 Phases'!$B$13)</f>
+        <f>IF('08 Phases'!$B$13="","",'08 Phases'!$B$13)</f>
         <v/>
       </c>
       <c r="C27" s="47">
-        <f>IF('08 Sous-phases'!$B$13="","",'08 Sous-phases'!$B$13)</f>
+        <f>IF('09 Sous-phases'!$B$13="","",'09 Sous-phases'!$B$13)</f>
         <v/>
       </c>
       <c r="D27" s="47">
-        <f>IF('09 Chantiers'!$C$13="","",'09 Chantiers'!$B$13&amp;" · "&amp;'09 Chantiers'!$C$13)</f>
+        <f>IF('10 Chantiers'!$C$13="","",'10 Chantiers'!$B$13&amp;" · "&amp;'10 Chantiers'!$C$13)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="47">
-        <f>IF('07 Phases'!$B$14="","",'07 Phases'!$B$14)</f>
+        <f>IF('08 Phases'!$B$14="","",'08 Phases'!$B$14)</f>
         <v/>
       </c>
       <c r="C28" s="47">
-        <f>IF('08 Sous-phases'!$B$14="","",'08 Sous-phases'!$B$14)</f>
+        <f>IF('09 Sous-phases'!$B$14="","",'09 Sous-phases'!$B$14)</f>
         <v/>
       </c>
       <c r="D28" s="47">
-        <f>IF('09 Chantiers'!$C$14="","",'09 Chantiers'!$B$14&amp;" · "&amp;'09 Chantiers'!$C$14)</f>
+        <f>IF('10 Chantiers'!$C$14="","",'10 Chantiers'!$B$14&amp;" · "&amp;'10 Chantiers'!$C$14)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="47">
-        <f>IF('07 Phases'!$B$15="","",'07 Phases'!$B$15)</f>
+        <f>IF('08 Phases'!$B$15="","",'08 Phases'!$B$15)</f>
         <v/>
       </c>
       <c r="C29" s="47">
-        <f>IF('08 Sous-phases'!$B$15="","",'08 Sous-phases'!$B$15)</f>
+        <f>IF('09 Sous-phases'!$B$15="","",'09 Sous-phases'!$B$15)</f>
         <v/>
       </c>
       <c r="D29" s="47">
-        <f>IF('09 Chantiers'!$C$15="","",'09 Chantiers'!$B$15&amp;" · "&amp;'09 Chantiers'!$C$15)</f>
+        <f>IF('10 Chantiers'!$C$15="","",'10 Chantiers'!$B$15&amp;" · "&amp;'10 Chantiers'!$C$15)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="47">
-        <f>IF('07 Phases'!$B$16="","",'07 Phases'!$B$16)</f>
+        <f>IF('08 Phases'!$B$16="","",'08 Phases'!$B$16)</f>
         <v/>
       </c>
       <c r="C30" s="47">
-        <f>IF('08 Sous-phases'!$B$16="","",'08 Sous-phases'!$B$16)</f>
+        <f>IF('09 Sous-phases'!$B$16="","",'09 Sous-phases'!$B$16)</f>
         <v/>
       </c>
       <c r="D30" s="47">
-        <f>IF('09 Chantiers'!$C$16="","",'09 Chantiers'!$B$16&amp;" · "&amp;'09 Chantiers'!$C$16)</f>
+        <f>IF('10 Chantiers'!$C$16="","",'10 Chantiers'!$B$16&amp;" · "&amp;'10 Chantiers'!$C$16)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="47">
-        <f>IF('07 Phases'!$B$17="","",'07 Phases'!$B$17)</f>
+        <f>IF('08 Phases'!$B$17="","",'08 Phases'!$B$17)</f>
         <v/>
       </c>
       <c r="C31" s="47">
-        <f>IF('08 Sous-phases'!$B$17="","",'08 Sous-phases'!$B$17)</f>
+        <f>IF('09 Sous-phases'!$B$17="","",'09 Sous-phases'!$B$17)</f>
         <v/>
       </c>
       <c r="D31" s="47">
-        <f>IF('09 Chantiers'!$C$17="","",'09 Chantiers'!$B$17&amp;" · "&amp;'09 Chantiers'!$C$17)</f>
+        <f>IF('10 Chantiers'!$C$17="","",'10 Chantiers'!$B$17&amp;" · "&amp;'10 Chantiers'!$C$17)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="47">
-        <f>IF('07 Phases'!$B$18="","",'07 Phases'!$B$18)</f>
+        <f>IF('08 Phases'!$B$18="","",'08 Phases'!$B$18)</f>
         <v/>
       </c>
       <c r="C32" s="47">
-        <f>IF('08 Sous-phases'!$B$18="","",'08 Sous-phases'!$B$18)</f>
+        <f>IF('09 Sous-phases'!$B$18="","",'09 Sous-phases'!$B$18)</f>
         <v/>
       </c>
       <c r="D32" s="47">
-        <f>IF('09 Chantiers'!$C$18="","",'09 Chantiers'!$B$18&amp;" · "&amp;'09 Chantiers'!$C$18)</f>
+        <f>IF('10 Chantiers'!$C$18="","",'10 Chantiers'!$B$18&amp;" · "&amp;'10 Chantiers'!$C$18)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="47">
-        <f>IF('07 Phases'!$B$19="","",'07 Phases'!$B$19)</f>
+        <f>IF('08 Phases'!$B$19="","",'08 Phases'!$B$19)</f>
         <v/>
       </c>
       <c r="C33" s="47">
-        <f>IF('08 Sous-phases'!$B$19="","",'08 Sous-phases'!$B$19)</f>
+        <f>IF('09 Sous-phases'!$B$19="","",'09 Sous-phases'!$B$19)</f>
         <v/>
       </c>
       <c r="D33" s="47">
-        <f>IF('09 Chantiers'!$C$19="","",'09 Chantiers'!$B$19&amp;" · "&amp;'09 Chantiers'!$C$19)</f>
+        <f>IF('10 Chantiers'!$C$19="","",'10 Chantiers'!$B$19&amp;" · "&amp;'10 Chantiers'!$C$19)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="47">
-        <f>IF('07 Phases'!$B$20="","",'07 Phases'!$B$20)</f>
+        <f>IF('08 Phases'!$B$20="","",'08 Phases'!$B$20)</f>
         <v/>
       </c>
       <c r="C34" s="47">
-        <f>IF('08 Sous-phases'!$B$20="","",'08 Sous-phases'!$B$20)</f>
+        <f>IF('09 Sous-phases'!$B$20="","",'09 Sous-phases'!$B$20)</f>
         <v/>
       </c>
       <c r="D34" s="47">
-        <f>IF('09 Chantiers'!$C$20="","",'09 Chantiers'!$B$20&amp;" · "&amp;'09 Chantiers'!$C$20)</f>
+        <f>IF('10 Chantiers'!$C$20="","",'10 Chantiers'!$B$20&amp;" · "&amp;'10 Chantiers'!$C$20)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="47">
-        <f>IF('07 Phases'!$B$21="","",'07 Phases'!$B$21)</f>
+        <f>IF('08 Phases'!$B$21="","",'08 Phases'!$B$21)</f>
         <v/>
       </c>
       <c r="C35" s="47">
-        <f>IF('08 Sous-phases'!$B$21="","",'08 Sous-phases'!$B$21)</f>
+        <f>IF('09 Sous-phases'!$B$21="","",'09 Sous-phases'!$B$21)</f>
         <v/>
       </c>
       <c r="D35" s="47">
-        <f>IF('09 Chantiers'!$C$21="","",'09 Chantiers'!$B$21&amp;" · "&amp;'09 Chantiers'!$C$21)</f>
+        <f>IF('10 Chantiers'!$C$21="","",'10 Chantiers'!$B$21&amp;" · "&amp;'10 Chantiers'!$C$21)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="47">
-        <f>IF('07 Phases'!$B$22="","",'07 Phases'!$B$22)</f>
+        <f>IF('08 Phases'!$B$22="","",'08 Phases'!$B$22)</f>
         <v/>
       </c>
       <c r="C36" s="47">
-        <f>IF('08 Sous-phases'!$B$22="","",'08 Sous-phases'!$B$22)</f>
+        <f>IF('09 Sous-phases'!$B$22="","",'09 Sous-phases'!$B$22)</f>
         <v/>
       </c>
       <c r="D36" s="47">
-        <f>IF('09 Chantiers'!$C$22="","",'09 Chantiers'!$B$22&amp;" · "&amp;'09 Chantiers'!$C$22)</f>
+        <f>IF('10 Chantiers'!$C$22="","",'10 Chantiers'!$B$22&amp;" · "&amp;'10 Chantiers'!$C$22)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="47">
-        <f>IF('07 Phases'!$B$23="","",'07 Phases'!$B$23)</f>
+        <f>IF('08 Phases'!$B$23="","",'08 Phases'!$B$23)</f>
         <v/>
       </c>
       <c r="C37" s="47">
-        <f>IF('08 Sous-phases'!$B$23="","",'08 Sous-phases'!$B$23)</f>
+        <f>IF('09 Sous-phases'!$B$23="","",'09 Sous-phases'!$B$23)</f>
         <v/>
       </c>
       <c r="D37" s="47">
-        <f>IF('09 Chantiers'!$C$23="","",'09 Chantiers'!$B$23&amp;" · "&amp;'09 Chantiers'!$C$23)</f>
+        <f>IF('10 Chantiers'!$C$23="","",'10 Chantiers'!$B$23&amp;" · "&amp;'10 Chantiers'!$C$23)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="47">
-        <f>IF('07 Phases'!$B$24="","",'07 Phases'!$B$24)</f>
+        <f>IF('08 Phases'!$B$24="","",'08 Phases'!$B$24)</f>
         <v/>
       </c>
       <c r="C38" s="47">
-        <f>IF('08 Sous-phases'!$B$24="","",'08 Sous-phases'!$B$24)</f>
+        <f>IF('09 Sous-phases'!$B$24="","",'09 Sous-phases'!$B$24)</f>
         <v/>
       </c>
       <c r="D38" s="47">
-        <f>IF('09 Chantiers'!$C$24="","",'09 Chantiers'!$B$24&amp;" · "&amp;'09 Chantiers'!$C$24)</f>
+        <f>IF('10 Chantiers'!$C$24="","",'10 Chantiers'!$B$24&amp;" · "&amp;'10 Chantiers'!$C$24)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="47">
-        <f>IF('07 Phases'!$B$25="","",'07 Phases'!$B$25)</f>
+        <f>IF('08 Phases'!$B$25="","",'08 Phases'!$B$25)</f>
         <v/>
       </c>
       <c r="C39" s="47">
-        <f>IF('08 Sous-phases'!$B$25="","",'08 Sous-phases'!$B$25)</f>
+        <f>IF('09 Sous-phases'!$B$25="","",'09 Sous-phases'!$B$25)</f>
         <v/>
       </c>
       <c r="D39" s="47">
-        <f>IF('09 Chantiers'!$C$25="","",'09 Chantiers'!$B$25&amp;" · "&amp;'09 Chantiers'!$C$25)</f>
+        <f>IF('10 Chantiers'!$C$25="","",'10 Chantiers'!$B$25&amp;" · "&amp;'10 Chantiers'!$C$25)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="47">
-        <f>IF('07 Phases'!$B$26="","",'07 Phases'!$B$26)</f>
+        <f>IF('08 Phases'!$B$26="","",'08 Phases'!$B$26)</f>
         <v/>
       </c>
       <c r="C40" s="47">
-        <f>IF('08 Sous-phases'!$B$26="","",'08 Sous-phases'!$B$26)</f>
+        <f>IF('09 Sous-phases'!$B$26="","",'09 Sous-phases'!$B$26)</f>
         <v/>
       </c>
       <c r="D40" s="47">
-        <f>IF('09 Chantiers'!$C$26="","",'09 Chantiers'!$B$26&amp;" · "&amp;'09 Chantiers'!$C$26)</f>
+        <f>IF('10 Chantiers'!$C$26="","",'10 Chantiers'!$B$26&amp;" · "&amp;'10 Chantiers'!$C$26)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="47">
-        <f>IF('07 Phases'!$B$27="","",'07 Phases'!$B$27)</f>
+        <f>IF('08 Phases'!$B$27="","",'08 Phases'!$B$27)</f>
         <v/>
       </c>
       <c r="C41" s="47">
-        <f>IF('08 Sous-phases'!$B$27="","",'08 Sous-phases'!$B$27)</f>
+        <f>IF('09 Sous-phases'!$B$27="","",'09 Sous-phases'!$B$27)</f>
         <v/>
       </c>
       <c r="D41" s="47">
-        <f>IF('09 Chantiers'!$C$27="","",'09 Chantiers'!$B$27&amp;" · "&amp;'09 Chantiers'!$C$27)</f>
+        <f>IF('10 Chantiers'!$C$27="","",'10 Chantiers'!$B$27&amp;" · "&amp;'10 Chantiers'!$C$27)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="47">
-        <f>IF('07 Phases'!$B$28="","",'07 Phases'!$B$28)</f>
+        <f>IF('08 Phases'!$B$28="","",'08 Phases'!$B$28)</f>
         <v/>
       </c>
       <c r="C42" s="47">
-        <f>IF('08 Sous-phases'!$B$28="","",'08 Sous-phases'!$B$28)</f>
+        <f>IF('09 Sous-phases'!$B$28="","",'09 Sous-phases'!$B$28)</f>
         <v/>
       </c>
       <c r="D42" s="47">
-        <f>IF('09 Chantiers'!$C$28="","",'09 Chantiers'!$B$28&amp;" · "&amp;'09 Chantiers'!$C$28)</f>
+        <f>IF('10 Chantiers'!$C$28="","",'10 Chantiers'!$B$28&amp;" · "&amp;'10 Chantiers'!$C$28)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="47">
-        <f>IF('07 Phases'!$B$29="","",'07 Phases'!$B$29)</f>
+        <f>IF('08 Phases'!$B$29="","",'08 Phases'!$B$29)</f>
         <v/>
       </c>
       <c r="C43" s="47">
-        <f>IF('08 Sous-phases'!$B$29="","",'08 Sous-phases'!$B$29)</f>
+        <f>IF('09 Sous-phases'!$B$29="","",'09 Sous-phases'!$B$29)</f>
         <v/>
       </c>
       <c r="D43" s="47">
-        <f>IF('09 Chantiers'!$C$29="","",'09 Chantiers'!$B$29&amp;" · "&amp;'09 Chantiers'!$C$29)</f>
+        <f>IF('10 Chantiers'!$C$29="","",'10 Chantiers'!$B$29&amp;" · "&amp;'10 Chantiers'!$C$29)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="47">
-        <f>IF('07 Phases'!$B$30="","",'07 Phases'!$B$30)</f>
+        <f>IF('08 Phases'!$B$30="","",'08 Phases'!$B$30)</f>
         <v/>
       </c>
       <c r="C44" s="47">
-        <f>IF('08 Sous-phases'!$B$30="","",'08 Sous-phases'!$B$30)</f>
+        <f>IF('09 Sous-phases'!$B$30="","",'09 Sous-phases'!$B$30)</f>
         <v/>
       </c>
       <c r="D44" s="47">
-        <f>IF('09 Chantiers'!$C$30="","",'09 Chantiers'!$B$30&amp;" · "&amp;'09 Chantiers'!$C$30)</f>
+        <f>IF('10 Chantiers'!$C$30="","",'10 Chantiers'!$B$30&amp;" · "&amp;'10 Chantiers'!$C$30)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="47">
-        <f>IF('07 Phases'!$B$31="","",'07 Phases'!$B$31)</f>
+        <f>IF('08 Phases'!$B$31="","",'08 Phases'!$B$31)</f>
         <v/>
       </c>
       <c r="C45" s="47">
-        <f>IF('08 Sous-phases'!$B$31="","",'08 Sous-phases'!$B$31)</f>
+        <f>IF('09 Sous-phases'!$B$31="","",'09 Sous-phases'!$B$31)</f>
         <v/>
       </c>
       <c r="D45" s="47">
-        <f>IF('09 Chantiers'!$C$31="","",'09 Chantiers'!$B$31&amp;" · "&amp;'09 Chantiers'!$C$31)</f>
+        <f>IF('10 Chantiers'!$C$31="","",'10 Chantiers'!$B$31&amp;" · "&amp;'10 Chantiers'!$C$31)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="47">
-        <f>IF('07 Phases'!$B$32="","",'07 Phases'!$B$32)</f>
+        <f>IF('08 Phases'!$B$32="","",'08 Phases'!$B$32)</f>
         <v/>
       </c>
       <c r="C46" s="47">
-        <f>IF('08 Sous-phases'!$B$32="","",'08 Sous-phases'!$B$32)</f>
+        <f>IF('09 Sous-phases'!$B$32="","",'09 Sous-phases'!$B$32)</f>
         <v/>
       </c>
       <c r="D46" s="47">
-        <f>IF('09 Chantiers'!$C$32="","",'09 Chantiers'!$B$32&amp;" · "&amp;'09 Chantiers'!$C$32)</f>
+        <f>IF('10 Chantiers'!$C$32="","",'10 Chantiers'!$B$32&amp;" · "&amp;'10 Chantiers'!$C$32)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="47">
-        <f>IF('07 Phases'!$B$33="","",'07 Phases'!$B$33)</f>
+        <f>IF('08 Phases'!$B$33="","",'08 Phases'!$B$33)</f>
         <v/>
       </c>
       <c r="C47" s="47">
-        <f>IF('08 Sous-phases'!$B$33="","",'08 Sous-phases'!$B$33)</f>
+        <f>IF('09 Sous-phases'!$B$33="","",'09 Sous-phases'!$B$33)</f>
         <v/>
       </c>
       <c r="D47" s="47">
-        <f>IF('09 Chantiers'!$C$33="","",'09 Chantiers'!$B$33&amp;" · "&amp;'09 Chantiers'!$C$33)</f>
+        <f>IF('10 Chantiers'!$C$33="","",'10 Chantiers'!$B$33&amp;" · "&amp;'10 Chantiers'!$C$33)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="47">
-        <f>IF('07 Phases'!$B$34="","",'07 Phases'!$B$34)</f>
+        <f>IF('08 Phases'!$B$34="","",'08 Phases'!$B$34)</f>
         <v/>
       </c>
       <c r="C48" s="47">
-        <f>IF('08 Sous-phases'!$B$34="","",'08 Sous-phases'!$B$34)</f>
+        <f>IF('09 Sous-phases'!$B$34="","",'09 Sous-phases'!$B$34)</f>
         <v/>
       </c>
       <c r="D48" s="47">
-        <f>IF('09 Chantiers'!$C$34="","",'09 Chantiers'!$B$34&amp;" · "&amp;'09 Chantiers'!$C$34)</f>
+        <f>IF('10 Chantiers'!$C$34="","",'10 Chantiers'!$B$34&amp;" · "&amp;'10 Chantiers'!$C$34)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="47">
-        <f>IF('07 Phases'!$B$35="","",'07 Phases'!$B$35)</f>
+        <f>IF('08 Phases'!$B$35="","",'08 Phases'!$B$35)</f>
         <v/>
       </c>
       <c r="C49" s="47">
-        <f>IF('08 Sous-phases'!$B$35="","",'08 Sous-phases'!$B$35)</f>
+        <f>IF('09 Sous-phases'!$B$35="","",'09 Sous-phases'!$B$35)</f>
         <v/>
       </c>
       <c r="D49" s="47">
-        <f>IF('09 Chantiers'!$C$35="","",'09 Chantiers'!$B$35&amp;" · "&amp;'09 Chantiers'!$C$35)</f>
+        <f>IF('10 Chantiers'!$C$35="","",'10 Chantiers'!$B$35&amp;" · "&amp;'10 Chantiers'!$C$35)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="47">
-        <f>IF('07 Phases'!$B$36="","",'07 Phases'!$B$36)</f>
+        <f>IF('08 Phases'!$B$36="","",'08 Phases'!$B$36)</f>
         <v/>
       </c>
       <c r="C50" s="47">
-        <f>IF('08 Sous-phases'!$B$36="","",'08 Sous-phases'!$B$36)</f>
+        <f>IF('09 Sous-phases'!$B$36="","",'09 Sous-phases'!$B$36)</f>
         <v/>
       </c>
       <c r="D50" s="47">
-        <f>IF('09 Chantiers'!$C$36="","",'09 Chantiers'!$B$36&amp;" · "&amp;'09 Chantiers'!$C$36)</f>
+        <f>IF('10 Chantiers'!$C$36="","",'10 Chantiers'!$B$36&amp;" · "&amp;'10 Chantiers'!$C$36)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="47">
-        <f>IF('07 Phases'!$B$37="","",'07 Phases'!$B$37)</f>
+        <f>IF('08 Phases'!$B$37="","",'08 Phases'!$B$37)</f>
         <v/>
       </c>
       <c r="C51" s="47">
-        <f>IF('08 Sous-phases'!$B$37="","",'08 Sous-phases'!$B$37)</f>
+        <f>IF('09 Sous-phases'!$B$37="","",'09 Sous-phases'!$B$37)</f>
         <v/>
       </c>
       <c r="D51" s="47">
-        <f>IF('09 Chantiers'!$C$37="","",'09 Chantiers'!$B$37&amp;" · "&amp;'09 Chantiers'!$C$37)</f>
+        <f>IF('10 Chantiers'!$C$37="","",'10 Chantiers'!$B$37&amp;" · "&amp;'10 Chantiers'!$C$37)</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="47">
-        <f>IF('07 Phases'!$B$38="","",'07 Phases'!$B$38)</f>
+        <f>IF('08 Phases'!$B$38="","",'08 Phases'!$B$38)</f>
         <v/>
       </c>
       <c r="C52" s="47">
-        <f>IF('08 Sous-phases'!$B$38="","",'08 Sous-phases'!$B$38)</f>
+        <f>IF('09 Sous-phases'!$B$38="","",'09 Sous-phases'!$B$38)</f>
         <v/>
       </c>
       <c r="D52" s="47">
-        <f>IF('09 Chantiers'!$C$38="","",'09 Chantiers'!$B$38&amp;" · "&amp;'09 Chantiers'!$C$38)</f>
+        <f>IF('10 Chantiers'!$C$38="","",'10 Chantiers'!$B$38&amp;" · "&amp;'10 Chantiers'!$C$38)</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="47" t="n"/>
       <c r="C53" s="47">
-        <f>IF('08 Sous-phases'!$B$39="","",'08 Sous-phases'!$B$39)</f>
+        <f>IF('09 Sous-phases'!$B$39="","",'09 Sous-phases'!$B$39)</f>
         <v/>
       </c>
       <c r="D53" s="47" t="n"/>
@@ -14723,7 +14729,7 @@
     <row r="54">
       <c r="B54" s="47" t="n"/>
       <c r="C54" s="47">
-        <f>IF('08 Sous-phases'!$B$40="","",'08 Sous-phases'!$B$40)</f>
+        <f>IF('09 Sous-phases'!$B$40="","",'09 Sous-phases'!$B$40)</f>
         <v/>
       </c>
       <c r="D54" s="47" t="n"/>
@@ -14731,7 +14737,7 @@
     <row r="55">
       <c r="B55" s="47" t="n"/>
       <c r="C55" s="47">
-        <f>IF('08 Sous-phases'!$B$41="","",'08 Sous-phases'!$B$41)</f>
+        <f>IF('09 Sous-phases'!$B$41="","",'09 Sous-phases'!$B$41)</f>
         <v/>
       </c>
       <c r="D55" s="47" t="n"/>
@@ -14739,7 +14745,7 @@
     <row r="56">
       <c r="B56" s="47" t="n"/>
       <c r="C56" s="47">
-        <f>IF('08 Sous-phases'!$B$42="","",'08 Sous-phases'!$B$42)</f>
+        <f>IF('09 Sous-phases'!$B$42="","",'09 Sous-phases'!$B$42)</f>
         <v/>
       </c>
       <c r="D56" s="47" t="n"/>
@@ -14747,7 +14753,7 @@
     <row r="57">
       <c r="B57" s="47" t="n"/>
       <c r="C57" s="47">
-        <f>IF('08 Sous-phases'!$B$43="","",'08 Sous-phases'!$B$43)</f>
+        <f>IF('09 Sous-phases'!$B$43="","",'09 Sous-phases'!$B$43)</f>
         <v/>
       </c>
       <c r="D57" s="47" t="n"/>
@@ -14755,7 +14761,7 @@
     <row r="58">
       <c r="B58" s="47" t="n"/>
       <c r="C58" s="47">
-        <f>IF('08 Sous-phases'!$B$44="","",'08 Sous-phases'!$B$44)</f>
+        <f>IF('09 Sous-phases'!$B$44="","",'09 Sous-phases'!$B$44)</f>
         <v/>
       </c>
       <c r="D58" s="47" t="n"/>
@@ -14763,7 +14769,7 @@
     <row r="59">
       <c r="B59" s="47" t="n"/>
       <c r="C59" s="47">
-        <f>IF('08 Sous-phases'!$B$45="","",'08 Sous-phases'!$B$45)</f>
+        <f>IF('09 Sous-phases'!$B$45="","",'09 Sous-phases'!$B$45)</f>
         <v/>
       </c>
       <c r="D59" s="47" t="n"/>
@@ -14771,7 +14777,7 @@
     <row r="60">
       <c r="B60" s="47" t="n"/>
       <c r="C60" s="47">
-        <f>IF('08 Sous-phases'!$B$46="","",'08 Sous-phases'!$B$46)</f>
+        <f>IF('09 Sous-phases'!$B$46="","",'09 Sous-phases'!$B$46)</f>
         <v/>
       </c>
       <c r="D60" s="47" t="n"/>
@@ -14779,7 +14785,7 @@
     <row r="61">
       <c r="B61" s="47" t="n"/>
       <c r="C61" s="47">
-        <f>IF('08 Sous-phases'!$B$47="","",'08 Sous-phases'!$B$47)</f>
+        <f>IF('09 Sous-phases'!$B$47="","",'09 Sous-phases'!$B$47)</f>
         <v/>
       </c>
       <c r="D61" s="47" t="n"/>
@@ -14787,7 +14793,7 @@
     <row r="62">
       <c r="B62" s="47" t="n"/>
       <c r="C62" s="47">
-        <f>IF('08 Sous-phases'!$B$48="","",'08 Sous-phases'!$B$48)</f>
+        <f>IF('09 Sous-phases'!$B$48="","",'09 Sous-phases'!$B$48)</f>
         <v/>
       </c>
       <c r="D62" s="47" t="n"/>
@@ -14795,7 +14801,7 @@
     <row r="63">
       <c r="B63" s="47" t="n"/>
       <c r="C63" s="47">
-        <f>IF('08 Sous-phases'!$B$49="","",'08 Sous-phases'!$B$49)</f>
+        <f>IF('09 Sous-phases'!$B$49="","",'09 Sous-phases'!$B$49)</f>
         <v/>
       </c>
       <c r="D63" s="47" t="n"/>
@@ -14803,7 +14809,7 @@
     <row r="64">
       <c r="B64" s="47" t="n"/>
       <c r="C64" s="47">
-        <f>IF('08 Sous-phases'!$B$50="","",'08 Sous-phases'!$B$50)</f>
+        <f>IF('09 Sous-phases'!$B$50="","",'09 Sous-phases'!$B$50)</f>
         <v/>
       </c>
       <c r="D64" s="47" t="n"/>
@@ -14811,7 +14817,7 @@
     <row r="65">
       <c r="B65" s="47" t="n"/>
       <c r="C65" s="47">
-        <f>IF('08 Sous-phases'!$B$51="","",'08 Sous-phases'!$B$51)</f>
+        <f>IF('09 Sous-phases'!$B$51="","",'09 Sous-phases'!$B$51)</f>
         <v/>
       </c>
       <c r="D65" s="47" t="n"/>
@@ -14819,7 +14825,7 @@
     <row r="66">
       <c r="B66" s="47" t="n"/>
       <c r="C66" s="47">
-        <f>IF('08 Sous-phases'!$B$52="","",'08 Sous-phases'!$B$52)</f>
+        <f>IF('09 Sous-phases'!$B$52="","",'09 Sous-phases'!$B$52)</f>
         <v/>
       </c>
       <c r="D66" s="47" t="n"/>
@@ -14827,7 +14833,7 @@
     <row r="67">
       <c r="B67" s="47" t="n"/>
       <c r="C67" s="47">
-        <f>IF('08 Sous-phases'!$B$53="","",'08 Sous-phases'!$B$53)</f>
+        <f>IF('09 Sous-phases'!$B$53="","",'09 Sous-phases'!$B$53)</f>
         <v/>
       </c>
       <c r="D67" s="47" t="n"/>
@@ -14835,7 +14841,7 @@
     <row r="68">
       <c r="B68" s="47" t="n"/>
       <c r="C68" s="47">
-        <f>IF('08 Sous-phases'!$B$54="","",'08 Sous-phases'!$B$54)</f>
+        <f>IF('09 Sous-phases'!$B$54="","",'09 Sous-phases'!$B$54)</f>
         <v/>
       </c>
       <c r="D68" s="47" t="n"/>
@@ -14843,7 +14849,7 @@
     <row r="69">
       <c r="B69" s="47" t="n"/>
       <c r="C69" s="47">
-        <f>IF('08 Sous-phases'!$B$55="","",'08 Sous-phases'!$B$55)</f>
+        <f>IF('09 Sous-phases'!$B$55="","",'09 Sous-phases'!$B$55)</f>
         <v/>
       </c>
       <c r="D69" s="47" t="n"/>
@@ -14851,7 +14857,7 @@
     <row r="70">
       <c r="B70" s="47" t="n"/>
       <c r="C70" s="47">
-        <f>IF('08 Sous-phases'!$B$56="","",'08 Sous-phases'!$B$56)</f>
+        <f>IF('09 Sous-phases'!$B$56="","",'09 Sous-phases'!$B$56)</f>
         <v/>
       </c>
       <c r="D70" s="47" t="n"/>
@@ -14859,7 +14865,7 @@
     <row r="71">
       <c r="B71" s="47" t="n"/>
       <c r="C71" s="47">
-        <f>IF('08 Sous-phases'!$B$57="","",'08 Sous-phases'!$B$57)</f>
+        <f>IF('09 Sous-phases'!$B$57="","",'09 Sous-phases'!$B$57)</f>
         <v/>
       </c>
       <c r="D71" s="47" t="n"/>
@@ -14867,7 +14873,7 @@
     <row r="72">
       <c r="B72" s="47" t="n"/>
       <c r="C72" s="47">
-        <f>IF('08 Sous-phases'!$B$58="","",'08 Sous-phases'!$B$58)</f>
+        <f>IF('09 Sous-phases'!$B$58="","",'09 Sous-phases'!$B$58)</f>
         <v/>
       </c>
       <c r="D72" s="47" t="n"/>
@@ -14875,7 +14881,7 @@
     <row r="73">
       <c r="B73" s="47" t="n"/>
       <c r="C73" s="47">
-        <f>IF('08 Sous-phases'!$B$59="","",'08 Sous-phases'!$B$59)</f>
+        <f>IF('09 Sous-phases'!$B$59="","",'09 Sous-phases'!$B$59)</f>
         <v/>
       </c>
       <c r="D73" s="47" t="n"/>
@@ -14883,7 +14889,7 @@
     <row r="74">
       <c r="B74" s="47" t="n"/>
       <c r="C74" s="47">
-        <f>IF('08 Sous-phases'!$B$60="","",'08 Sous-phases'!$B$60)</f>
+        <f>IF('09 Sous-phases'!$B$60="","",'09 Sous-phases'!$B$60)</f>
         <v/>
       </c>
       <c r="D74" s="47" t="n"/>
@@ -14891,7 +14897,7 @@
     <row r="75">
       <c r="B75" s="47" t="n"/>
       <c r="C75" s="47">
-        <f>IF('08 Sous-phases'!$B$61="","",'08 Sous-phases'!$B$61)</f>
+        <f>IF('09 Sous-phases'!$B$61="","",'09 Sous-phases'!$B$61)</f>
         <v/>
       </c>
       <c r="D75" s="47" t="n"/>
@@ -14899,7 +14905,7 @@
     <row r="76">
       <c r="B76" s="47" t="n"/>
       <c r="C76" s="47">
-        <f>IF('08 Sous-phases'!$B$62="","",'08 Sous-phases'!$B$62)</f>
+        <f>IF('09 Sous-phases'!$B$62="","",'09 Sous-phases'!$B$62)</f>
         <v/>
       </c>
       <c r="D76" s="47" t="n"/>
@@ -14907,7 +14913,7 @@
     <row r="77">
       <c r="B77" s="47" t="n"/>
       <c r="C77" s="47">
-        <f>IF('08 Sous-phases'!$B$63="","",'08 Sous-phases'!$B$63)</f>
+        <f>IF('09 Sous-phases'!$B$63="","",'09 Sous-phases'!$B$63)</f>
         <v/>
       </c>
       <c r="D77" s="47" t="n"/>
@@ -14915,7 +14921,7 @@
     <row r="78">
       <c r="B78" s="47" t="n"/>
       <c r="C78" s="47">
-        <f>IF('08 Sous-phases'!$B$64="","",'08 Sous-phases'!$B$64)</f>
+        <f>IF('09 Sous-phases'!$B$64="","",'09 Sous-phases'!$B$64)</f>
         <v/>
       </c>
       <c r="D78" s="47" t="n"/>
@@ -14923,7 +14929,7 @@
     <row r="79">
       <c r="B79" s="47" t="n"/>
       <c r="C79" s="47">
-        <f>IF('08 Sous-phases'!$B$65="","",'08 Sous-phases'!$B$65)</f>
+        <f>IF('09 Sous-phases'!$B$65="","",'09 Sous-phases'!$B$65)</f>
         <v/>
       </c>
       <c r="D79" s="47" t="n"/>
@@ -14931,7 +14937,7 @@
     <row r="80">
       <c r="B80" s="47" t="n"/>
       <c r="C80" s="47">
-        <f>IF('08 Sous-phases'!$B$66="","",'08 Sous-phases'!$B$66)</f>
+        <f>IF('09 Sous-phases'!$B$66="","",'09 Sous-phases'!$B$66)</f>
         <v/>
       </c>
       <c r="D80" s="47" t="n"/>
@@ -14939,7 +14945,7 @@
     <row r="81">
       <c r="B81" s="47" t="n"/>
       <c r="C81" s="47">
-        <f>IF('08 Sous-phases'!$B$67="","",'08 Sous-phases'!$B$67)</f>
+        <f>IF('09 Sous-phases'!$B$67="","",'09 Sous-phases'!$B$67)</f>
         <v/>
       </c>
       <c r="D81" s="47" t="n"/>
@@ -14947,7 +14953,7 @@
     <row r="82">
       <c r="B82" s="47" t="n"/>
       <c r="C82" s="47">
-        <f>IF('08 Sous-phases'!$B$68="","",'08 Sous-phases'!$B$68)</f>
+        <f>IF('09 Sous-phases'!$B$68="","",'09 Sous-phases'!$B$68)</f>
         <v/>
       </c>
       <c r="D82" s="47" t="n"/>
@@ -14955,7 +14961,7 @@
     <row r="83">
       <c r="B83" s="47" t="n"/>
       <c r="C83" s="47">
-        <f>IF('08 Sous-phases'!$B$69="","",'08 Sous-phases'!$B$69)</f>
+        <f>IF('09 Sous-phases'!$B$69="","",'09 Sous-phases'!$B$69)</f>
         <v/>
       </c>
       <c r="D83" s="47" t="n"/>
@@ -14963,7 +14969,7 @@
     <row r="84">
       <c r="B84" s="47" t="n"/>
       <c r="C84" s="47">
-        <f>IF('08 Sous-phases'!$B$70="","",'08 Sous-phases'!$B$70)</f>
+        <f>IF('09 Sous-phases'!$B$70="","",'09 Sous-phases'!$B$70)</f>
         <v/>
       </c>
       <c r="D84" s="47" t="n"/>
@@ -14971,7 +14977,7 @@
     <row r="85">
       <c r="B85" s="47" t="n"/>
       <c r="C85" s="47">
-        <f>IF('08 Sous-phases'!$B$71="","",'08 Sous-phases'!$B$71)</f>
+        <f>IF('09 Sous-phases'!$B$71="","",'09 Sous-phases'!$B$71)</f>
         <v/>
       </c>
       <c r="D85" s="47" t="n"/>
@@ -14979,7 +14985,7 @@
     <row r="86">
       <c r="B86" s="47" t="n"/>
       <c r="C86" s="47">
-        <f>IF('08 Sous-phases'!$B$72="","",'08 Sous-phases'!$B$72)</f>
+        <f>IF('09 Sous-phases'!$B$72="","",'09 Sous-phases'!$B$72)</f>
         <v/>
       </c>
       <c r="D86" s="47" t="n"/>
@@ -14987,7 +14993,7 @@
     <row r="87">
       <c r="B87" s="47" t="n"/>
       <c r="C87" s="47">
-        <f>IF('08 Sous-phases'!$B$73="","",'08 Sous-phases'!$B$73)</f>
+        <f>IF('09 Sous-phases'!$B$73="","",'09 Sous-phases'!$B$73)</f>
         <v/>
       </c>
       <c r="D87" s="47" t="n"/>
@@ -14995,7 +15001,7 @@
     <row r="88">
       <c r="B88" s="47" t="n"/>
       <c r="C88" s="47">
-        <f>IF('08 Sous-phases'!$B$74="","",'08 Sous-phases'!$B$74)</f>
+        <f>IF('09 Sous-phases'!$B$74="","",'09 Sous-phases'!$B$74)</f>
         <v/>
       </c>
       <c r="D88" s="47" t="n"/>
@@ -15003,7 +15009,7 @@
     <row r="89">
       <c r="B89" s="47" t="n"/>
       <c r="C89" s="47">
-        <f>IF('08 Sous-phases'!$B$75="","",'08 Sous-phases'!$B$75)</f>
+        <f>IF('09 Sous-phases'!$B$75="","",'09 Sous-phases'!$B$75)</f>
         <v/>
       </c>
       <c r="D89" s="47" t="n"/>
@@ -15011,7 +15017,7 @@
     <row r="90">
       <c r="B90" s="47" t="n"/>
       <c r="C90" s="47">
-        <f>IF('08 Sous-phases'!$B$76="","",'08 Sous-phases'!$B$76)</f>
+        <f>IF('09 Sous-phases'!$B$76="","",'09 Sous-phases'!$B$76)</f>
         <v/>
       </c>
       <c r="D90" s="47" t="n"/>
@@ -15019,7 +15025,7 @@
     <row r="91">
       <c r="B91" s="47" t="n"/>
       <c r="C91" s="47">
-        <f>IF('08 Sous-phases'!$B$77="","",'08 Sous-phases'!$B$77)</f>
+        <f>IF('09 Sous-phases'!$B$77="","",'09 Sous-phases'!$B$77)</f>
         <v/>
       </c>
       <c r="D91" s="47" t="n"/>
@@ -15027,7 +15033,7 @@
     <row r="92">
       <c r="B92" s="47" t="n"/>
       <c r="C92" s="47">
-        <f>IF('08 Sous-phases'!$B$78="","",'08 Sous-phases'!$B$78)</f>
+        <f>IF('09 Sous-phases'!$B$78="","",'09 Sous-phases'!$B$78)</f>
         <v/>
       </c>
       <c r="D92" s="47" t="n"/>
@@ -15035,7 +15041,7 @@
     <row r="93">
       <c r="B93" s="47" t="n"/>
       <c r="C93" s="47">
-        <f>IF('08 Sous-phases'!$B$79="","",'08 Sous-phases'!$B$79)</f>
+        <f>IF('09 Sous-phases'!$B$79="","",'09 Sous-phases'!$B$79)</f>
         <v/>
       </c>
       <c r="D93" s="47" t="n"/>
@@ -15043,7 +15049,7 @@
     <row r="94">
       <c r="B94" s="47" t="n"/>
       <c r="C94" s="47">
-        <f>IF('08 Sous-phases'!$B$80="","",'08 Sous-phases'!$B$80)</f>
+        <f>IF('09 Sous-phases'!$B$80="","",'09 Sous-phases'!$B$80)</f>
         <v/>
       </c>
       <c r="D94" s="47" t="n"/>
@@ -15051,7 +15057,7 @@
     <row r="95">
       <c r="B95" s="47" t="n"/>
       <c r="C95" s="47">
-        <f>IF('08 Sous-phases'!$B$81="","",'08 Sous-phases'!$B$81)</f>
+        <f>IF('09 Sous-phases'!$B$81="","",'09 Sous-phases'!$B$81)</f>
         <v/>
       </c>
       <c r="D95" s="47" t="n"/>
@@ -15059,7 +15065,7 @@
     <row r="96">
       <c r="B96" s="47" t="n"/>
       <c r="C96" s="47">
-        <f>IF('08 Sous-phases'!$B$82="","",'08 Sous-phases'!$B$82)</f>
+        <f>IF('09 Sous-phases'!$B$82="","",'09 Sous-phases'!$B$82)</f>
         <v/>
       </c>
       <c r="D96" s="47" t="n"/>
@@ -15067,7 +15073,7 @@
     <row r="97">
       <c r="B97" s="47" t="n"/>
       <c r="C97" s="47">
-        <f>IF('08 Sous-phases'!$B$83="","",'08 Sous-phases'!$B$83)</f>
+        <f>IF('09 Sous-phases'!$B$83="","",'09 Sous-phases'!$B$83)</f>
         <v/>
       </c>
       <c r="D97" s="47" t="n"/>
@@ -15075,7 +15081,7 @@
     <row r="98">
       <c r="B98" s="47" t="n"/>
       <c r="C98" s="47">
-        <f>IF('08 Sous-phases'!$B$84="","",'08 Sous-phases'!$B$84)</f>
+        <f>IF('09 Sous-phases'!$B$84="","",'09 Sous-phases'!$B$84)</f>
         <v/>
       </c>
       <c r="D98" s="47" t="n"/>
@@ -15083,7 +15089,7 @@
     <row r="99">
       <c r="B99" s="47" t="n"/>
       <c r="C99" s="47">
-        <f>IF('08 Sous-phases'!$B$85="","",'08 Sous-phases'!$B$85)</f>
+        <f>IF('09 Sous-phases'!$B$85="","",'09 Sous-phases'!$B$85)</f>
         <v/>
       </c>
       <c r="D99" s="47" t="n"/>
@@ -15091,7 +15097,7 @@
     <row r="100">
       <c r="B100" s="47" t="n"/>
       <c r="C100" s="47">
-        <f>IF('08 Sous-phases'!$B$86="","",'08 Sous-phases'!$B$86)</f>
+        <f>IF('09 Sous-phases'!$B$86="","",'09 Sous-phases'!$B$86)</f>
         <v/>
       </c>
       <c r="D100" s="47" t="n"/>
@@ -15099,7 +15105,7 @@
     <row r="101">
       <c r="B101" s="47" t="n"/>
       <c r="C101" s="47">
-        <f>IF('08 Sous-phases'!$B$87="","",'08 Sous-phases'!$B$87)</f>
+        <f>IF('09 Sous-phases'!$B$87="","",'09 Sous-phases'!$B$87)</f>
         <v/>
       </c>
       <c r="D101" s="47" t="n"/>
@@ -15107,7 +15113,7 @@
     <row r="102">
       <c r="B102" s="47" t="n"/>
       <c r="C102" s="47">
-        <f>IF('08 Sous-phases'!$B$88="","",'08 Sous-phases'!$B$88)</f>
+        <f>IF('09 Sous-phases'!$B$88="","",'09 Sous-phases'!$B$88)</f>
         <v/>
       </c>
       <c r="D102" s="47" t="n"/>
@@ -15125,7 +15131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E38"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -15620,7 +15626,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="E3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -15634,7 +15640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:D48"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -16070,7 +16076,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="D3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -16084,7 +16090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H158"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -18086,7 +18092,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="H3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -18100,7 +18106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H208"/>
+  <dimension ref="A1:H208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -21896,7 +21902,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="H3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -21910,7 +21916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E24"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -21983,6 +21989,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="50" t="inlineStr">
         <is>
@@ -22203,6 +22210,7 @@
       </c>
       <c r="D22" s="53" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="D24" s="57">
         <f>IF(OR(D17="",D18=""),"",IF(D18&lt;D17,"⚠ Fin cible avant démarrage","✓ Dates cohérentes"))</f>
@@ -22274,7 +22282,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" location="#'Complétude'!A1" r:id="rId1"/>
+    <hyperlink ref="E3" location="#'Complétude'!A1"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -22288,7 +22296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -22347,7 +22355,7 @@
               <color rgb="FF10233A"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Étape 05b   </t>
+            <t xml:space="preserve">Étape 06   </t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Sous-phases : numérotation libre, choisie par le directeur de projet
Règle « le N° commence par celui de la phase » retirée (import, Référentiel,
écran, colonne CONTRÔLE du modèle) ; restent : N° unique, sans espace, « ; »
ni « · ». Consigne de la skill de préremplissage mise à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontends/Referentiel RISE - initialisation.xlsx
+++ b/frontends/Referentiel RISE - initialisation.xlsx
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="B2:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2413,7 +2413,6 @@
         <v/>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="16" customHeight="1">
       <c r="B36" s="28" t="inlineStr">
         <is>
@@ -2486,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="B2:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3200,7 +3199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="B2:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3961,7 +3960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="B2:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3990,7 +3989,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Découpage de chaque phase. Le numéro reprend celui de la phase : 5.1, 5.2…</t>
+          <t>Découpage de chaque phase. Numérotation libre, propre au projet et unique : 5.1, 5.2… ou la vôtre.</t>
         </is>
       </c>
       <c r="J3" s="39" t="inlineStr">
@@ -4146,7 +4145,7 @@
       <c r="H9" s="46" t="n"/>
       <c r="I9" s="46" t="n"/>
       <c r="J9" s="48">
-        <f>IF(OR(C9="",D9=""),"",IF(LEFT(D9,LEN(LEFT(C9,FIND(" ·",C9&amp;" ·")-1))+1)&lt;&gt;LEFT(C9,FIND(" ·",C9&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F9&lt;&gt;"",G9&lt;&gt;"",G9&lt;F9),"⚠ Fin avant début",IF(AND(F9&lt;&gt;"",IFERROR(F9&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G9&lt;&gt;"",IFERROR(G9&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C9="",D9=""),"",IF(COUNTIF($D$9:$D$88,D9)&gt;1,"⚠ N° en double",IF(AND(F9&lt;&gt;"",G9&lt;&gt;"",G9&lt;F9),"⚠ Fin avant début",IF(AND(F9&lt;&gt;"",IFERROR(F9&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G9&lt;&gt;"",IFERROR(G9&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C9,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4163,7 +4162,7 @@
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
       <c r="J10" s="48">
-        <f>IF(OR(C10="",D10=""),"",IF(LEFT(D10,LEN(LEFT(C10,FIND(" ·",C10&amp;" ·")-1))+1)&lt;&gt;LEFT(C10,FIND(" ·",C10&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F10&lt;&gt;"",G10&lt;&gt;"",G10&lt;F10),"⚠ Fin avant début",IF(AND(F10&lt;&gt;"",IFERROR(F10&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G10&lt;&gt;"",IFERROR(G10&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C10="",D10=""),"",IF(COUNTIF($D$9:$D$88,D10)&gt;1,"⚠ N° en double",IF(AND(F10&lt;&gt;"",G10&lt;&gt;"",G10&lt;F10),"⚠ Fin avant début",IF(AND(F10&lt;&gt;"",IFERROR(F10&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G10&lt;&gt;"",IFERROR(G10&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C10,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4180,7 +4179,7 @@
       <c r="H11" s="46" t="n"/>
       <c r="I11" s="46" t="n"/>
       <c r="J11" s="48">
-        <f>IF(OR(C11="",D11=""),"",IF(LEFT(D11,LEN(LEFT(C11,FIND(" ·",C11&amp;" ·")-1))+1)&lt;&gt;LEFT(C11,FIND(" ·",C11&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F11&lt;&gt;"",G11&lt;&gt;"",G11&lt;F11),"⚠ Fin avant début",IF(AND(F11&lt;&gt;"",IFERROR(F11&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G11&lt;&gt;"",IFERROR(G11&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C11="",D11=""),"",IF(COUNTIF($D$9:$D$88,D11)&gt;1,"⚠ N° en double",IF(AND(F11&lt;&gt;"",G11&lt;&gt;"",G11&lt;F11),"⚠ Fin avant début",IF(AND(F11&lt;&gt;"",IFERROR(F11&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G11&lt;&gt;"",IFERROR(G11&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C11,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4197,7 +4196,7 @@
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="46" t="n"/>
       <c r="J12" s="48">
-        <f>IF(OR(C12="",D12=""),"",IF(LEFT(D12,LEN(LEFT(C12,FIND(" ·",C12&amp;" ·")-1))+1)&lt;&gt;LEFT(C12,FIND(" ·",C12&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F12&lt;&gt;"",G12&lt;&gt;"",G12&lt;F12),"⚠ Fin avant début",IF(AND(F12&lt;&gt;"",IFERROR(F12&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G12&lt;&gt;"",IFERROR(G12&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C12="",D12=""),"",IF(COUNTIF($D$9:$D$88,D12)&gt;1,"⚠ N° en double",IF(AND(F12&lt;&gt;"",G12&lt;&gt;"",G12&lt;F12),"⚠ Fin avant début",IF(AND(F12&lt;&gt;"",IFERROR(F12&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G12&lt;&gt;"",IFERROR(G12&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C12,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4214,7 +4213,7 @@
       <c r="H13" s="46" t="n"/>
       <c r="I13" s="46" t="n"/>
       <c r="J13" s="48">
-        <f>IF(OR(C13="",D13=""),"",IF(LEFT(D13,LEN(LEFT(C13,FIND(" ·",C13&amp;" ·")-1))+1)&lt;&gt;LEFT(C13,FIND(" ·",C13&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F13&lt;&gt;"",G13&lt;&gt;"",G13&lt;F13),"⚠ Fin avant début",IF(AND(F13&lt;&gt;"",IFERROR(F13&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G13&lt;&gt;"",IFERROR(G13&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C13="",D13=""),"",IF(COUNTIF($D$9:$D$88,D13)&gt;1,"⚠ N° en double",IF(AND(F13&lt;&gt;"",G13&lt;&gt;"",G13&lt;F13),"⚠ Fin avant début",IF(AND(F13&lt;&gt;"",IFERROR(F13&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G13&lt;&gt;"",IFERROR(G13&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C13,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4231,7 +4230,7 @@
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
       <c r="J14" s="48">
-        <f>IF(OR(C14="",D14=""),"",IF(LEFT(D14,LEN(LEFT(C14,FIND(" ·",C14&amp;" ·")-1))+1)&lt;&gt;LEFT(C14,FIND(" ·",C14&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F14&lt;&gt;"",G14&lt;&gt;"",G14&lt;F14),"⚠ Fin avant début",IF(AND(F14&lt;&gt;"",IFERROR(F14&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G14&lt;&gt;"",IFERROR(G14&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C14="",D14=""),"",IF(COUNTIF($D$9:$D$88,D14)&gt;1,"⚠ N° en double",IF(AND(F14&lt;&gt;"",G14&lt;&gt;"",G14&lt;F14),"⚠ Fin avant début",IF(AND(F14&lt;&gt;"",IFERROR(F14&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G14&lt;&gt;"",IFERROR(G14&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C14,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4248,7 +4247,7 @@
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="46" t="n"/>
       <c r="J15" s="48">
-        <f>IF(OR(C15="",D15=""),"",IF(LEFT(D15,LEN(LEFT(C15,FIND(" ·",C15&amp;" ·")-1))+1)&lt;&gt;LEFT(C15,FIND(" ·",C15&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F15&lt;&gt;"",G15&lt;&gt;"",G15&lt;F15),"⚠ Fin avant début",IF(AND(F15&lt;&gt;"",IFERROR(F15&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G15&lt;&gt;"",IFERROR(G15&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C15="",D15=""),"",IF(COUNTIF($D$9:$D$88,D15)&gt;1,"⚠ N° en double",IF(AND(F15&lt;&gt;"",G15&lt;&gt;"",G15&lt;F15),"⚠ Fin avant début",IF(AND(F15&lt;&gt;"",IFERROR(F15&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G15&lt;&gt;"",IFERROR(G15&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C15,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4265,7 +4264,7 @@
       <c r="H16" s="46" t="n"/>
       <c r="I16" s="46" t="n"/>
       <c r="J16" s="48">
-        <f>IF(OR(C16="",D16=""),"",IF(LEFT(D16,LEN(LEFT(C16,FIND(" ·",C16&amp;" ·")-1))+1)&lt;&gt;LEFT(C16,FIND(" ·",C16&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F16&lt;&gt;"",G16&lt;&gt;"",G16&lt;F16),"⚠ Fin avant début",IF(AND(F16&lt;&gt;"",IFERROR(F16&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G16&lt;&gt;"",IFERROR(G16&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C16="",D16=""),"",IF(COUNTIF($D$9:$D$88,D16)&gt;1,"⚠ N° en double",IF(AND(F16&lt;&gt;"",G16&lt;&gt;"",G16&lt;F16),"⚠ Fin avant début",IF(AND(F16&lt;&gt;"",IFERROR(F16&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G16&lt;&gt;"",IFERROR(G16&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C16,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4282,7 +4281,7 @@
       <c r="H17" s="46" t="n"/>
       <c r="I17" s="46" t="n"/>
       <c r="J17" s="48">
-        <f>IF(OR(C17="",D17=""),"",IF(LEFT(D17,LEN(LEFT(C17,FIND(" ·",C17&amp;" ·")-1))+1)&lt;&gt;LEFT(C17,FIND(" ·",C17&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F17&lt;&gt;"",G17&lt;&gt;"",G17&lt;F17),"⚠ Fin avant début",IF(AND(F17&lt;&gt;"",IFERROR(F17&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G17&lt;&gt;"",IFERROR(G17&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C17="",D17=""),"",IF(COUNTIF($D$9:$D$88,D17)&gt;1,"⚠ N° en double",IF(AND(F17&lt;&gt;"",G17&lt;&gt;"",G17&lt;F17),"⚠ Fin avant début",IF(AND(F17&lt;&gt;"",IFERROR(F17&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G17&lt;&gt;"",IFERROR(G17&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C17,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4299,7 +4298,7 @@
       <c r="H18" s="46" t="n"/>
       <c r="I18" s="46" t="n"/>
       <c r="J18" s="48">
-        <f>IF(OR(C18="",D18=""),"",IF(LEFT(D18,LEN(LEFT(C18,FIND(" ·",C18&amp;" ·")-1))+1)&lt;&gt;LEFT(C18,FIND(" ·",C18&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F18&lt;&gt;"",G18&lt;&gt;"",G18&lt;F18),"⚠ Fin avant début",IF(AND(F18&lt;&gt;"",IFERROR(F18&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G18&lt;&gt;"",IFERROR(G18&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C18="",D18=""),"",IF(COUNTIF($D$9:$D$88,D18)&gt;1,"⚠ N° en double",IF(AND(F18&lt;&gt;"",G18&lt;&gt;"",G18&lt;F18),"⚠ Fin avant début",IF(AND(F18&lt;&gt;"",IFERROR(F18&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G18&lt;&gt;"",IFERROR(G18&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C18,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4316,7 +4315,7 @@
       <c r="H19" s="46" t="n"/>
       <c r="I19" s="46" t="n"/>
       <c r="J19" s="48">
-        <f>IF(OR(C19="",D19=""),"",IF(LEFT(D19,LEN(LEFT(C19,FIND(" ·",C19&amp;" ·")-1))+1)&lt;&gt;LEFT(C19,FIND(" ·",C19&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F19&lt;&gt;"",G19&lt;&gt;"",G19&lt;F19),"⚠ Fin avant début",IF(AND(F19&lt;&gt;"",IFERROR(F19&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G19&lt;&gt;"",IFERROR(G19&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C19="",D19=""),"",IF(COUNTIF($D$9:$D$88,D19)&gt;1,"⚠ N° en double",IF(AND(F19&lt;&gt;"",G19&lt;&gt;"",G19&lt;F19),"⚠ Fin avant début",IF(AND(F19&lt;&gt;"",IFERROR(F19&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G19&lt;&gt;"",IFERROR(G19&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C19,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4333,7 +4332,7 @@
       <c r="H20" s="46" t="n"/>
       <c r="I20" s="46" t="n"/>
       <c r="J20" s="48">
-        <f>IF(OR(C20="",D20=""),"",IF(LEFT(D20,LEN(LEFT(C20,FIND(" ·",C20&amp;" ·")-1))+1)&lt;&gt;LEFT(C20,FIND(" ·",C20&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F20&lt;&gt;"",G20&lt;&gt;"",G20&lt;F20),"⚠ Fin avant début",IF(AND(F20&lt;&gt;"",IFERROR(F20&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G20&lt;&gt;"",IFERROR(G20&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C20="",D20=""),"",IF(COUNTIF($D$9:$D$88,D20)&gt;1,"⚠ N° en double",IF(AND(F20&lt;&gt;"",G20&lt;&gt;"",G20&lt;F20),"⚠ Fin avant début",IF(AND(F20&lt;&gt;"",IFERROR(F20&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G20&lt;&gt;"",IFERROR(G20&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C20,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4350,7 +4349,7 @@
       <c r="H21" s="46" t="n"/>
       <c r="I21" s="46" t="n"/>
       <c r="J21" s="48">
-        <f>IF(OR(C21="",D21=""),"",IF(LEFT(D21,LEN(LEFT(C21,FIND(" ·",C21&amp;" ·")-1))+1)&lt;&gt;LEFT(C21,FIND(" ·",C21&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F21&lt;&gt;"",G21&lt;&gt;"",G21&lt;F21),"⚠ Fin avant début",IF(AND(F21&lt;&gt;"",IFERROR(F21&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G21&lt;&gt;"",IFERROR(G21&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C21="",D21=""),"",IF(COUNTIF($D$9:$D$88,D21)&gt;1,"⚠ N° en double",IF(AND(F21&lt;&gt;"",G21&lt;&gt;"",G21&lt;F21),"⚠ Fin avant début",IF(AND(F21&lt;&gt;"",IFERROR(F21&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G21&lt;&gt;"",IFERROR(G21&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C21,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4367,7 +4366,7 @@
       <c r="H22" s="46" t="n"/>
       <c r="I22" s="46" t="n"/>
       <c r="J22" s="48">
-        <f>IF(OR(C22="",D22=""),"",IF(LEFT(D22,LEN(LEFT(C22,FIND(" ·",C22&amp;" ·")-1))+1)&lt;&gt;LEFT(C22,FIND(" ·",C22&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F22&lt;&gt;"",G22&lt;&gt;"",G22&lt;F22),"⚠ Fin avant début",IF(AND(F22&lt;&gt;"",IFERROR(F22&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G22&lt;&gt;"",IFERROR(G22&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C22="",D22=""),"",IF(COUNTIF($D$9:$D$88,D22)&gt;1,"⚠ N° en double",IF(AND(F22&lt;&gt;"",G22&lt;&gt;"",G22&lt;F22),"⚠ Fin avant début",IF(AND(F22&lt;&gt;"",IFERROR(F22&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G22&lt;&gt;"",IFERROR(G22&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C22,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4384,7 +4383,7 @@
       <c r="H23" s="46" t="n"/>
       <c r="I23" s="46" t="n"/>
       <c r="J23" s="48">
-        <f>IF(OR(C23="",D23=""),"",IF(LEFT(D23,LEN(LEFT(C23,FIND(" ·",C23&amp;" ·")-1))+1)&lt;&gt;LEFT(C23,FIND(" ·",C23&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F23&lt;&gt;"",G23&lt;&gt;"",G23&lt;F23),"⚠ Fin avant début",IF(AND(F23&lt;&gt;"",IFERROR(F23&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G23&lt;&gt;"",IFERROR(G23&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C23="",D23=""),"",IF(COUNTIF($D$9:$D$88,D23)&gt;1,"⚠ N° en double",IF(AND(F23&lt;&gt;"",G23&lt;&gt;"",G23&lt;F23),"⚠ Fin avant début",IF(AND(F23&lt;&gt;"",IFERROR(F23&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G23&lt;&gt;"",IFERROR(G23&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C23,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4401,7 +4400,7 @@
       <c r="H24" s="46" t="n"/>
       <c r="I24" s="46" t="n"/>
       <c r="J24" s="48">
-        <f>IF(OR(C24="",D24=""),"",IF(LEFT(D24,LEN(LEFT(C24,FIND(" ·",C24&amp;" ·")-1))+1)&lt;&gt;LEFT(C24,FIND(" ·",C24&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F24&lt;&gt;"",G24&lt;&gt;"",G24&lt;F24),"⚠ Fin avant début",IF(AND(F24&lt;&gt;"",IFERROR(F24&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G24&lt;&gt;"",IFERROR(G24&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C24="",D24=""),"",IF(COUNTIF($D$9:$D$88,D24)&gt;1,"⚠ N° en double",IF(AND(F24&lt;&gt;"",G24&lt;&gt;"",G24&lt;F24),"⚠ Fin avant début",IF(AND(F24&lt;&gt;"",IFERROR(F24&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G24&lt;&gt;"",IFERROR(G24&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C24,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4418,7 +4417,7 @@
       <c r="H25" s="46" t="n"/>
       <c r="I25" s="46" t="n"/>
       <c r="J25" s="48">
-        <f>IF(OR(C25="",D25=""),"",IF(LEFT(D25,LEN(LEFT(C25,FIND(" ·",C25&amp;" ·")-1))+1)&lt;&gt;LEFT(C25,FIND(" ·",C25&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F25&lt;&gt;"",G25&lt;&gt;"",G25&lt;F25),"⚠ Fin avant début",IF(AND(F25&lt;&gt;"",IFERROR(F25&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G25&lt;&gt;"",IFERROR(G25&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C25="",D25=""),"",IF(COUNTIF($D$9:$D$88,D25)&gt;1,"⚠ N° en double",IF(AND(F25&lt;&gt;"",G25&lt;&gt;"",G25&lt;F25),"⚠ Fin avant début",IF(AND(F25&lt;&gt;"",IFERROR(F25&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G25&lt;&gt;"",IFERROR(G25&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C25,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4435,7 +4434,7 @@
       <c r="H26" s="46" t="n"/>
       <c r="I26" s="46" t="n"/>
       <c r="J26" s="48">
-        <f>IF(OR(C26="",D26=""),"",IF(LEFT(D26,LEN(LEFT(C26,FIND(" ·",C26&amp;" ·")-1))+1)&lt;&gt;LEFT(C26,FIND(" ·",C26&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F26&lt;&gt;"",G26&lt;&gt;"",G26&lt;F26),"⚠ Fin avant début",IF(AND(F26&lt;&gt;"",IFERROR(F26&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G26&lt;&gt;"",IFERROR(G26&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C26="",D26=""),"",IF(COUNTIF($D$9:$D$88,D26)&gt;1,"⚠ N° en double",IF(AND(F26&lt;&gt;"",G26&lt;&gt;"",G26&lt;F26),"⚠ Fin avant début",IF(AND(F26&lt;&gt;"",IFERROR(F26&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G26&lt;&gt;"",IFERROR(G26&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C26,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4452,7 +4451,7 @@
       <c r="H27" s="46" t="n"/>
       <c r="I27" s="46" t="n"/>
       <c r="J27" s="48">
-        <f>IF(OR(C27="",D27=""),"",IF(LEFT(D27,LEN(LEFT(C27,FIND(" ·",C27&amp;" ·")-1))+1)&lt;&gt;LEFT(C27,FIND(" ·",C27&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F27&lt;&gt;"",G27&lt;&gt;"",G27&lt;F27),"⚠ Fin avant début",IF(AND(F27&lt;&gt;"",IFERROR(F27&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G27&lt;&gt;"",IFERROR(G27&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C27="",D27=""),"",IF(COUNTIF($D$9:$D$88,D27)&gt;1,"⚠ N° en double",IF(AND(F27&lt;&gt;"",G27&lt;&gt;"",G27&lt;F27),"⚠ Fin avant début",IF(AND(F27&lt;&gt;"",IFERROR(F27&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G27&lt;&gt;"",IFERROR(G27&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C27,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4469,7 +4468,7 @@
       <c r="H28" s="46" t="n"/>
       <c r="I28" s="46" t="n"/>
       <c r="J28" s="48">
-        <f>IF(OR(C28="",D28=""),"",IF(LEFT(D28,LEN(LEFT(C28,FIND(" ·",C28&amp;" ·")-1))+1)&lt;&gt;LEFT(C28,FIND(" ·",C28&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F28&lt;&gt;"",G28&lt;&gt;"",G28&lt;F28),"⚠ Fin avant début",IF(AND(F28&lt;&gt;"",IFERROR(F28&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G28&lt;&gt;"",IFERROR(G28&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C28="",D28=""),"",IF(COUNTIF($D$9:$D$88,D28)&gt;1,"⚠ N° en double",IF(AND(F28&lt;&gt;"",G28&lt;&gt;"",G28&lt;F28),"⚠ Fin avant début",IF(AND(F28&lt;&gt;"",IFERROR(F28&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G28&lt;&gt;"",IFERROR(G28&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C28,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4486,7 +4485,7 @@
       <c r="H29" s="46" t="n"/>
       <c r="I29" s="46" t="n"/>
       <c r="J29" s="48">
-        <f>IF(OR(C29="",D29=""),"",IF(LEFT(D29,LEN(LEFT(C29,FIND(" ·",C29&amp;" ·")-1))+1)&lt;&gt;LEFT(C29,FIND(" ·",C29&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F29&lt;&gt;"",G29&lt;&gt;"",G29&lt;F29),"⚠ Fin avant début",IF(AND(F29&lt;&gt;"",IFERROR(F29&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G29&lt;&gt;"",IFERROR(G29&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C29="",D29=""),"",IF(COUNTIF($D$9:$D$88,D29)&gt;1,"⚠ N° en double",IF(AND(F29&lt;&gt;"",G29&lt;&gt;"",G29&lt;F29),"⚠ Fin avant début",IF(AND(F29&lt;&gt;"",IFERROR(F29&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G29&lt;&gt;"",IFERROR(G29&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C29,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4503,7 +4502,7 @@
       <c r="H30" s="46" t="n"/>
       <c r="I30" s="46" t="n"/>
       <c r="J30" s="48">
-        <f>IF(OR(C30="",D30=""),"",IF(LEFT(D30,LEN(LEFT(C30,FIND(" ·",C30&amp;" ·")-1))+1)&lt;&gt;LEFT(C30,FIND(" ·",C30&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F30&lt;&gt;"",G30&lt;&gt;"",G30&lt;F30),"⚠ Fin avant début",IF(AND(F30&lt;&gt;"",IFERROR(F30&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G30&lt;&gt;"",IFERROR(G30&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C30="",D30=""),"",IF(COUNTIF($D$9:$D$88,D30)&gt;1,"⚠ N° en double",IF(AND(F30&lt;&gt;"",G30&lt;&gt;"",G30&lt;F30),"⚠ Fin avant début",IF(AND(F30&lt;&gt;"",IFERROR(F30&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G30&lt;&gt;"",IFERROR(G30&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C30,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4520,7 +4519,7 @@
       <c r="H31" s="46" t="n"/>
       <c r="I31" s="46" t="n"/>
       <c r="J31" s="48">
-        <f>IF(OR(C31="",D31=""),"",IF(LEFT(D31,LEN(LEFT(C31,FIND(" ·",C31&amp;" ·")-1))+1)&lt;&gt;LEFT(C31,FIND(" ·",C31&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F31&lt;&gt;"",G31&lt;&gt;"",G31&lt;F31),"⚠ Fin avant début",IF(AND(F31&lt;&gt;"",IFERROR(F31&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G31&lt;&gt;"",IFERROR(G31&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C31="",D31=""),"",IF(COUNTIF($D$9:$D$88,D31)&gt;1,"⚠ N° en double",IF(AND(F31&lt;&gt;"",G31&lt;&gt;"",G31&lt;F31),"⚠ Fin avant début",IF(AND(F31&lt;&gt;"",IFERROR(F31&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G31&lt;&gt;"",IFERROR(G31&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C31,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4537,7 +4536,7 @@
       <c r="H32" s="46" t="n"/>
       <c r="I32" s="46" t="n"/>
       <c r="J32" s="48">
-        <f>IF(OR(C32="",D32=""),"",IF(LEFT(D32,LEN(LEFT(C32,FIND(" ·",C32&amp;" ·")-1))+1)&lt;&gt;LEFT(C32,FIND(" ·",C32&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F32&lt;&gt;"",G32&lt;&gt;"",G32&lt;F32),"⚠ Fin avant début",IF(AND(F32&lt;&gt;"",IFERROR(F32&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G32&lt;&gt;"",IFERROR(G32&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C32="",D32=""),"",IF(COUNTIF($D$9:$D$88,D32)&gt;1,"⚠ N° en double",IF(AND(F32&lt;&gt;"",G32&lt;&gt;"",G32&lt;F32),"⚠ Fin avant début",IF(AND(F32&lt;&gt;"",IFERROR(F32&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G32&lt;&gt;"",IFERROR(G32&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C32,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4554,7 +4553,7 @@
       <c r="H33" s="46" t="n"/>
       <c r="I33" s="46" t="n"/>
       <c r="J33" s="48">
-        <f>IF(OR(C33="",D33=""),"",IF(LEFT(D33,LEN(LEFT(C33,FIND(" ·",C33&amp;" ·")-1))+1)&lt;&gt;LEFT(C33,FIND(" ·",C33&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F33&lt;&gt;"",G33&lt;&gt;"",G33&lt;F33),"⚠ Fin avant début",IF(AND(F33&lt;&gt;"",IFERROR(F33&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G33&lt;&gt;"",IFERROR(G33&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C33="",D33=""),"",IF(COUNTIF($D$9:$D$88,D33)&gt;1,"⚠ N° en double",IF(AND(F33&lt;&gt;"",G33&lt;&gt;"",G33&lt;F33),"⚠ Fin avant début",IF(AND(F33&lt;&gt;"",IFERROR(F33&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G33&lt;&gt;"",IFERROR(G33&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C33,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4571,7 +4570,7 @@
       <c r="H34" s="46" t="n"/>
       <c r="I34" s="46" t="n"/>
       <c r="J34" s="48">
-        <f>IF(OR(C34="",D34=""),"",IF(LEFT(D34,LEN(LEFT(C34,FIND(" ·",C34&amp;" ·")-1))+1)&lt;&gt;LEFT(C34,FIND(" ·",C34&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F34&lt;&gt;"",G34&lt;&gt;"",G34&lt;F34),"⚠ Fin avant début",IF(AND(F34&lt;&gt;"",IFERROR(F34&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G34&lt;&gt;"",IFERROR(G34&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C34="",D34=""),"",IF(COUNTIF($D$9:$D$88,D34)&gt;1,"⚠ N° en double",IF(AND(F34&lt;&gt;"",G34&lt;&gt;"",G34&lt;F34),"⚠ Fin avant début",IF(AND(F34&lt;&gt;"",IFERROR(F34&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G34&lt;&gt;"",IFERROR(G34&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C34,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4588,7 +4587,7 @@
       <c r="H35" s="46" t="n"/>
       <c r="I35" s="46" t="n"/>
       <c r="J35" s="48">
-        <f>IF(OR(C35="",D35=""),"",IF(LEFT(D35,LEN(LEFT(C35,FIND(" ·",C35&amp;" ·")-1))+1)&lt;&gt;LEFT(C35,FIND(" ·",C35&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F35&lt;&gt;"",G35&lt;&gt;"",G35&lt;F35),"⚠ Fin avant début",IF(AND(F35&lt;&gt;"",IFERROR(F35&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G35&lt;&gt;"",IFERROR(G35&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C35="",D35=""),"",IF(COUNTIF($D$9:$D$88,D35)&gt;1,"⚠ N° en double",IF(AND(F35&lt;&gt;"",G35&lt;&gt;"",G35&lt;F35),"⚠ Fin avant début",IF(AND(F35&lt;&gt;"",IFERROR(F35&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G35&lt;&gt;"",IFERROR(G35&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C35,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4605,7 +4604,7 @@
       <c r="H36" s="46" t="n"/>
       <c r="I36" s="46" t="n"/>
       <c r="J36" s="48">
-        <f>IF(OR(C36="",D36=""),"",IF(LEFT(D36,LEN(LEFT(C36,FIND(" ·",C36&amp;" ·")-1))+1)&lt;&gt;LEFT(C36,FIND(" ·",C36&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F36&lt;&gt;"",G36&lt;&gt;"",G36&lt;F36),"⚠ Fin avant début",IF(AND(F36&lt;&gt;"",IFERROR(F36&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G36&lt;&gt;"",IFERROR(G36&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C36="",D36=""),"",IF(COUNTIF($D$9:$D$88,D36)&gt;1,"⚠ N° en double",IF(AND(F36&lt;&gt;"",G36&lt;&gt;"",G36&lt;F36),"⚠ Fin avant début",IF(AND(F36&lt;&gt;"",IFERROR(F36&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G36&lt;&gt;"",IFERROR(G36&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C36,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4622,7 +4621,7 @@
       <c r="H37" s="46" t="n"/>
       <c r="I37" s="46" t="n"/>
       <c r="J37" s="48">
-        <f>IF(OR(C37="",D37=""),"",IF(LEFT(D37,LEN(LEFT(C37,FIND(" ·",C37&amp;" ·")-1))+1)&lt;&gt;LEFT(C37,FIND(" ·",C37&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F37&lt;&gt;"",G37&lt;&gt;"",G37&lt;F37),"⚠ Fin avant début",IF(AND(F37&lt;&gt;"",IFERROR(F37&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G37&lt;&gt;"",IFERROR(G37&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C37="",D37=""),"",IF(COUNTIF($D$9:$D$88,D37)&gt;1,"⚠ N° en double",IF(AND(F37&lt;&gt;"",G37&lt;&gt;"",G37&lt;F37),"⚠ Fin avant début",IF(AND(F37&lt;&gt;"",IFERROR(F37&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G37&lt;&gt;"",IFERROR(G37&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C37,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4639,7 +4638,7 @@
       <c r="H38" s="46" t="n"/>
       <c r="I38" s="46" t="n"/>
       <c r="J38" s="48">
-        <f>IF(OR(C38="",D38=""),"",IF(LEFT(D38,LEN(LEFT(C38,FIND(" ·",C38&amp;" ·")-1))+1)&lt;&gt;LEFT(C38,FIND(" ·",C38&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F38&lt;&gt;"",G38&lt;&gt;"",G38&lt;F38),"⚠ Fin avant début",IF(AND(F38&lt;&gt;"",IFERROR(F38&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G38&lt;&gt;"",IFERROR(G38&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C38="",D38=""),"",IF(COUNTIF($D$9:$D$88,D38)&gt;1,"⚠ N° en double",IF(AND(F38&lt;&gt;"",G38&lt;&gt;"",G38&lt;F38),"⚠ Fin avant début",IF(AND(F38&lt;&gt;"",IFERROR(F38&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G38&lt;&gt;"",IFERROR(G38&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C38,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4656,7 +4655,7 @@
       <c r="H39" s="46" t="n"/>
       <c r="I39" s="46" t="n"/>
       <c r="J39" s="48">
-        <f>IF(OR(C39="",D39=""),"",IF(LEFT(D39,LEN(LEFT(C39,FIND(" ·",C39&amp;" ·")-1))+1)&lt;&gt;LEFT(C39,FIND(" ·",C39&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F39&lt;&gt;"",G39&lt;&gt;"",G39&lt;F39),"⚠ Fin avant début",IF(AND(F39&lt;&gt;"",IFERROR(F39&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G39&lt;&gt;"",IFERROR(G39&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C39="",D39=""),"",IF(COUNTIF($D$9:$D$88,D39)&gt;1,"⚠ N° en double",IF(AND(F39&lt;&gt;"",G39&lt;&gt;"",G39&lt;F39),"⚠ Fin avant début",IF(AND(F39&lt;&gt;"",IFERROR(F39&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G39&lt;&gt;"",IFERROR(G39&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C39,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4673,7 +4672,7 @@
       <c r="H40" s="46" t="n"/>
       <c r="I40" s="46" t="n"/>
       <c r="J40" s="48">
-        <f>IF(OR(C40="",D40=""),"",IF(LEFT(D40,LEN(LEFT(C40,FIND(" ·",C40&amp;" ·")-1))+1)&lt;&gt;LEFT(C40,FIND(" ·",C40&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F40&lt;&gt;"",G40&lt;&gt;"",G40&lt;F40),"⚠ Fin avant début",IF(AND(F40&lt;&gt;"",IFERROR(F40&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G40&lt;&gt;"",IFERROR(G40&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C40="",D40=""),"",IF(COUNTIF($D$9:$D$88,D40)&gt;1,"⚠ N° en double",IF(AND(F40&lt;&gt;"",G40&lt;&gt;"",G40&lt;F40),"⚠ Fin avant début",IF(AND(F40&lt;&gt;"",IFERROR(F40&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G40&lt;&gt;"",IFERROR(G40&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C40,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4690,7 +4689,7 @@
       <c r="H41" s="46" t="n"/>
       <c r="I41" s="46" t="n"/>
       <c r="J41" s="48">
-        <f>IF(OR(C41="",D41=""),"",IF(LEFT(D41,LEN(LEFT(C41,FIND(" ·",C41&amp;" ·")-1))+1)&lt;&gt;LEFT(C41,FIND(" ·",C41&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F41&lt;&gt;"",G41&lt;&gt;"",G41&lt;F41),"⚠ Fin avant début",IF(AND(F41&lt;&gt;"",IFERROR(F41&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G41&lt;&gt;"",IFERROR(G41&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C41="",D41=""),"",IF(COUNTIF($D$9:$D$88,D41)&gt;1,"⚠ N° en double",IF(AND(F41&lt;&gt;"",G41&lt;&gt;"",G41&lt;F41),"⚠ Fin avant début",IF(AND(F41&lt;&gt;"",IFERROR(F41&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G41&lt;&gt;"",IFERROR(G41&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C41,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4707,7 +4706,7 @@
       <c r="H42" s="46" t="n"/>
       <c r="I42" s="46" t="n"/>
       <c r="J42" s="48">
-        <f>IF(OR(C42="",D42=""),"",IF(LEFT(D42,LEN(LEFT(C42,FIND(" ·",C42&amp;" ·")-1))+1)&lt;&gt;LEFT(C42,FIND(" ·",C42&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F42&lt;&gt;"",G42&lt;&gt;"",G42&lt;F42),"⚠ Fin avant début",IF(AND(F42&lt;&gt;"",IFERROR(F42&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G42&lt;&gt;"",IFERROR(G42&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C42="",D42=""),"",IF(COUNTIF($D$9:$D$88,D42)&gt;1,"⚠ N° en double",IF(AND(F42&lt;&gt;"",G42&lt;&gt;"",G42&lt;F42),"⚠ Fin avant début",IF(AND(F42&lt;&gt;"",IFERROR(F42&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G42&lt;&gt;"",IFERROR(G42&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C42,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4724,7 +4723,7 @@
       <c r="H43" s="46" t="n"/>
       <c r="I43" s="46" t="n"/>
       <c r="J43" s="48">
-        <f>IF(OR(C43="",D43=""),"",IF(LEFT(D43,LEN(LEFT(C43,FIND(" ·",C43&amp;" ·")-1))+1)&lt;&gt;LEFT(C43,FIND(" ·",C43&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F43&lt;&gt;"",G43&lt;&gt;"",G43&lt;F43),"⚠ Fin avant début",IF(AND(F43&lt;&gt;"",IFERROR(F43&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G43&lt;&gt;"",IFERROR(G43&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C43="",D43=""),"",IF(COUNTIF($D$9:$D$88,D43)&gt;1,"⚠ N° en double",IF(AND(F43&lt;&gt;"",G43&lt;&gt;"",G43&lt;F43),"⚠ Fin avant début",IF(AND(F43&lt;&gt;"",IFERROR(F43&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G43&lt;&gt;"",IFERROR(G43&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C43,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4741,7 +4740,7 @@
       <c r="H44" s="46" t="n"/>
       <c r="I44" s="46" t="n"/>
       <c r="J44" s="48">
-        <f>IF(OR(C44="",D44=""),"",IF(LEFT(D44,LEN(LEFT(C44,FIND(" ·",C44&amp;" ·")-1))+1)&lt;&gt;LEFT(C44,FIND(" ·",C44&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F44&lt;&gt;"",G44&lt;&gt;"",G44&lt;F44),"⚠ Fin avant début",IF(AND(F44&lt;&gt;"",IFERROR(F44&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G44&lt;&gt;"",IFERROR(G44&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C44="",D44=""),"",IF(COUNTIF($D$9:$D$88,D44)&gt;1,"⚠ N° en double",IF(AND(F44&lt;&gt;"",G44&lt;&gt;"",G44&lt;F44),"⚠ Fin avant début",IF(AND(F44&lt;&gt;"",IFERROR(F44&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G44&lt;&gt;"",IFERROR(G44&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C44,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4758,7 +4757,7 @@
       <c r="H45" s="46" t="n"/>
       <c r="I45" s="46" t="n"/>
       <c r="J45" s="48">
-        <f>IF(OR(C45="",D45=""),"",IF(LEFT(D45,LEN(LEFT(C45,FIND(" ·",C45&amp;" ·")-1))+1)&lt;&gt;LEFT(C45,FIND(" ·",C45&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F45&lt;&gt;"",G45&lt;&gt;"",G45&lt;F45),"⚠ Fin avant début",IF(AND(F45&lt;&gt;"",IFERROR(F45&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G45&lt;&gt;"",IFERROR(G45&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C45="",D45=""),"",IF(COUNTIF($D$9:$D$88,D45)&gt;1,"⚠ N° en double",IF(AND(F45&lt;&gt;"",G45&lt;&gt;"",G45&lt;F45),"⚠ Fin avant début",IF(AND(F45&lt;&gt;"",IFERROR(F45&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G45&lt;&gt;"",IFERROR(G45&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C45,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4775,7 +4774,7 @@
       <c r="H46" s="46" t="n"/>
       <c r="I46" s="46" t="n"/>
       <c r="J46" s="48">
-        <f>IF(OR(C46="",D46=""),"",IF(LEFT(D46,LEN(LEFT(C46,FIND(" ·",C46&amp;" ·")-1))+1)&lt;&gt;LEFT(C46,FIND(" ·",C46&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F46&lt;&gt;"",G46&lt;&gt;"",G46&lt;F46),"⚠ Fin avant début",IF(AND(F46&lt;&gt;"",IFERROR(F46&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G46&lt;&gt;"",IFERROR(G46&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C46="",D46=""),"",IF(COUNTIF($D$9:$D$88,D46)&gt;1,"⚠ N° en double",IF(AND(F46&lt;&gt;"",G46&lt;&gt;"",G46&lt;F46),"⚠ Fin avant début",IF(AND(F46&lt;&gt;"",IFERROR(F46&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G46&lt;&gt;"",IFERROR(G46&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C46,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4792,7 +4791,7 @@
       <c r="H47" s="46" t="n"/>
       <c r="I47" s="46" t="n"/>
       <c r="J47" s="48">
-        <f>IF(OR(C47="",D47=""),"",IF(LEFT(D47,LEN(LEFT(C47,FIND(" ·",C47&amp;" ·")-1))+1)&lt;&gt;LEFT(C47,FIND(" ·",C47&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F47&lt;&gt;"",G47&lt;&gt;"",G47&lt;F47),"⚠ Fin avant début",IF(AND(F47&lt;&gt;"",IFERROR(F47&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G47&lt;&gt;"",IFERROR(G47&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C47="",D47=""),"",IF(COUNTIF($D$9:$D$88,D47)&gt;1,"⚠ N° en double",IF(AND(F47&lt;&gt;"",G47&lt;&gt;"",G47&lt;F47),"⚠ Fin avant début",IF(AND(F47&lt;&gt;"",IFERROR(F47&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G47&lt;&gt;"",IFERROR(G47&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C47,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4809,7 +4808,7 @@
       <c r="H48" s="46" t="n"/>
       <c r="I48" s="46" t="n"/>
       <c r="J48" s="48">
-        <f>IF(OR(C48="",D48=""),"",IF(LEFT(D48,LEN(LEFT(C48,FIND(" ·",C48&amp;" ·")-1))+1)&lt;&gt;LEFT(C48,FIND(" ·",C48&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F48&lt;&gt;"",G48&lt;&gt;"",G48&lt;F48),"⚠ Fin avant début",IF(AND(F48&lt;&gt;"",IFERROR(F48&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G48&lt;&gt;"",IFERROR(G48&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C48="",D48=""),"",IF(COUNTIF($D$9:$D$88,D48)&gt;1,"⚠ N° en double",IF(AND(F48&lt;&gt;"",G48&lt;&gt;"",G48&lt;F48),"⚠ Fin avant début",IF(AND(F48&lt;&gt;"",IFERROR(F48&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G48&lt;&gt;"",IFERROR(G48&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C48,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4826,7 +4825,7 @@
       <c r="H49" s="46" t="n"/>
       <c r="I49" s="46" t="n"/>
       <c r="J49" s="48">
-        <f>IF(OR(C49="",D49=""),"",IF(LEFT(D49,LEN(LEFT(C49,FIND(" ·",C49&amp;" ·")-1))+1)&lt;&gt;LEFT(C49,FIND(" ·",C49&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F49&lt;&gt;"",G49&lt;&gt;"",G49&lt;F49),"⚠ Fin avant début",IF(AND(F49&lt;&gt;"",IFERROR(F49&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G49&lt;&gt;"",IFERROR(G49&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C49="",D49=""),"",IF(COUNTIF($D$9:$D$88,D49)&gt;1,"⚠ N° en double",IF(AND(F49&lt;&gt;"",G49&lt;&gt;"",G49&lt;F49),"⚠ Fin avant début",IF(AND(F49&lt;&gt;"",IFERROR(F49&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G49&lt;&gt;"",IFERROR(G49&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C49,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4843,7 +4842,7 @@
       <c r="H50" s="46" t="n"/>
       <c r="I50" s="46" t="n"/>
       <c r="J50" s="48">
-        <f>IF(OR(C50="",D50=""),"",IF(LEFT(D50,LEN(LEFT(C50,FIND(" ·",C50&amp;" ·")-1))+1)&lt;&gt;LEFT(C50,FIND(" ·",C50&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F50&lt;&gt;"",G50&lt;&gt;"",G50&lt;F50),"⚠ Fin avant début",IF(AND(F50&lt;&gt;"",IFERROR(F50&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G50&lt;&gt;"",IFERROR(G50&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C50="",D50=""),"",IF(COUNTIF($D$9:$D$88,D50)&gt;1,"⚠ N° en double",IF(AND(F50&lt;&gt;"",G50&lt;&gt;"",G50&lt;F50),"⚠ Fin avant début",IF(AND(F50&lt;&gt;"",IFERROR(F50&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G50&lt;&gt;"",IFERROR(G50&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C50,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4860,7 +4859,7 @@
       <c r="H51" s="46" t="n"/>
       <c r="I51" s="46" t="n"/>
       <c r="J51" s="48">
-        <f>IF(OR(C51="",D51=""),"",IF(LEFT(D51,LEN(LEFT(C51,FIND(" ·",C51&amp;" ·")-1))+1)&lt;&gt;LEFT(C51,FIND(" ·",C51&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F51&lt;&gt;"",G51&lt;&gt;"",G51&lt;F51),"⚠ Fin avant début",IF(AND(F51&lt;&gt;"",IFERROR(F51&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G51&lt;&gt;"",IFERROR(G51&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C51="",D51=""),"",IF(COUNTIF($D$9:$D$88,D51)&gt;1,"⚠ N° en double",IF(AND(F51&lt;&gt;"",G51&lt;&gt;"",G51&lt;F51),"⚠ Fin avant début",IF(AND(F51&lt;&gt;"",IFERROR(F51&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G51&lt;&gt;"",IFERROR(G51&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C51,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4877,7 +4876,7 @@
       <c r="H52" s="46" t="n"/>
       <c r="I52" s="46" t="n"/>
       <c r="J52" s="48">
-        <f>IF(OR(C52="",D52=""),"",IF(LEFT(D52,LEN(LEFT(C52,FIND(" ·",C52&amp;" ·")-1))+1)&lt;&gt;LEFT(C52,FIND(" ·",C52&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F52&lt;&gt;"",G52&lt;&gt;"",G52&lt;F52),"⚠ Fin avant début",IF(AND(F52&lt;&gt;"",IFERROR(F52&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G52&lt;&gt;"",IFERROR(G52&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C52="",D52=""),"",IF(COUNTIF($D$9:$D$88,D52)&gt;1,"⚠ N° en double",IF(AND(F52&lt;&gt;"",G52&lt;&gt;"",G52&lt;F52),"⚠ Fin avant début",IF(AND(F52&lt;&gt;"",IFERROR(F52&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G52&lt;&gt;"",IFERROR(G52&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C52,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4894,7 +4893,7 @@
       <c r="H53" s="46" t="n"/>
       <c r="I53" s="46" t="n"/>
       <c r="J53" s="48">
-        <f>IF(OR(C53="",D53=""),"",IF(LEFT(D53,LEN(LEFT(C53,FIND(" ·",C53&amp;" ·")-1))+1)&lt;&gt;LEFT(C53,FIND(" ·",C53&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F53&lt;&gt;"",G53&lt;&gt;"",G53&lt;F53),"⚠ Fin avant début",IF(AND(F53&lt;&gt;"",IFERROR(F53&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G53&lt;&gt;"",IFERROR(G53&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C53="",D53=""),"",IF(COUNTIF($D$9:$D$88,D53)&gt;1,"⚠ N° en double",IF(AND(F53&lt;&gt;"",G53&lt;&gt;"",G53&lt;F53),"⚠ Fin avant début",IF(AND(F53&lt;&gt;"",IFERROR(F53&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G53&lt;&gt;"",IFERROR(G53&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C53,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4911,7 +4910,7 @@
       <c r="H54" s="46" t="n"/>
       <c r="I54" s="46" t="n"/>
       <c r="J54" s="48">
-        <f>IF(OR(C54="",D54=""),"",IF(LEFT(D54,LEN(LEFT(C54,FIND(" ·",C54&amp;" ·")-1))+1)&lt;&gt;LEFT(C54,FIND(" ·",C54&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F54&lt;&gt;"",G54&lt;&gt;"",G54&lt;F54),"⚠ Fin avant début",IF(AND(F54&lt;&gt;"",IFERROR(F54&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G54&lt;&gt;"",IFERROR(G54&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C54="",D54=""),"",IF(COUNTIF($D$9:$D$88,D54)&gt;1,"⚠ N° en double",IF(AND(F54&lt;&gt;"",G54&lt;&gt;"",G54&lt;F54),"⚠ Fin avant début",IF(AND(F54&lt;&gt;"",IFERROR(F54&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G54&lt;&gt;"",IFERROR(G54&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C54,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4928,7 +4927,7 @@
       <c r="H55" s="46" t="n"/>
       <c r="I55" s="46" t="n"/>
       <c r="J55" s="48">
-        <f>IF(OR(C55="",D55=""),"",IF(LEFT(D55,LEN(LEFT(C55,FIND(" ·",C55&amp;" ·")-1))+1)&lt;&gt;LEFT(C55,FIND(" ·",C55&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F55&lt;&gt;"",G55&lt;&gt;"",G55&lt;F55),"⚠ Fin avant début",IF(AND(F55&lt;&gt;"",IFERROR(F55&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G55&lt;&gt;"",IFERROR(G55&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C55="",D55=""),"",IF(COUNTIF($D$9:$D$88,D55)&gt;1,"⚠ N° en double",IF(AND(F55&lt;&gt;"",G55&lt;&gt;"",G55&lt;F55),"⚠ Fin avant début",IF(AND(F55&lt;&gt;"",IFERROR(F55&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G55&lt;&gt;"",IFERROR(G55&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C55,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4945,7 +4944,7 @@
       <c r="H56" s="46" t="n"/>
       <c r="I56" s="46" t="n"/>
       <c r="J56" s="48">
-        <f>IF(OR(C56="",D56=""),"",IF(LEFT(D56,LEN(LEFT(C56,FIND(" ·",C56&amp;" ·")-1))+1)&lt;&gt;LEFT(C56,FIND(" ·",C56&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F56&lt;&gt;"",G56&lt;&gt;"",G56&lt;F56),"⚠ Fin avant début",IF(AND(F56&lt;&gt;"",IFERROR(F56&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G56&lt;&gt;"",IFERROR(G56&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C56="",D56=""),"",IF(COUNTIF($D$9:$D$88,D56)&gt;1,"⚠ N° en double",IF(AND(F56&lt;&gt;"",G56&lt;&gt;"",G56&lt;F56),"⚠ Fin avant début",IF(AND(F56&lt;&gt;"",IFERROR(F56&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G56&lt;&gt;"",IFERROR(G56&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C56,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4962,7 +4961,7 @@
       <c r="H57" s="46" t="n"/>
       <c r="I57" s="46" t="n"/>
       <c r="J57" s="48">
-        <f>IF(OR(C57="",D57=""),"",IF(LEFT(D57,LEN(LEFT(C57,FIND(" ·",C57&amp;" ·")-1))+1)&lt;&gt;LEFT(C57,FIND(" ·",C57&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F57&lt;&gt;"",G57&lt;&gt;"",G57&lt;F57),"⚠ Fin avant début",IF(AND(F57&lt;&gt;"",IFERROR(F57&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G57&lt;&gt;"",IFERROR(G57&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C57="",D57=""),"",IF(COUNTIF($D$9:$D$88,D57)&gt;1,"⚠ N° en double",IF(AND(F57&lt;&gt;"",G57&lt;&gt;"",G57&lt;F57),"⚠ Fin avant début",IF(AND(F57&lt;&gt;"",IFERROR(F57&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G57&lt;&gt;"",IFERROR(G57&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C57,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4979,7 +4978,7 @@
       <c r="H58" s="46" t="n"/>
       <c r="I58" s="46" t="n"/>
       <c r="J58" s="48">
-        <f>IF(OR(C58="",D58=""),"",IF(LEFT(D58,LEN(LEFT(C58,FIND(" ·",C58&amp;" ·")-1))+1)&lt;&gt;LEFT(C58,FIND(" ·",C58&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F58&lt;&gt;"",G58&lt;&gt;"",G58&lt;F58),"⚠ Fin avant début",IF(AND(F58&lt;&gt;"",IFERROR(F58&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G58&lt;&gt;"",IFERROR(G58&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C58="",D58=""),"",IF(COUNTIF($D$9:$D$88,D58)&gt;1,"⚠ N° en double",IF(AND(F58&lt;&gt;"",G58&lt;&gt;"",G58&lt;F58),"⚠ Fin avant début",IF(AND(F58&lt;&gt;"",IFERROR(F58&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G58&lt;&gt;"",IFERROR(G58&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C58,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -4996,7 +4995,7 @@
       <c r="H59" s="46" t="n"/>
       <c r="I59" s="46" t="n"/>
       <c r="J59" s="48">
-        <f>IF(OR(C59="",D59=""),"",IF(LEFT(D59,LEN(LEFT(C59,FIND(" ·",C59&amp;" ·")-1))+1)&lt;&gt;LEFT(C59,FIND(" ·",C59&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F59&lt;&gt;"",G59&lt;&gt;"",G59&lt;F59),"⚠ Fin avant début",IF(AND(F59&lt;&gt;"",IFERROR(F59&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G59&lt;&gt;"",IFERROR(G59&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C59="",D59=""),"",IF(COUNTIF($D$9:$D$88,D59)&gt;1,"⚠ N° en double",IF(AND(F59&lt;&gt;"",G59&lt;&gt;"",G59&lt;F59),"⚠ Fin avant début",IF(AND(F59&lt;&gt;"",IFERROR(F59&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G59&lt;&gt;"",IFERROR(G59&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C59,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5013,7 +5012,7 @@
       <c r="H60" s="46" t="n"/>
       <c r="I60" s="46" t="n"/>
       <c r="J60" s="48">
-        <f>IF(OR(C60="",D60=""),"",IF(LEFT(D60,LEN(LEFT(C60,FIND(" ·",C60&amp;" ·")-1))+1)&lt;&gt;LEFT(C60,FIND(" ·",C60&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F60&lt;&gt;"",G60&lt;&gt;"",G60&lt;F60),"⚠ Fin avant début",IF(AND(F60&lt;&gt;"",IFERROR(F60&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G60&lt;&gt;"",IFERROR(G60&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C60="",D60=""),"",IF(COUNTIF($D$9:$D$88,D60)&gt;1,"⚠ N° en double",IF(AND(F60&lt;&gt;"",G60&lt;&gt;"",G60&lt;F60),"⚠ Fin avant début",IF(AND(F60&lt;&gt;"",IFERROR(F60&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G60&lt;&gt;"",IFERROR(G60&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C60,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5030,7 +5029,7 @@
       <c r="H61" s="46" t="n"/>
       <c r="I61" s="46" t="n"/>
       <c r="J61" s="48">
-        <f>IF(OR(C61="",D61=""),"",IF(LEFT(D61,LEN(LEFT(C61,FIND(" ·",C61&amp;" ·")-1))+1)&lt;&gt;LEFT(C61,FIND(" ·",C61&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F61&lt;&gt;"",G61&lt;&gt;"",G61&lt;F61),"⚠ Fin avant début",IF(AND(F61&lt;&gt;"",IFERROR(F61&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G61&lt;&gt;"",IFERROR(G61&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C61="",D61=""),"",IF(COUNTIF($D$9:$D$88,D61)&gt;1,"⚠ N° en double",IF(AND(F61&lt;&gt;"",G61&lt;&gt;"",G61&lt;F61),"⚠ Fin avant début",IF(AND(F61&lt;&gt;"",IFERROR(F61&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G61&lt;&gt;"",IFERROR(G61&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C61,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5047,7 +5046,7 @@
       <c r="H62" s="46" t="n"/>
       <c r="I62" s="46" t="n"/>
       <c r="J62" s="48">
-        <f>IF(OR(C62="",D62=""),"",IF(LEFT(D62,LEN(LEFT(C62,FIND(" ·",C62&amp;" ·")-1))+1)&lt;&gt;LEFT(C62,FIND(" ·",C62&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F62&lt;&gt;"",G62&lt;&gt;"",G62&lt;F62),"⚠ Fin avant début",IF(AND(F62&lt;&gt;"",IFERROR(F62&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G62&lt;&gt;"",IFERROR(G62&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C62="",D62=""),"",IF(COUNTIF($D$9:$D$88,D62)&gt;1,"⚠ N° en double",IF(AND(F62&lt;&gt;"",G62&lt;&gt;"",G62&lt;F62),"⚠ Fin avant début",IF(AND(F62&lt;&gt;"",IFERROR(F62&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G62&lt;&gt;"",IFERROR(G62&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C62,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5064,7 +5063,7 @@
       <c r="H63" s="46" t="n"/>
       <c r="I63" s="46" t="n"/>
       <c r="J63" s="48">
-        <f>IF(OR(C63="",D63=""),"",IF(LEFT(D63,LEN(LEFT(C63,FIND(" ·",C63&amp;" ·")-1))+1)&lt;&gt;LEFT(C63,FIND(" ·",C63&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F63&lt;&gt;"",G63&lt;&gt;"",G63&lt;F63),"⚠ Fin avant début",IF(AND(F63&lt;&gt;"",IFERROR(F63&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G63&lt;&gt;"",IFERROR(G63&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C63="",D63=""),"",IF(COUNTIF($D$9:$D$88,D63)&gt;1,"⚠ N° en double",IF(AND(F63&lt;&gt;"",G63&lt;&gt;"",G63&lt;F63),"⚠ Fin avant début",IF(AND(F63&lt;&gt;"",IFERROR(F63&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G63&lt;&gt;"",IFERROR(G63&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C63,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5081,7 +5080,7 @@
       <c r="H64" s="46" t="n"/>
       <c r="I64" s="46" t="n"/>
       <c r="J64" s="48">
-        <f>IF(OR(C64="",D64=""),"",IF(LEFT(D64,LEN(LEFT(C64,FIND(" ·",C64&amp;" ·")-1))+1)&lt;&gt;LEFT(C64,FIND(" ·",C64&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F64&lt;&gt;"",G64&lt;&gt;"",G64&lt;F64),"⚠ Fin avant début",IF(AND(F64&lt;&gt;"",IFERROR(F64&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G64&lt;&gt;"",IFERROR(G64&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C64="",D64=""),"",IF(COUNTIF($D$9:$D$88,D64)&gt;1,"⚠ N° en double",IF(AND(F64&lt;&gt;"",G64&lt;&gt;"",G64&lt;F64),"⚠ Fin avant début",IF(AND(F64&lt;&gt;"",IFERROR(F64&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G64&lt;&gt;"",IFERROR(G64&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C64,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5098,7 +5097,7 @@
       <c r="H65" s="46" t="n"/>
       <c r="I65" s="46" t="n"/>
       <c r="J65" s="48">
-        <f>IF(OR(C65="",D65=""),"",IF(LEFT(D65,LEN(LEFT(C65,FIND(" ·",C65&amp;" ·")-1))+1)&lt;&gt;LEFT(C65,FIND(" ·",C65&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F65&lt;&gt;"",G65&lt;&gt;"",G65&lt;F65),"⚠ Fin avant début",IF(AND(F65&lt;&gt;"",IFERROR(F65&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G65&lt;&gt;"",IFERROR(G65&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C65="",D65=""),"",IF(COUNTIF($D$9:$D$88,D65)&gt;1,"⚠ N° en double",IF(AND(F65&lt;&gt;"",G65&lt;&gt;"",G65&lt;F65),"⚠ Fin avant début",IF(AND(F65&lt;&gt;"",IFERROR(F65&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G65&lt;&gt;"",IFERROR(G65&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C65,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5115,7 +5114,7 @@
       <c r="H66" s="46" t="n"/>
       <c r="I66" s="46" t="n"/>
       <c r="J66" s="48">
-        <f>IF(OR(C66="",D66=""),"",IF(LEFT(D66,LEN(LEFT(C66,FIND(" ·",C66&amp;" ·")-1))+1)&lt;&gt;LEFT(C66,FIND(" ·",C66&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F66&lt;&gt;"",G66&lt;&gt;"",G66&lt;F66),"⚠ Fin avant début",IF(AND(F66&lt;&gt;"",IFERROR(F66&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G66&lt;&gt;"",IFERROR(G66&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C66="",D66=""),"",IF(COUNTIF($D$9:$D$88,D66)&gt;1,"⚠ N° en double",IF(AND(F66&lt;&gt;"",G66&lt;&gt;"",G66&lt;F66),"⚠ Fin avant début",IF(AND(F66&lt;&gt;"",IFERROR(F66&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G66&lt;&gt;"",IFERROR(G66&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C66,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5132,7 +5131,7 @@
       <c r="H67" s="46" t="n"/>
       <c r="I67" s="46" t="n"/>
       <c r="J67" s="48">
-        <f>IF(OR(C67="",D67=""),"",IF(LEFT(D67,LEN(LEFT(C67,FIND(" ·",C67&amp;" ·")-1))+1)&lt;&gt;LEFT(C67,FIND(" ·",C67&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F67&lt;&gt;"",G67&lt;&gt;"",G67&lt;F67),"⚠ Fin avant début",IF(AND(F67&lt;&gt;"",IFERROR(F67&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G67&lt;&gt;"",IFERROR(G67&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C67="",D67=""),"",IF(COUNTIF($D$9:$D$88,D67)&gt;1,"⚠ N° en double",IF(AND(F67&lt;&gt;"",G67&lt;&gt;"",G67&lt;F67),"⚠ Fin avant début",IF(AND(F67&lt;&gt;"",IFERROR(F67&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G67&lt;&gt;"",IFERROR(G67&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C67,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5149,7 +5148,7 @@
       <c r="H68" s="46" t="n"/>
       <c r="I68" s="46" t="n"/>
       <c r="J68" s="48">
-        <f>IF(OR(C68="",D68=""),"",IF(LEFT(D68,LEN(LEFT(C68,FIND(" ·",C68&amp;" ·")-1))+1)&lt;&gt;LEFT(C68,FIND(" ·",C68&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F68&lt;&gt;"",G68&lt;&gt;"",G68&lt;F68),"⚠ Fin avant début",IF(AND(F68&lt;&gt;"",IFERROR(F68&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G68&lt;&gt;"",IFERROR(G68&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C68="",D68=""),"",IF(COUNTIF($D$9:$D$88,D68)&gt;1,"⚠ N° en double",IF(AND(F68&lt;&gt;"",G68&lt;&gt;"",G68&lt;F68),"⚠ Fin avant début",IF(AND(F68&lt;&gt;"",IFERROR(F68&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G68&lt;&gt;"",IFERROR(G68&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C68,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5166,7 +5165,7 @@
       <c r="H69" s="46" t="n"/>
       <c r="I69" s="46" t="n"/>
       <c r="J69" s="48">
-        <f>IF(OR(C69="",D69=""),"",IF(LEFT(D69,LEN(LEFT(C69,FIND(" ·",C69&amp;" ·")-1))+1)&lt;&gt;LEFT(C69,FIND(" ·",C69&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F69&lt;&gt;"",G69&lt;&gt;"",G69&lt;F69),"⚠ Fin avant début",IF(AND(F69&lt;&gt;"",IFERROR(F69&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G69&lt;&gt;"",IFERROR(G69&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C69="",D69=""),"",IF(COUNTIF($D$9:$D$88,D69)&gt;1,"⚠ N° en double",IF(AND(F69&lt;&gt;"",G69&lt;&gt;"",G69&lt;F69),"⚠ Fin avant début",IF(AND(F69&lt;&gt;"",IFERROR(F69&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G69&lt;&gt;"",IFERROR(G69&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C69,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5183,7 +5182,7 @@
       <c r="H70" s="46" t="n"/>
       <c r="I70" s="46" t="n"/>
       <c r="J70" s="48">
-        <f>IF(OR(C70="",D70=""),"",IF(LEFT(D70,LEN(LEFT(C70,FIND(" ·",C70&amp;" ·")-1))+1)&lt;&gt;LEFT(C70,FIND(" ·",C70&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F70&lt;&gt;"",G70&lt;&gt;"",G70&lt;F70),"⚠ Fin avant début",IF(AND(F70&lt;&gt;"",IFERROR(F70&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G70&lt;&gt;"",IFERROR(G70&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C70="",D70=""),"",IF(COUNTIF($D$9:$D$88,D70)&gt;1,"⚠ N° en double",IF(AND(F70&lt;&gt;"",G70&lt;&gt;"",G70&lt;F70),"⚠ Fin avant début",IF(AND(F70&lt;&gt;"",IFERROR(F70&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G70&lt;&gt;"",IFERROR(G70&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C70,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5200,7 +5199,7 @@
       <c r="H71" s="46" t="n"/>
       <c r="I71" s="46" t="n"/>
       <c r="J71" s="48">
-        <f>IF(OR(C71="",D71=""),"",IF(LEFT(D71,LEN(LEFT(C71,FIND(" ·",C71&amp;" ·")-1))+1)&lt;&gt;LEFT(C71,FIND(" ·",C71&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F71&lt;&gt;"",G71&lt;&gt;"",G71&lt;F71),"⚠ Fin avant début",IF(AND(F71&lt;&gt;"",IFERROR(F71&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G71&lt;&gt;"",IFERROR(G71&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C71="",D71=""),"",IF(COUNTIF($D$9:$D$88,D71)&gt;1,"⚠ N° en double",IF(AND(F71&lt;&gt;"",G71&lt;&gt;"",G71&lt;F71),"⚠ Fin avant début",IF(AND(F71&lt;&gt;"",IFERROR(F71&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G71&lt;&gt;"",IFERROR(G71&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C71,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5217,7 +5216,7 @@
       <c r="H72" s="46" t="n"/>
       <c r="I72" s="46" t="n"/>
       <c r="J72" s="48">
-        <f>IF(OR(C72="",D72=""),"",IF(LEFT(D72,LEN(LEFT(C72,FIND(" ·",C72&amp;" ·")-1))+1)&lt;&gt;LEFT(C72,FIND(" ·",C72&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F72&lt;&gt;"",G72&lt;&gt;"",G72&lt;F72),"⚠ Fin avant début",IF(AND(F72&lt;&gt;"",IFERROR(F72&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G72&lt;&gt;"",IFERROR(G72&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C72="",D72=""),"",IF(COUNTIF($D$9:$D$88,D72)&gt;1,"⚠ N° en double",IF(AND(F72&lt;&gt;"",G72&lt;&gt;"",G72&lt;F72),"⚠ Fin avant début",IF(AND(F72&lt;&gt;"",IFERROR(F72&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G72&lt;&gt;"",IFERROR(G72&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C72,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5234,7 +5233,7 @@
       <c r="H73" s="46" t="n"/>
       <c r="I73" s="46" t="n"/>
       <c r="J73" s="48">
-        <f>IF(OR(C73="",D73=""),"",IF(LEFT(D73,LEN(LEFT(C73,FIND(" ·",C73&amp;" ·")-1))+1)&lt;&gt;LEFT(C73,FIND(" ·",C73&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F73&lt;&gt;"",G73&lt;&gt;"",G73&lt;F73),"⚠ Fin avant début",IF(AND(F73&lt;&gt;"",IFERROR(F73&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G73&lt;&gt;"",IFERROR(G73&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C73="",D73=""),"",IF(COUNTIF($D$9:$D$88,D73)&gt;1,"⚠ N° en double",IF(AND(F73&lt;&gt;"",G73&lt;&gt;"",G73&lt;F73),"⚠ Fin avant début",IF(AND(F73&lt;&gt;"",IFERROR(F73&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G73&lt;&gt;"",IFERROR(G73&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C73,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5251,7 +5250,7 @@
       <c r="H74" s="46" t="n"/>
       <c r="I74" s="46" t="n"/>
       <c r="J74" s="48">
-        <f>IF(OR(C74="",D74=""),"",IF(LEFT(D74,LEN(LEFT(C74,FIND(" ·",C74&amp;" ·")-1))+1)&lt;&gt;LEFT(C74,FIND(" ·",C74&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F74&lt;&gt;"",G74&lt;&gt;"",G74&lt;F74),"⚠ Fin avant début",IF(AND(F74&lt;&gt;"",IFERROR(F74&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G74&lt;&gt;"",IFERROR(G74&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C74="",D74=""),"",IF(COUNTIF($D$9:$D$88,D74)&gt;1,"⚠ N° en double",IF(AND(F74&lt;&gt;"",G74&lt;&gt;"",G74&lt;F74),"⚠ Fin avant début",IF(AND(F74&lt;&gt;"",IFERROR(F74&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G74&lt;&gt;"",IFERROR(G74&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C74,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5268,7 +5267,7 @@
       <c r="H75" s="46" t="n"/>
       <c r="I75" s="46" t="n"/>
       <c r="J75" s="48">
-        <f>IF(OR(C75="",D75=""),"",IF(LEFT(D75,LEN(LEFT(C75,FIND(" ·",C75&amp;" ·")-1))+1)&lt;&gt;LEFT(C75,FIND(" ·",C75&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F75&lt;&gt;"",G75&lt;&gt;"",G75&lt;F75),"⚠ Fin avant début",IF(AND(F75&lt;&gt;"",IFERROR(F75&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G75&lt;&gt;"",IFERROR(G75&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C75="",D75=""),"",IF(COUNTIF($D$9:$D$88,D75)&gt;1,"⚠ N° en double",IF(AND(F75&lt;&gt;"",G75&lt;&gt;"",G75&lt;F75),"⚠ Fin avant début",IF(AND(F75&lt;&gt;"",IFERROR(F75&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G75&lt;&gt;"",IFERROR(G75&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C75,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5285,7 +5284,7 @@
       <c r="H76" s="46" t="n"/>
       <c r="I76" s="46" t="n"/>
       <c r="J76" s="48">
-        <f>IF(OR(C76="",D76=""),"",IF(LEFT(D76,LEN(LEFT(C76,FIND(" ·",C76&amp;" ·")-1))+1)&lt;&gt;LEFT(C76,FIND(" ·",C76&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F76&lt;&gt;"",G76&lt;&gt;"",G76&lt;F76),"⚠ Fin avant début",IF(AND(F76&lt;&gt;"",IFERROR(F76&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G76&lt;&gt;"",IFERROR(G76&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C76="",D76=""),"",IF(COUNTIF($D$9:$D$88,D76)&gt;1,"⚠ N° en double",IF(AND(F76&lt;&gt;"",G76&lt;&gt;"",G76&lt;F76),"⚠ Fin avant début",IF(AND(F76&lt;&gt;"",IFERROR(F76&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G76&lt;&gt;"",IFERROR(G76&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C76,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5302,7 +5301,7 @@
       <c r="H77" s="46" t="n"/>
       <c r="I77" s="46" t="n"/>
       <c r="J77" s="48">
-        <f>IF(OR(C77="",D77=""),"",IF(LEFT(D77,LEN(LEFT(C77,FIND(" ·",C77&amp;" ·")-1))+1)&lt;&gt;LEFT(C77,FIND(" ·",C77&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F77&lt;&gt;"",G77&lt;&gt;"",G77&lt;F77),"⚠ Fin avant début",IF(AND(F77&lt;&gt;"",IFERROR(F77&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G77&lt;&gt;"",IFERROR(G77&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C77="",D77=""),"",IF(COUNTIF($D$9:$D$88,D77)&gt;1,"⚠ N° en double",IF(AND(F77&lt;&gt;"",G77&lt;&gt;"",G77&lt;F77),"⚠ Fin avant début",IF(AND(F77&lt;&gt;"",IFERROR(F77&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G77&lt;&gt;"",IFERROR(G77&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C77,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5319,7 +5318,7 @@
       <c r="H78" s="46" t="n"/>
       <c r="I78" s="46" t="n"/>
       <c r="J78" s="48">
-        <f>IF(OR(C78="",D78=""),"",IF(LEFT(D78,LEN(LEFT(C78,FIND(" ·",C78&amp;" ·")-1))+1)&lt;&gt;LEFT(C78,FIND(" ·",C78&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F78&lt;&gt;"",G78&lt;&gt;"",G78&lt;F78),"⚠ Fin avant début",IF(AND(F78&lt;&gt;"",IFERROR(F78&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G78&lt;&gt;"",IFERROR(G78&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C78="",D78=""),"",IF(COUNTIF($D$9:$D$88,D78)&gt;1,"⚠ N° en double",IF(AND(F78&lt;&gt;"",G78&lt;&gt;"",G78&lt;F78),"⚠ Fin avant début",IF(AND(F78&lt;&gt;"",IFERROR(F78&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G78&lt;&gt;"",IFERROR(G78&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C78,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5336,7 +5335,7 @@
       <c r="H79" s="46" t="n"/>
       <c r="I79" s="46" t="n"/>
       <c r="J79" s="48">
-        <f>IF(OR(C79="",D79=""),"",IF(LEFT(D79,LEN(LEFT(C79,FIND(" ·",C79&amp;" ·")-1))+1)&lt;&gt;LEFT(C79,FIND(" ·",C79&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F79&lt;&gt;"",G79&lt;&gt;"",G79&lt;F79),"⚠ Fin avant début",IF(AND(F79&lt;&gt;"",IFERROR(F79&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G79&lt;&gt;"",IFERROR(G79&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C79="",D79=""),"",IF(COUNTIF($D$9:$D$88,D79)&gt;1,"⚠ N° en double",IF(AND(F79&lt;&gt;"",G79&lt;&gt;"",G79&lt;F79),"⚠ Fin avant début",IF(AND(F79&lt;&gt;"",IFERROR(F79&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G79&lt;&gt;"",IFERROR(G79&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C79,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5353,7 +5352,7 @@
       <c r="H80" s="46" t="n"/>
       <c r="I80" s="46" t="n"/>
       <c r="J80" s="48">
-        <f>IF(OR(C80="",D80=""),"",IF(LEFT(D80,LEN(LEFT(C80,FIND(" ·",C80&amp;" ·")-1))+1)&lt;&gt;LEFT(C80,FIND(" ·",C80&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F80&lt;&gt;"",G80&lt;&gt;"",G80&lt;F80),"⚠ Fin avant début",IF(AND(F80&lt;&gt;"",IFERROR(F80&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G80&lt;&gt;"",IFERROR(G80&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C80="",D80=""),"",IF(COUNTIF($D$9:$D$88,D80)&gt;1,"⚠ N° en double",IF(AND(F80&lt;&gt;"",G80&lt;&gt;"",G80&lt;F80),"⚠ Fin avant début",IF(AND(F80&lt;&gt;"",IFERROR(F80&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G80&lt;&gt;"",IFERROR(G80&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C80,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5370,7 +5369,7 @@
       <c r="H81" s="46" t="n"/>
       <c r="I81" s="46" t="n"/>
       <c r="J81" s="48">
-        <f>IF(OR(C81="",D81=""),"",IF(LEFT(D81,LEN(LEFT(C81,FIND(" ·",C81&amp;" ·")-1))+1)&lt;&gt;LEFT(C81,FIND(" ·",C81&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F81&lt;&gt;"",G81&lt;&gt;"",G81&lt;F81),"⚠ Fin avant début",IF(AND(F81&lt;&gt;"",IFERROR(F81&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G81&lt;&gt;"",IFERROR(G81&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C81="",D81=""),"",IF(COUNTIF($D$9:$D$88,D81)&gt;1,"⚠ N° en double",IF(AND(F81&lt;&gt;"",G81&lt;&gt;"",G81&lt;F81),"⚠ Fin avant début",IF(AND(F81&lt;&gt;"",IFERROR(F81&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G81&lt;&gt;"",IFERROR(G81&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C81,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5387,7 +5386,7 @@
       <c r="H82" s="46" t="n"/>
       <c r="I82" s="46" t="n"/>
       <c r="J82" s="48">
-        <f>IF(OR(C82="",D82=""),"",IF(LEFT(D82,LEN(LEFT(C82,FIND(" ·",C82&amp;" ·")-1))+1)&lt;&gt;LEFT(C82,FIND(" ·",C82&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F82&lt;&gt;"",G82&lt;&gt;"",G82&lt;F82),"⚠ Fin avant début",IF(AND(F82&lt;&gt;"",IFERROR(F82&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G82&lt;&gt;"",IFERROR(G82&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C82="",D82=""),"",IF(COUNTIF($D$9:$D$88,D82)&gt;1,"⚠ N° en double",IF(AND(F82&lt;&gt;"",G82&lt;&gt;"",G82&lt;F82),"⚠ Fin avant début",IF(AND(F82&lt;&gt;"",IFERROR(F82&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G82&lt;&gt;"",IFERROR(G82&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C82,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5404,7 +5403,7 @@
       <c r="H83" s="46" t="n"/>
       <c r="I83" s="46" t="n"/>
       <c r="J83" s="48">
-        <f>IF(OR(C83="",D83=""),"",IF(LEFT(D83,LEN(LEFT(C83,FIND(" ·",C83&amp;" ·")-1))+1)&lt;&gt;LEFT(C83,FIND(" ·",C83&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F83&lt;&gt;"",G83&lt;&gt;"",G83&lt;F83),"⚠ Fin avant début",IF(AND(F83&lt;&gt;"",IFERROR(F83&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G83&lt;&gt;"",IFERROR(G83&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C83="",D83=""),"",IF(COUNTIF($D$9:$D$88,D83)&gt;1,"⚠ N° en double",IF(AND(F83&lt;&gt;"",G83&lt;&gt;"",G83&lt;F83),"⚠ Fin avant début",IF(AND(F83&lt;&gt;"",IFERROR(F83&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G83&lt;&gt;"",IFERROR(G83&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C83,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5421,7 +5420,7 @@
       <c r="H84" s="46" t="n"/>
       <c r="I84" s="46" t="n"/>
       <c r="J84" s="48">
-        <f>IF(OR(C84="",D84=""),"",IF(LEFT(D84,LEN(LEFT(C84,FIND(" ·",C84&amp;" ·")-1))+1)&lt;&gt;LEFT(C84,FIND(" ·",C84&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F84&lt;&gt;"",G84&lt;&gt;"",G84&lt;F84),"⚠ Fin avant début",IF(AND(F84&lt;&gt;"",IFERROR(F84&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G84&lt;&gt;"",IFERROR(G84&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C84="",D84=""),"",IF(COUNTIF($D$9:$D$88,D84)&gt;1,"⚠ N° en double",IF(AND(F84&lt;&gt;"",G84&lt;&gt;"",G84&lt;F84),"⚠ Fin avant début",IF(AND(F84&lt;&gt;"",IFERROR(F84&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G84&lt;&gt;"",IFERROR(G84&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C84,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5438,7 +5437,7 @@
       <c r="H85" s="46" t="n"/>
       <c r="I85" s="46" t="n"/>
       <c r="J85" s="48">
-        <f>IF(OR(C85="",D85=""),"",IF(LEFT(D85,LEN(LEFT(C85,FIND(" ·",C85&amp;" ·")-1))+1)&lt;&gt;LEFT(C85,FIND(" ·",C85&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F85&lt;&gt;"",G85&lt;&gt;"",G85&lt;F85),"⚠ Fin avant début",IF(AND(F85&lt;&gt;"",IFERROR(F85&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G85&lt;&gt;"",IFERROR(G85&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C85="",D85=""),"",IF(COUNTIF($D$9:$D$88,D85)&gt;1,"⚠ N° en double",IF(AND(F85&lt;&gt;"",G85&lt;&gt;"",G85&lt;F85),"⚠ Fin avant début",IF(AND(F85&lt;&gt;"",IFERROR(F85&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G85&lt;&gt;"",IFERROR(G85&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C85,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5455,7 +5454,7 @@
       <c r="H86" s="46" t="n"/>
       <c r="I86" s="46" t="n"/>
       <c r="J86" s="48">
-        <f>IF(OR(C86="",D86=""),"",IF(LEFT(D86,LEN(LEFT(C86,FIND(" ·",C86&amp;" ·")-1))+1)&lt;&gt;LEFT(C86,FIND(" ·",C86&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F86&lt;&gt;"",G86&lt;&gt;"",G86&lt;F86),"⚠ Fin avant début",IF(AND(F86&lt;&gt;"",IFERROR(F86&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G86&lt;&gt;"",IFERROR(G86&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C86="",D86=""),"",IF(COUNTIF($D$9:$D$88,D86)&gt;1,"⚠ N° en double",IF(AND(F86&lt;&gt;"",G86&lt;&gt;"",G86&lt;F86),"⚠ Fin avant début",IF(AND(F86&lt;&gt;"",IFERROR(F86&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G86&lt;&gt;"",IFERROR(G86&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C86,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5472,7 +5471,7 @@
       <c r="H87" s="46" t="n"/>
       <c r="I87" s="46" t="n"/>
       <c r="J87" s="48">
-        <f>IF(OR(C87="",D87=""),"",IF(LEFT(D87,LEN(LEFT(C87,FIND(" ·",C87&amp;" ·")-1))+1)&lt;&gt;LEFT(C87,FIND(" ·",C87&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F87&lt;&gt;"",G87&lt;&gt;"",G87&lt;F87),"⚠ Fin avant début",IF(AND(F87&lt;&gt;"",IFERROR(F87&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G87&lt;&gt;"",IFERROR(G87&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C87="",D87=""),"",IF(COUNTIF($D$9:$D$88,D87)&gt;1,"⚠ N° en double",IF(AND(F87&lt;&gt;"",G87&lt;&gt;"",G87&lt;F87),"⚠ Fin avant début",IF(AND(F87&lt;&gt;"",IFERROR(F87&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G87&lt;&gt;"",IFERROR(G87&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C87,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5489,7 +5488,7 @@
       <c r="H88" s="46" t="n"/>
       <c r="I88" s="46" t="n"/>
       <c r="J88" s="48">
-        <f>IF(OR(C88="",D88=""),"",IF(LEFT(D88,LEN(LEFT(C88,FIND(" ·",C88&amp;" ·")-1))+1)&lt;&gt;LEFT(C88,FIND(" ·",C88&amp;" ·")-1)&amp;".","⚠ N° hors phase",IF(AND(F88&lt;&gt;"",G88&lt;&gt;"",G88&lt;F88),"⚠ Fin avant début",IF(AND(F88&lt;&gt;"",IFERROR(F88&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G88&lt;&gt;"",IFERROR(G88&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
+        <f>IF(OR(C88="",D88=""),"",IF(COUNTIF($D$9:$D$88,D88)&gt;1,"⚠ N° en double",IF(AND(F88&lt;&gt;"",G88&lt;&gt;"",G88&lt;F88),"⚠ Fin avant début",IF(AND(F88&lt;&gt;"",IFERROR(F88&lt;INDEX('08 Phases'!$F$9:$F$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Début avant la phase",IF(AND(G88&lt;&gt;"",IFERROR(G88&gt;INDEX('08 Phases'!$G$9:$G$38,MATCH(C88,'08 Phases'!$B$9:$B$38,0)),FALSE)),"◔ Fin après la phase","✓")))))</f>
         <v/>
       </c>
     </row>
@@ -5554,7 +5553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="B2:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6336,7 +6335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="B2:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6993,7 +6992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="B2:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8967,7 +8966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="B2:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -11030,7 +11029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H158"/>
+  <dimension ref="B2:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -13434,7 +13433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="B2:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -13460,7 +13459,6 @@
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
-    <row r="5"/>
     <row r="6" ht="24" customHeight="1">
       <c r="B6" s="29" t="inlineStr">
         <is>
@@ -13992,7 +13990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E102"/>
+  <dimension ref="B2:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -14005,7 +14003,6 @@
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -14020,7 +14017,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
@@ -14050,7 +14046,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
@@ -14264,8 +14259,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
@@ -15131,7 +15124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="B2:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -15640,7 +15633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="B2:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -16090,7 +16083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H158"/>
+  <dimension ref="B2:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -18106,7 +18099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H208"/>
+  <dimension ref="B2:H208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -21916,7 +21909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="B2:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -21989,7 +21982,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="50" t="inlineStr">
         <is>
@@ -22210,7 +22202,6 @@
       </c>
       <c r="D22" s="53" t="n"/>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="D24" s="57">
         <f>IF(OR(D17="",D18=""),"",IF(D18&lt;D17,"⚠ Fin cible avant démarrage","✓ Dates cohérentes"))</f>
@@ -22296,7 +22287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="B2:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Projet : code postal (référentiel, Excel d'initialisation) et géocodage de la météo et du trafic
Project.postalCode (migration 20261118000400), ligne « Code postal » du référentiel après la ville, PATCH /project ;
onglet « 05 Projet » du modèle : « Ville du projet » et « Code postal » après « Pays » (lignes décalées, Complétude et
chaîne de calcul mises à jour), lus à l'import ; météo et trafic géocodés d'abord par le code postal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontends/Referentiel RISE - initialisation.xlsx
+++ b/frontends/Referentiel RISE - initialisation.xlsx
@@ -3182,7 +3182,7 @@
         <v>À démarrer</v>
       </c>
       <c r="K23" s="19">
-        <f>('05 Projet'!D8&lt;&gt;"")+('05 Projet'!D10&lt;&gt;"")+('05 Projet'!D12&lt;&gt;"")+('05 Projet'!D13&lt;&gt;"")+('05 Projet'!D17&lt;&gt;"")+('05 Projet'!D18&lt;&gt;"")+('05 Projet'!D19&lt;&gt;"")+('05 Projet'!D21&lt;&gt;"")</f>
+        <f>('05 Projet'!D8&lt;&gt;"")+('05 Projet'!D10&lt;&gt;"")+('05 Projet'!D14&lt;&gt;"")+('05 Projet'!D15&lt;&gt;"")+('05 Projet'!D19&lt;&gt;"")+('05 Projet'!D20&lt;&gt;"")+('05 Projet'!D21&lt;&gt;"")+('05 Projet'!D23&lt;&gt;"")</f>
         <v>0</v>
       </c>
       <c r="L23" s="19">
@@ -21967,7 +21967,7 @@
     <tabColor rgb="FF1D8F86"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E24"/>
+  <dimension ref="B1:E26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -21983,7 +21983,7 @@
         <v>37</v>
       </c>
       <c r="E2" s="35">
-        <f>Complétude!$I23</f>
+        <f>Complétude!$I25</f>
         <v>0</v>
       </c>
     </row>
@@ -22039,109 +22039,127 @@
       </c>
       <c r="D10" s="50"/>
     </row>
-    <row r="11" spans="2:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
+    <row r="11" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Ville du projet</t>
+        </is>
+      </c>
+      <c r="C11" s="51" t="inlineStr">
+        <is>
+          <t>FACULTATIF</t>
+        </is>
+      </c>
+      <c r="D11" s="50"/>
+      <c r="E11" s="52" t="inlineStr">
+        <is>
+          <t>Une seule commune, ex. Palaiseau</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Code postal</t>
+        </is>
+      </c>
+      <c r="C12" s="51" t="inlineStr">
+        <is>
+          <t>FACULTATIF</t>
+        </is>
+      </c>
+      <c r="D12" s="50"/>
+      <c r="E12" s="52" t="inlineStr">
+        <is>
+          <t>Ex. 91120 : précise la météo et le trafic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="48"/>
-    </row>
-    <row r="12" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="C12" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="D12" s="50"/>
-      <c r="E12" s="52" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="C13" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="D13" s="50"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
     </row>
     <row r="14" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="13" t="s">
-        <v>236</v>
-      </c>
-      <c r="C14" s="51" t="s">
-        <v>199</v>
+        <v>233</v>
+      </c>
+      <c r="C14" s="49" t="s">
+        <v>198</v>
       </c>
       <c r="D14" s="50"/>
       <c r="E14" s="52" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="C15" s="51" t="s">
-        <v>213</v>
+        <v>235</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>198</v>
       </c>
       <c r="D15" s="50"/>
-      <c r="E15" s="52" t="s">
-        <v>239</v>
-      </c>
     </row>
     <row r="16" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D16" s="50"/>
       <c r="E16" s="52" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="C17" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="D17" s="50"/>
+      <c r="E17" s="52" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="C17" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="D17" s="53"/>
-    </row>
-    <row r="18" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="C18" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="D18" s="53"/>
+        <v>240</v>
+      </c>
+      <c r="C18" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="D18" s="50"/>
+      <c r="E18" s="52" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="19" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>212</v>
-      </c>
-      <c r="D19" s="50"/>
+        <v>198</v>
+      </c>
+      <c r="D19" s="53"/>
     </row>
     <row r="20" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="51" t="s">
-        <v>213</v>
-      </c>
-      <c r="D20" s="50"/>
+        <v>242</v>
+      </c>
+      <c r="C20" s="49" t="s">
+        <v>198</v>
+      </c>
+      <c r="D20" s="53"/>
     </row>
     <row r="21" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C21" s="49" t="s">
         <v>212</v>
@@ -22150,16 +22168,34 @@
     </row>
     <row r="22" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="13" t="s">
-        <v>245</v>
+        <v>19</v>
       </c>
       <c r="C22" s="51" t="s">
         <v>213</v>
       </c>
       <c r="D22" s="50"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D24" s="54" t="str">
-        <f>IF(OR(D17="",D18=""),"",IF(D18&lt;D17,"⚠ Fin cible avant démarrage","✓ Dates cohérentes"))</f>
+    <row r="23" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="C23" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="D23" s="50"/>
+    </row>
+    <row r="24" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="C24" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="D24" s="50"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="54" t="str">
+        <f>IF(OR(D19="",D20=""),"",IF(D20&lt;D19,"⚠ Fin cible avant démarrage","✓ Dates cohérentes"))</f>
         <v/>
       </c>
     </row>
@@ -22175,35 +22211,35 @@
       <formula>D10=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D13">
+  <conditionalFormatting sqref="D14:D15">
     <cfRule type="expression" dxfId="45" priority="3">
-      <formula>D12=""</formula>
+      <formula>D14=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D19">
+  <conditionalFormatting sqref="D19:D21">
     <cfRule type="expression" dxfId="44" priority="5">
-      <formula>D17=""</formula>
+      <formula>D19=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D21">
+  <conditionalFormatting sqref="D23">
     <cfRule type="expression" dxfId="43" priority="8">
-      <formula>D21=""</formula>
+      <formula>D23=""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D15:D16" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D17:D18" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>L_Equipes</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Date attendue" error="Saisissez une date au format JJ/MM/AAAA." sqref="D17:D18" xr:uid="{00000000-0002-0000-0700-000001000000}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Date attendue" error="Saisissez une date au format JJ/MM/AAAA." sqref="D19:D20" xr:uid="{00000000-0002-0000-0700-000001000000}">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D19" xr:uid="{00000000-0002-0000-0700-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D21" xr:uid="{00000000-0002-0000-0700-000002000000}">
       <formula1>L_Fuseau</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D20" xr:uid="{00000000-0002-0000-0700-000003000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D22" xr:uid="{00000000-0002-0000-0700-000003000000}">
       <formula1>L_StatutProjet</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D21:D22" xr:uid="{00000000-0002-0000-0700-000004000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valeur hors liste" error="Choisissez une valeur dans la liste." sqref="D23:D24" xr:uid="{00000000-0002-0000-0700-000004000000}">
       <formula1>L_Personnes</formula1>
     </dataValidation>
   </dataValidations>
@@ -22217,7 +22253,7 @@
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="containsText" priority="9" operator="containsText" id="{00000000-000E-0000-0700-000009000000}">
-            <xm:f>NOT(ISERROR(SEARCH("⚠",D24)))</xm:f>
+            <xm:f>NOT(ISERROR(SEARCH("⚠",D26)))</xm:f>
             <x14:dxf>
               <font>
                 <b/>
@@ -22225,7 +22261,7 @@
               </font>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>D24</xm:sqref>
+          <xm:sqref>D26</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>